<commit_message>
MNP prepaid checkout uses the shared prepaid checkout
prepaidCheckoutStep takes its own lines, detail rows, fees, a panel above and totals mapping; the port-in validation gate becomes MnpGatePanel; MnpCheckout removed.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -1266,7 +1266,7 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>The order read-back before signing and payment (plan, add-ons, discount, number, billing, monthly and one-off totals); publishes the totals and read-back rows the CAF and Payment reuse. An optional panel above it (the port-in validation gate). Includes the prepaid cart (Add another subscription) and prepaid checkout.</t>
+          <t>The order read-back before signing and payment (plan, add-ons, discount, number, billing, monthly and one-off totals); publishes the totals and read-back rows the CAF and Payment reuse. An optional panel above it (the port-in validation gate). Includes the prepaid cart (Add another subscription) and the prepaid checkout, which a prepaid port-in also uses with its own lines, details and fees.</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
@@ -2703,7 +2703,7 @@
       <c r="G27" s="17" t="inlineStr"/>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3147,7 +3147,7 @@
       <c r="G39" s="17" t="inlineStr"/>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3227,7 +3227,7 @@
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3307,7 +3307,7 @@
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4411,7 +4411,7 @@
       <c r="G72" s="17" t="inlineStr"/>
       <c r="H72" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4727,7 +4727,7 @@
       </c>
       <c r="H80" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4995,7 +4995,7 @@
       </c>
       <c r="H87" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5035,7 +5035,7 @@
       </c>
       <c r="H88" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5071,7 +5071,7 @@
       <c r="G89" s="17" t="inlineStr"/>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Capability Library: live samples, Appointment Booking rebuild, shared Drawer style, single-layout Billing Account
Appointment Booking: date strip, slots and technicians, specific date/time request, notes, documents the technician collects. Shared Drawer: eyebrow header and equal-width footer. Billing Account one layout with the Create card in the account row. Manual MSISDN entry removed from the number picker. Samples for Guided activation wizard, Customer Qualification, Plan, CAF and Checkout variants. Journey customer lock removed from the library listing. Benefits and Included in this offer in one row; toast title bold; eligibility icon centred.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -14,7 +14,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Method" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$111</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$110</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$55</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -715,10 +715,10 @@
         </is>
       </c>
       <c r="C7" s="17" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>4</v>
@@ -855,14 +855,14 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>110 UI components + 54 non-UI files</t>
+          <t>109 UI components + 54 non-UI files</t>
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>21</v>
@@ -887,11 +887,11 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>22 named - see the Capabilities sheet</t>
+          <t>21 named - see the Capabilities sheet</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>22</v>
+        <v>21</v>
       </c>
       <c r="D15" s="17" t="inlineStr"/>
       <c r="E15" s="17" t="inlineStr"/>
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E23"/>
+  <dimension ref="A1:E22"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37.80" customWidth="1" min="1" max="1"/>
@@ -948,72 +948,42 @@
     <row r="2">
       <c r="A2" s="17" t="inlineStr">
         <is>
-          <t>Journey customer lock</t>
+          <t>Toasts and notifications</t>
         </is>
       </c>
       <c r="B2" s="17" t="inlineStr">
         <is>
-          <t>The state every guided journey keeps: the customer lock, draft, confirmed order, header badge (name, QID, customer ID) and exit destinations.</t>
+          <t>One-line toasts below the header; structured cards at the bottom.</t>
         </is>
       </c>
       <c r="C2" s="17" t="inlineStr">
-        <is>
-          <t>capabilities/JourneyCustomerLock/JourneyCustomerBadge.tsx
-capabilities/JourneyCustomerLock/index.ts
-capabilities/JourneyCustomerLock/journeyModel.ts
-capabilities/JourneyCustomerLock/useJourneyCustomerLock.ts
-capabilities/JourneyCustomerLock/useJourneySession.ts
-stores/customerContextStore.ts</t>
-        </is>
-      </c>
-      <c r="D2" s="17" t="n">
-        <v>22</v>
-      </c>
-      <c r="E2" s="17" t="inlineStr">
-        <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-    </row>
-    <row r="3">
-      <c r="A3" s="17" t="inlineStr">
-        <is>
-          <t>Toasts and notifications</t>
-        </is>
-      </c>
-      <c r="B3" s="17" t="inlineStr">
-        <is>
-          <t>One-line toasts below the header; structured cards at the bottom.</t>
-        </is>
-      </c>
-      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>capabilities/Toasts/Toast.tsx
 capabilities/Toasts/index.ts
 stores/notificationStore.ts</t>
         </is>
       </c>
-      <c r="D3" s="17" t="n">
+      <c r="D2" s="17" t="n">
         <v>19</v>
       </c>
-      <c r="E3" s="17" t="inlineStr">
+      <c r="E2" s="17" t="inlineStr">
         <is>
           <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="A4" s="17" t="inlineStr">
+    <row r="3">
+      <c r="A3" s="17" t="inlineStr">
         <is>
           <t>Customer Identification</t>
         </is>
       </c>
-      <c r="B4" s="17" t="inlineStr">
+      <c r="B3" s="17" t="inlineStr">
         <is>
           <t>Select an ID type, scan the document, validate with MOI and show the validated Identity Details in one card, in every journey.</t>
         </is>
       </c>
-      <c r="C4" s="17" t="inlineStr">
+      <c r="C3" s="17" t="inlineStr">
         <is>
           <t>capabilities/CustomerIdentification/CustomerIdentification.tsx
 capabilities/CustomerIdentification/IdentityDetailsCard.tsx
@@ -1034,12 +1004,38 @@
 components/domain/qidImageUploadModel.ts</t>
         </is>
       </c>
+      <c r="D3" s="17" t="n">
+        <v>12</v>
+      </c>
+      <c r="E3" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" s="17" t="inlineStr">
+        <is>
+          <t>Guided activation wizard</t>
+        </is>
+      </c>
+      <c r="B4" s="17" t="inlineStr">
+        <is>
+          <t>The step shell every activation / migration / port-in journey runs in.</t>
+        </is>
+      </c>
+      <c r="C4" s="17" t="inlineStr">
+        <is>
+          <t>capabilities/GuidedActivationWizard/GuidedActivationWizard.tsx
+capabilities/GuidedActivationWizard/index.ts</t>
+        </is>
+      </c>
       <c r="D4" s="17" t="n">
-        <v>12</v>
+        <v>10</v>
       </c>
       <c r="E4" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
     </row>
@@ -1076,41 +1072,15 @@
     <row r="6">
       <c r="A6" s="17" t="inlineStr">
         <is>
-          <t>Guided activation wizard</t>
+          <t>SIM Type</t>
         </is>
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>The step shell every activation / migration / port-in journey runs in.</t>
+          <t>Choose and validate the SIM: Physical (scan or enter the serial) or eSIM (issued, handed over after payment).</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
-        <is>
-          <t>capabilities/GuidedActivationWizard/GuidedActivationWizard.tsx
-capabilities/GuidedActivationWizard/index.ts</t>
-        </is>
-      </c>
-      <c r="D6" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="E6" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
-        </is>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="17" t="inlineStr">
-        <is>
-          <t>SIM Type</t>
-        </is>
-      </c>
-      <c r="B7" s="17" t="inlineStr">
-        <is>
-          <t>Choose and validate the SIM: Physical (scan or enter the serial) or eSIM (issued, handed over after payment).</t>
-        </is>
-      </c>
-      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>capabilities/SimType/SimSerial.tsx
 capabilities/SimType/SimType.tsx
@@ -1121,27 +1091,27 @@
 components/domain/SimSerialScanner.tsx</t>
         </is>
       </c>
-      <c r="D7" s="17" t="n">
+      <c r="D6" s="17" t="n">
         <v>9</v>
       </c>
-      <c r="E7" s="17" t="inlineStr">
+      <c r="E6" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="17" t="inlineStr">
+    <row r="7">
+      <c r="A7" s="17" t="inlineStr">
         <is>
           <t>Billing Account</t>
         </is>
       </c>
-      <c r="B8" s="17" t="inlineStr">
-        <is>
-          <t>Set up what an order bills to: pick or create a billing account, or just the order's billing settings.</t>
-        </is>
-      </c>
-      <c r="C8" s="17" t="inlineStr">
+      <c r="B7" s="17" t="inlineStr">
+        <is>
+          <t>Set up what an order bills to: one layout everywhere - the customer's existing billing accounts, or Create New Billing Account (contact, billing address, payment, card on file, primary payment profile, billing profile setup).</t>
+        </is>
+      </c>
+      <c r="C7" s="17" t="inlineStr">
         <is>
           <t>capabilities/BillingAccount/BillingAccount.tsx
 capabilities/BillingAccount/index.ts
@@ -1149,33 +1119,32 @@
 capabilities/BillingAccount/step.tsx
 capabilities/BillingAccount/summary.ts
 components/patterns/BillingAccountStep.tsx
-components/patterns/BillingProfileStep.tsx
 components/patterns/BillingProfileSetupDrawer.tsx
 components/patterns/BillingAccountAutoResolver.tsx
 components/patterns/billingAccountModel.ts</t>
         </is>
       </c>
-      <c r="D8" s="17" t="n">
+      <c r="D7" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E8" s="17" t="inlineStr">
+      <c r="E7" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="9">
-      <c r="A9" s="17" t="inlineStr">
+    <row r="8">
+      <c r="A8" s="17" t="inlineStr">
         <is>
           <t>Service Address</t>
         </is>
       </c>
-      <c r="B9" s="17" t="inlineStr">
+      <c r="B8" s="17" t="inlineStr">
         <is>
           <t>The address a service is activated at: one layout everywhere: Service Information (Kahramaa Meter ID / Vodafone Premise ID with Search), then Zone / Street / Building, then Additional Details, with Qatari-ID prefill.</t>
         </is>
       </c>
-      <c r="C9" s="17" t="inlineStr">
+      <c r="C8" s="17" t="inlineStr">
         <is>
           <t>capabilities/ServiceAddress/ServiceAddress.tsx
 capabilities/ServiceAddress/index.ts
@@ -1184,27 +1153,27 @@
 components/patterns/ZsbAddressStep.tsx</t>
         </is>
       </c>
-      <c r="D9" s="17" t="n">
+      <c r="D8" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E9" s="17" t="inlineStr">
+      <c r="E8" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="10">
-      <c r="A10" s="17" t="inlineStr">
+    <row r="9">
+      <c r="A9" s="17" t="inlineStr">
         <is>
           <t>Plan Selection</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B9" s="17" t="inlineStr">
         <is>
           <t>Choose the plan: postpaid plan cards then Add-ons (discounts, bill limit), prepaid packs then Add-ons, or the fixed-line / fibre plan cards with the credit check.</t>
         </is>
       </c>
-      <c r="C10" s="17" t="inlineStr">
+      <c r="C9" s="17" t="inlineStr">
         <is>
           <t>capabilities/PlanSelection/PlanSelection.tsx
 capabilities/PlanSelection/index.ts
@@ -1218,27 +1187,27 @@
 components/patterns/PlanGroupPanel.tsx</t>
         </is>
       </c>
-      <c r="D10" s="17" t="n">
+      <c r="D9" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E10" s="17" t="inlineStr">
+      <c r="E9" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="17" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="17" t="inlineStr">
         <is>
           <t>CAF &amp; Signature</t>
         </is>
       </c>
-      <c r="B11" s="17" t="inlineStr">
+      <c r="B10" s="17" t="inlineStr">
         <is>
           <t>The Customer Agreement Form: terms, CAF type, signature and supporting documents. Standard variant (name, key information, signature) and full variant (the customer reads back the Checkout Summary order, agrees the terms and signs; the journey locks once signed); postpaid and prepaid forms.</t>
         </is>
       </c>
-      <c r="C11" s="17" t="inlineStr">
+      <c r="C10" s="17" t="inlineStr">
         <is>
           <t>capabilities/CafSignature/CafSignature.tsx
 capabilities/CafSignature/index.ts
@@ -1249,27 +1218,27 @@
 components/patterns/cafTypes.ts</t>
         </is>
       </c>
-      <c r="D11" s="17" t="n">
+      <c r="D10" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E11" s="17" t="inlineStr">
+      <c r="E10" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="17" t="inlineStr">
+    <row r="11">
+      <c r="A11" s="17" t="inlineStr">
         <is>
           <t>Checkout Summary</t>
         </is>
       </c>
-      <c r="B12" s="17" t="inlineStr">
+      <c r="B11" s="17" t="inlineStr">
         <is>
           <t>The order read-back before signing and payment (plan, add-ons, discount, number, billing, monthly and one-off totals); publishes the totals and read-back rows the CAF and Payment reuse. An optional panel above it (the port-in validation gate). Includes the prepaid cart (Add another subscription) and the prepaid checkout, which a prepaid port-in also uses with its own lines, details and fees.</t>
         </is>
       </c>
-      <c r="C12" s="17" t="inlineStr">
+      <c r="C11" s="17" t="inlineStr">
         <is>
           <t>capabilities/CheckoutSummary/CheckoutSummary.tsx
 capabilities/CheckoutSummary/PrepaidCartBody.tsx
@@ -1288,27 +1257,27 @@
 components/patterns/prepaidCartModel.ts</t>
         </is>
       </c>
-      <c r="D12" s="17" t="n">
+      <c r="D11" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E12" s="17" t="inlineStr">
+      <c r="E11" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="17" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="17" t="inlineStr">
         <is>
           <t>Payment</t>
         </is>
       </c>
-      <c r="B13" s="17" t="inlineStr">
+      <c r="B12" s="17" t="inlineStr">
         <is>
           <t>Take the amount due at the counter through WinCash and record the outcome.</t>
         </is>
       </c>
-      <c r="C13" s="17" t="inlineStr">
+      <c r="C12" s="17" t="inlineStr">
         <is>
           <t>capabilities/Payment/Payment.tsx
 capabilities/Payment/index.ts
@@ -1316,27 +1285,27 @@
 components/patterns/WinCashPaymentStep.tsx</t>
         </is>
       </c>
-      <c r="D13" s="17" t="n">
+      <c r="D12" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E13" s="17" t="inlineStr">
+      <c r="E12" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="17" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="17" t="inlineStr">
         <is>
           <t>Activation Complete</t>
         </is>
       </c>
-      <c r="B14" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>The confirmation page for a submitted activation (facts, status, follow-on actions, eSIM handover, email) and the confirmed-order shape journeys hand it.</t>
         </is>
       </c>
-      <c r="C14" s="17" t="inlineStr">
+      <c r="C13" s="17" t="inlineStr">
         <is>
           <t>capabilities/ActivationComplete/ActivationComplete.tsx
 capabilities/ActivationComplete/confirmedOrder.ts
@@ -1345,27 +1314,27 @@
 components/patterns/OrderConfirmationScreen.tsx</t>
         </is>
       </c>
-      <c r="D14" s="17" t="n">
+      <c r="D13" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E14" s="17" t="inlineStr">
+      <c r="E13" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="17" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="17" t="inlineStr">
         <is>
           <t>Eligibility gate</t>
         </is>
       </c>
-      <c r="B15" s="17" t="inlineStr">
+      <c r="B14" s="17" t="inlineStr">
         <is>
           <t>Hard-stop / soft-stop / pass eligibility check shown after identification, with the outcome panel, checks report and footer actions.</t>
         </is>
       </c>
-      <c r="C15" s="17" t="inlineStr">
+      <c r="C14" s="17" t="inlineStr">
         <is>
           <t>capabilities/EligibilityGate/EligibilityGateStep.tsx
 capabilities/EligibilityGate/EligibilityOutcomes.tsx
@@ -1373,6 +1342,32 @@
 capabilities/EligibilityGate/index.ts</t>
         </is>
       </c>
+      <c r="D14" s="17" t="n">
+        <v>8</v>
+      </c>
+      <c r="E14" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="15">
+      <c r="A15" s="17" t="inlineStr">
+        <is>
+          <t>Add-ons selection</t>
+        </is>
+      </c>
+      <c r="B15" s="17" t="inlineStr">
+        <is>
+          <t>Add-on cards with included-benefit handling.</t>
+        </is>
+      </c>
+      <c r="C15" s="17" t="inlineStr">
+        <is>
+          <t>capabilities/AddonsSelection/AddonsPicker.tsx
+capabilities/AddonsSelection/index.ts</t>
+        </is>
+      </c>
       <c r="D15" s="17" t="n">
         <v>8</v>
       </c>
@@ -1385,18 +1380,20 @@
     <row r="16">
       <c r="A16" s="17" t="inlineStr">
         <is>
-          <t>Add-ons selection</t>
+          <t>Customer Qualification</t>
         </is>
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>Add-on cards with included-benefit handling.</t>
+          <t>Identify the customer, run eligibility, then offer the special-discount types - the whole "Customer Identification" step of an activation, with its outcomes and footer actions.</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>capabilities/AddonsSelection/AddonsPicker.tsx
-capabilities/AddonsSelection/index.ts</t>
+          <t>capabilities/CustomerQualification/JourneyBanners.tsx
+capabilities/CustomerQualification/index.ts
+capabilities/CustomerQualification/step.tsx
+capabilities/CustomerQualification/summary.ts</t>
         </is>
       </c>
       <c r="D16" s="17" t="n">
@@ -1479,7 +1476,7 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>Book the installation visit: cluster, date and time slot.</t>
+          <t>Book the installation visit: SLA cluster, the date strip (next working days from the earliest, with each day's open slots), the day's time slots and technicians free, the customer's request for a specific date and time (a later date makes the order future-dated), appointment notes and the documents the technician collects (defaulted from the persona).</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
@@ -1487,7 +1484,8 @@
           <t>capabilities/AppointmentBooking/AppointmentBooking.tsx
 capabilities/AppointmentBooking/index.ts
 capabilities/AppointmentBooking/step.tsx
-components/patterns/AppointmentBookingStep.tsx</t>
+components/patterns/AppointmentBookingStep.tsx
+components/patterns/appointmentModel.ts</t>
         </is>
       </c>
       <c r="D19" s="17" t="n">
@@ -1502,43 +1500,15 @@
     <row r="20">
       <c r="A20" s="17" t="inlineStr">
         <is>
-          <t>Customer Qualification</t>
+          <t>Activity Comments</t>
         </is>
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>Identify the customer, run eligibility, then offer the special-discount types - the whole "Customer Identification" step of an activation, with its outcomes and footer actions.</t>
+          <t>The closing note on the actions performed, with an optional channel.</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
-        <is>
-          <t>capabilities/CustomerQualification/JourneyBanners.tsx
-capabilities/CustomerQualification/index.ts
-capabilities/CustomerQualification/step.tsx
-capabilities/CustomerQualification/summary.ts</t>
-        </is>
-      </c>
-      <c r="D20" s="17" t="n">
-        <v>7</v>
-      </c>
-      <c r="E20" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration</t>
-        </is>
-      </c>
-    </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
-        <is>
-          <t>Activity Comments</t>
-        </is>
-      </c>
-      <c r="B21" s="17" t="inlineStr">
-        <is>
-          <t>The closing note on the actions performed, with an optional channel.</t>
-        </is>
-      </c>
-      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>capabilities/ActivityComments/ActivityComments.tsx
 capabilities/ActivityComments/index.ts
@@ -1546,60 +1516,60 @@
 components/patterns/ActivityCommentsStep.tsx</t>
         </is>
       </c>
+      <c r="D20" s="17" t="n">
+        <v>3</v>
+      </c>
+      <c r="E20" s="17" t="inlineStr">
+        <is>
+          <t>pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
+        <is>
+          <t>Selectable card styling</t>
+        </is>
+      </c>
+      <c r="B21" s="17" t="inlineStr">
+        <is>
+          <t>One selected / idle / highlighted surface for plans, offers, numbers, add-ons, discounts and ID/customer type.</t>
+        </is>
+      </c>
+      <c r="C21" s="17" t="inlineStr">
+        <is>
+          <t>capabilities/SelectableCard/index.ts</t>
+        </is>
+      </c>
       <c r="D21" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="E21" s="17" t="inlineStr">
         <is>
-          <t>pre-to-post-migration, sim-number-management, administration</t>
+          <t>administration</t>
         </is>
       </c>
     </row>
     <row r="22">
       <c r="A22" s="17" t="inlineStr">
         <is>
-          <t>Selectable card styling</t>
+          <t>Side drawer</t>
         </is>
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>One selected / idle / highlighted surface for plans, offers, numbers, add-ons, discounts and ID/customer type.</t>
+          <t>Fixed 50%-width drawer for forms, details and multi-step flows: the title as a small uppercase label beside the close control, the body on the page tint, and a footer whose buttons share its width equally.</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>capabilities/SelectableCard/index.ts</t>
+          <t>capabilities/SideDrawer/index.ts</t>
         </is>
       </c>
       <c r="D22" s="17" t="n">
         <v>1</v>
       </c>
       <c r="E22" s="17" t="inlineStr">
-        <is>
-          <t>administration</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Side drawer</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>Fixed 50%-width drawer for forms, details and multi-step flows.</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>capabilities/SideDrawer/index.ts</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>administration</t>
         </is>
@@ -1616,7 +1586,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H110"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.85" customWidth="1" min="1" max="1"/>
@@ -1742,7 +1712,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ValidationStatus, ZsbAddressStep, StepSummarySection, WizardFooter, WizardStepHeader, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ValidationStatus, ZsbAddressStep, StepSummarySection, WizardFooter, WizardStepHeader, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
@@ -1822,7 +1792,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BillingProfileStep, BulkOperationPortal, DonorAttachmentStep, DonorDetailsStep, GuidedContactStep, TicketCreationModal, ZsbAddressStep</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, DonorAttachmentStep, DonorDetailsStep, GuidedContactStep, TicketCreationModal, ZsbAddressStep</t>
         </is>
       </c>
       <c r="H5" s="17" t="inlineStr">
@@ -1862,7 +1832,7 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, BillLimitEditor, CpeSerialScanner, MsisdnPicker, SimSerialScanner, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, DonorDetailsStep, GuidedContactStep, IdLookupStep, PostpaidDiscountsPanel, TicketCreationModal, VerificationGate, ZsbAddressStep, PhoneNumberInput</t>
+          <t>AdditionalDocumentsUpload, BillLimitEditor, CpeSerialScanner, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, DonorDetailsStep, GuidedContactStep, IdLookupStep, PostpaidDiscountsPanel, TicketCreationModal, VerificationGate, ZsbAddressStep, PhoneNumberInput</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -2102,7 +2072,7 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>CreditCheckPanel, MsisdnPicker, BillingAccountStep, CafSignatureCapture, PrepaidPlanStep</t>
+          <t>CreditCheckPanel, MsisdnPicker, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, PrepaidPlanStep</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
@@ -2302,7 +2272,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, QidInput, BillingAccountStep, DiscountCard, FixedPlanStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
+          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
@@ -4199,12 +4169,12 @@
       </c>
       <c r="B67" s="17" t="inlineStr">
         <is>
-          <t>BillingProfileStep</t>
+          <t>CafSignatureCapture</t>
         </is>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingProfileStep.tsx</t>
+          <t>components/patterns/CafSignatureCapture.tsx</t>
         </is>
       </c>
       <c r="D67" s="20" t="inlineStr">
@@ -4223,7 +4193,7 @@
       <c r="G67" s="17" t="inlineStr"/>
       <c r="H67" s="17" t="inlineStr">
         <is>
-          <t>2026-09-26</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4235,12 +4205,12 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture</t>
+          <t>CheckoutDefaultLayout</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafSignatureCapture.tsx</t>
+          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
         </is>
       </c>
       <c r="D68" s="20" t="inlineStr">
@@ -4256,7 +4226,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G68" s="17" t="inlineStr"/>
+      <c r="G68" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep</t>
+        </is>
+      </c>
       <c r="H68" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4271,12 +4245,12 @@
       </c>
       <c r="B69" s="17" t="inlineStr">
         <is>
-          <t>CheckoutDefaultLayout</t>
+          <t>CheckoutSummaryStep</t>
         </is>
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
+          <t>components/patterns/CheckoutSummaryStep.tsx</t>
         </is>
       </c>
       <c r="D69" s="20" t="inlineStr">
@@ -4292,14 +4266,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G69" s="17" t="inlineStr">
-        <is>
-          <t>CheckoutSummaryStep</t>
-        </is>
-      </c>
+      <c r="G69" s="17" t="inlineStr"/>
       <c r="H69" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4311,12 +4281,12 @@
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>CheckoutSummaryStep</t>
+          <t>DiscountCard</t>
         </is>
       </c>
       <c r="C70" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryStep.tsx</t>
+          <t>components/patterns/DiscountCard.tsx</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
@@ -4332,7 +4302,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G70" s="17" t="inlineStr"/>
+      <c r="G70" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidDiscountsPanel</t>
+        </is>
+      </c>
       <c r="H70" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -4347,12 +4321,12 @@
       </c>
       <c r="B71" s="17" t="inlineStr">
         <is>
-          <t>DiscountCard</t>
+          <t>FixedPlanStep</t>
         </is>
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DiscountCard.tsx</t>
+          <t>components/patterns/FixedPlanStep.tsx</t>
         </is>
       </c>
       <c r="D71" s="20" t="inlineStr">
@@ -4368,14 +4342,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G71" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidDiscountsPanel</t>
-        </is>
-      </c>
+      <c r="G71" s="17" t="inlineStr"/>
       <c r="H71" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4387,12 +4357,12 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>FixedPlanStep</t>
+          <t>FullTerms</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/FixedPlanStep.tsx</t>
+          <t>components/patterns/CafTerms.tsx</t>
         </is>
       </c>
       <c r="D72" s="20" t="inlineStr">
@@ -4408,10 +4378,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G72" s="17" t="inlineStr"/>
+      <c r="G72" s="17" t="inlineStr">
+        <is>
+          <t>CafSignatureCapture</t>
+        </is>
+      </c>
       <c r="H72" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4423,12 +4397,12 @@
       </c>
       <c r="B73" s="17" t="inlineStr">
         <is>
-          <t>FullTerms</t>
+          <t>KeyInformationPanel</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafTerms.tsx</t>
+          <t>components/patterns/KeyInformationPanel.tsx</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
@@ -4444,11 +4418,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G73" s="17" t="inlineStr">
-        <is>
-          <t>CafSignatureCapture</t>
-        </is>
-      </c>
+      <c r="G73" s="17" t="inlineStr"/>
       <c r="H73" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -4463,12 +4433,12 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>KeyInformationPanel</t>
+          <t>OrderConfirmationScreen</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/KeyInformationPanel.tsx</t>
+          <t>components/patterns/OrderConfirmationScreen.tsx</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
@@ -4484,10 +4454,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G74" s="17" t="inlineStr"/>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>ActivationCompleteScreen</t>
+        </is>
+      </c>
       <c r="H74" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4499,12 +4473,12 @@
       </c>
       <c r="B75" s="17" t="inlineStr">
         <is>
-          <t>OrderConfirmationScreen</t>
+          <t>PlanDetailsDrawer</t>
         </is>
       </c>
       <c r="C75" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/OrderConfirmationScreen.tsx</t>
+          <t>components/patterns/PlanDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D75" s="20" t="inlineStr">
@@ -4522,12 +4496,12 @@
       </c>
       <c r="G75" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4539,12 +4513,12 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>PlanDetailsDrawer</t>
+          <t>PlanGroupPanel</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanDetailsDrawer.tsx</t>
+          <t>components/patterns/PlanGroupPanel.tsx</t>
         </is>
       </c>
       <c r="D76" s="20" t="inlineStr">
@@ -4579,12 +4553,12 @@
       </c>
       <c r="B77" s="17" t="inlineStr">
         <is>
-          <t>PlanGroupPanel</t>
+          <t>PlanSearchBox</t>
         </is>
       </c>
       <c r="C77" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanGroupPanel.tsx</t>
+          <t>components/patterns/PlanSearchBox.tsx</t>
         </is>
       </c>
       <c r="D77" s="20" t="inlineStr">
@@ -4619,12 +4593,12 @@
       </c>
       <c r="B78" s="17" t="inlineStr">
         <is>
-          <t>PlanSearchBox</t>
+          <t>PlanTabStrip</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanSearchBox.tsx</t>
+          <t>components/patterns/PlanTabStrip.tsx</t>
         </is>
       </c>
       <c r="D78" s="20" t="inlineStr">
@@ -4647,7 +4621,7 @@
       </c>
       <c r="H78" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4659,12 +4633,12 @@
       </c>
       <c r="B79" s="17" t="inlineStr">
         <is>
-          <t>PlanTabStrip</t>
+          <t>PostpaidAddonsPanel</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanTabStrip.tsx</t>
+          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
         </is>
       </c>
       <c r="D79" s="20" t="inlineStr">
@@ -4699,12 +4673,12 @@
       </c>
       <c r="B80" s="17" t="inlineStr">
         <is>
-          <t>PostpaidAddonsPanel</t>
+          <t>PostpaidDiscountsPanel</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
+          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
         </is>
       </c>
       <c r="D80" s="20" t="inlineStr">
@@ -4727,7 +4701,7 @@
       </c>
       <c r="H80" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4739,12 +4713,12 @@
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>PostpaidDiscountsPanel</t>
+          <t>PostpaidMonthlySummary</t>
         </is>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
+          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
         </is>
       </c>
       <c r="D81" s="20" t="inlineStr">
@@ -4767,7 +4741,7 @@
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4779,12 +4753,12 @@
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>PostpaidMonthlySummary</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
+          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
         </is>
       </c>
       <c r="D82" s="20" t="inlineStr">
@@ -4800,11 +4774,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G82" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidPlanAddonsStep</t>
-        </is>
-      </c>
+      <c r="G82" s="17" t="inlineStr"/>
       <c r="H82" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4819,12 +4789,12 @@
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanAddonsStep</t>
+          <t>PostpaidPlanCard</t>
         </is>
       </c>
       <c r="C83" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
+          <t>components/patterns/PostpaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D83" s="20" t="inlineStr">
@@ -4840,7 +4810,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G83" s="17" t="inlineStr"/>
+      <c r="G83" s="17" t="inlineStr">
+        <is>
+          <t>PlanGroupPanel</t>
+        </is>
+      </c>
       <c r="H83" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4855,12 +4829,12 @@
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanCard</t>
+          <t>PrepaidCartStep</t>
         </is>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanCard.tsx</t>
+          <t>components/patterns/PrepaidCartStep.tsx</t>
         </is>
       </c>
       <c r="D84" s="20" t="inlineStr">
@@ -4876,14 +4850,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G84" s="17" t="inlineStr">
-        <is>
-          <t>PlanGroupPanel</t>
-        </is>
-      </c>
+      <c r="G84" s="17" t="inlineStr"/>
       <c r="H84" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4895,12 +4865,12 @@
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCartStep</t>
+          <t>PrepaidCheckoutStep</t>
         </is>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCartStep.tsx</t>
+          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
         </is>
       </c>
       <c r="D85" s="20" t="inlineStr">
@@ -4919,7 +4889,7 @@
       <c r="G85" s="17" t="inlineStr"/>
       <c r="H85" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4931,12 +4901,12 @@
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCheckoutStep</t>
+          <t>PrepaidPackDetailsDrawer</t>
         </is>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
+          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D86" s="20" t="inlineStr">
@@ -4952,7 +4922,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G86" s="17" t="inlineStr"/>
+      <c r="G86" s="17" t="inlineStr">
+        <is>
+          <t>PrepaidPlanStep</t>
+        </is>
+      </c>
       <c r="H86" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4967,12 +4941,12 @@
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPackDetailsDrawer</t>
+          <t>PrepaidPlanCard</t>
         </is>
       </c>
       <c r="C87" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
+          <t>components/patterns/PrepaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D87" s="20" t="inlineStr">
@@ -5007,12 +4981,12 @@
       </c>
       <c r="B88" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanCard</t>
+          <t>PrepaidPlanStep</t>
         </is>
       </c>
       <c r="C88" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanCard.tsx</t>
+          <t>components/patterns/PrepaidPlanStep.tsx</t>
         </is>
       </c>
       <c r="D88" s="20" t="inlineStr">
@@ -5028,11 +5002,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G88" s="17" t="inlineStr">
-        <is>
-          <t>PrepaidPlanStep</t>
-        </is>
-      </c>
+      <c r="G88" s="17" t="inlineStr"/>
       <c r="H88" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -5047,12 +5017,12 @@
       </c>
       <c r="B89" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanStep</t>
+          <t>SummaryTables</t>
         </is>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanStep.tsx</t>
+          <t>components/patterns/CheckoutSummaryTables.tsx</t>
         </is>
       </c>
       <c r="D89" s="20" t="inlineStr">
@@ -5068,10 +5038,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G89" s="17" t="inlineStr"/>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
+        </is>
+      </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5083,12 +5057,12 @@
       </c>
       <c r="B90" s="17" t="inlineStr">
         <is>
-          <t>SummaryTables</t>
+          <t>WinCashPaymentStep</t>
         </is>
       </c>
       <c r="C90" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryTables.tsx</t>
+          <t>components/patterns/WinCashPaymentStep.tsx</t>
         </is>
       </c>
       <c r="D90" s="20" t="inlineStr">
@@ -5104,11 +5078,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G90" s="17" t="inlineStr">
-        <is>
-          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
-        </is>
-      </c>
+      <c r="G90" s="17" t="inlineStr"/>
       <c r="H90" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5123,12 +5093,12 @@
       </c>
       <c r="B91" s="17" t="inlineStr">
         <is>
-          <t>WinCashPaymentStep</t>
+          <t>ZsbAddressStep</t>
         </is>
       </c>
       <c r="C91" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/WinCashPaymentStep.tsx</t>
+          <t>components/patterns/ZsbAddressStep.tsx</t>
         </is>
       </c>
       <c r="D91" s="20" t="inlineStr">
@@ -5147,7 +5117,7 @@
       <c r="G91" s="17" t="inlineStr"/>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5159,12 +5129,12 @@
       </c>
       <c r="B92" s="17" t="inlineStr">
         <is>
-          <t>ZsbAddressStep</t>
+          <t>AppointmentBookingStep</t>
         </is>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ZsbAddressStep.tsx</t>
+          <t>components/patterns/AppointmentBookingStep.tsx</t>
         </is>
       </c>
       <c r="D92" s="20" t="inlineStr">
@@ -5173,11 +5143,11 @@
         </is>
       </c>
       <c r="E92" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F92" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
         </is>
       </c>
       <c r="G92" s="17" t="inlineStr"/>
@@ -5195,12 +5165,12 @@
       </c>
       <c r="B93" s="17" t="inlineStr">
         <is>
-          <t>AppointmentBookingStep</t>
+          <t>DemoFaultPanel</t>
         </is>
       </c>
       <c r="C93" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/AppointmentBookingStep.tsx</t>
+          <t>components/patterns/DemoFaultPanel.tsx</t>
         </is>
       </c>
       <c r="D93" s="20" t="inlineStr">
@@ -5209,17 +5179,17 @@
         </is>
       </c>
       <c r="E93" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G93" s="17" t="inlineStr"/>
       <c r="H93" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5231,12 +5201,12 @@
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel</t>
+          <t>DonorAttachmentStep</t>
         </is>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DemoFaultPanel.tsx</t>
+          <t>components/patterns/DonorAttachmentStep.tsx</t>
         </is>
       </c>
       <c r="D94" s="20" t="inlineStr">
@@ -5267,12 +5237,12 @@
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>DonorAttachmentStep</t>
+          <t>DonorDetailsStep</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorAttachmentStep.tsx</t>
+          <t>components/patterns/DonorDetailsStep.tsx</t>
         </is>
       </c>
       <c r="D95" s="20" t="inlineStr">
@@ -5288,7 +5258,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
-      <c r="G95" s="17" t="inlineStr"/>
+      <c r="G95" s="17" t="inlineStr">
+        <is>
+          <t>DonorAttachmentStep</t>
+        </is>
+      </c>
       <c r="H95" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5303,12 +5277,12 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>DonorDetailsStep</t>
+          <t>EntityMissing</t>
         </is>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorDetailsStep.tsx</t>
+          <t>components/patterns/EntityMissing.tsx</t>
         </is>
       </c>
       <c r="D96" s="20" t="inlineStr">
@@ -5321,14 +5295,10 @@
       </c>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
-        </is>
-      </c>
-      <c r="G96" s="17" t="inlineStr">
-        <is>
-          <t>DonorAttachmentStep</t>
-        </is>
-      </c>
+          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
+        </is>
+      </c>
+      <c r="G96" s="17" t="inlineStr"/>
       <c r="H96" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5343,12 +5313,12 @@
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>EntityMissing</t>
+          <t>ActivityCommentsStep</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/EntityMissing.tsx</t>
+          <t>components/patterns/ActivityCommentsStep.tsx</t>
         </is>
       </c>
       <c r="D97" s="20" t="inlineStr">
@@ -5357,17 +5327,17 @@
         </is>
       </c>
       <c r="E97" s="17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
+          <t>pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G97" s="17" t="inlineStr"/>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5379,12 +5349,12 @@
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>ActivityCommentsStep</t>
+          <t>TicketCreationModal</t>
         </is>
       </c>
       <c r="C98" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ActivityCommentsStep.tsx</t>
+          <t>components/patterns/TicketCreationModal.tsx</t>
         </is>
       </c>
       <c r="D98" s="20" t="inlineStr">
@@ -5397,13 +5367,13 @@
       </c>
       <c r="F98" s="17" t="inlineStr">
         <is>
-          <t>pre-to-post-migration, sim-number-management, administration</t>
+          <t>trouble-ticketing-complaints, customer360, support</t>
         </is>
       </c>
       <c r="G98" s="17" t="inlineStr"/>
       <c r="H98" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5415,25 +5385,25 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>TicketCreationModal</t>
+          <t>BulkOperationPortal</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/TicketCreationModal.tsx</t>
-        </is>
-      </c>
-      <c r="D99" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/patterns/BulkOperationPortal.tsx</t>
+        </is>
+      </c>
+      <c r="D99" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E99" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, customer360, support</t>
+          <t>enterprise-iot-b2b</t>
         </is>
       </c>
       <c r="G99" s="17" t="inlineStr"/>
@@ -5451,12 +5421,12 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>BulkOperationPortal</t>
+          <t>DualPlaySerialCheckStep</t>
         </is>
       </c>
       <c r="C100" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BulkOperationPortal.tsx</t>
+          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
         </is>
       </c>
       <c r="D100" s="21" t="inlineStr">
@@ -5469,7 +5439,7 @@
       </c>
       <c r="F100" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b</t>
+          <t>fwa-5g-home</t>
         </is>
       </c>
       <c r="G100" s="17" t="inlineStr"/>
@@ -5487,12 +5457,12 @@
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>DualPlaySerialCheckStep</t>
+          <t>SimSwapFormStep</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
+          <t>components/patterns/SimSwapFormStep.tsx</t>
         </is>
       </c>
       <c r="D101" s="21" t="inlineStr">
@@ -5505,7 +5475,7 @@
       </c>
       <c r="F101" s="17" t="inlineStr">
         <is>
-          <t>fwa-5g-home</t>
+          <t>sim-number-management</t>
         </is>
       </c>
       <c r="G101" s="17" t="inlineStr"/>
@@ -5523,12 +5493,12 @@
       </c>
       <c r="B102" s="17" t="inlineStr">
         <is>
-          <t>SimSwapFormStep</t>
+          <t>VerificationGate</t>
         </is>
       </c>
       <c r="C102" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/SimSwapFormStep.tsx</t>
+          <t>components/patterns/VerificationGate.tsx</t>
         </is>
       </c>
       <c r="D102" s="21" t="inlineStr">
@@ -5541,7 +5511,7 @@
       </c>
       <c r="F102" s="17" t="inlineStr">
         <is>
-          <t>sim-number-management</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G102" s="17" t="inlineStr"/>
@@ -5554,30 +5524,30 @@
     <row r="103">
       <c r="A103" s="17" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Wizard</t>
         </is>
       </c>
       <c r="B103" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>AbandonDialog</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/VerificationGate.tsx</t>
-        </is>
-      </c>
-      <c r="D103" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/patterns/wizard/WizardDialogs.tsx</t>
+        </is>
+      </c>
+      <c r="D103" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E103" s="17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G103" s="17" t="inlineStr"/>
@@ -5595,12 +5565,12 @@
       </c>
       <c r="B104" s="17" t="inlineStr">
         <is>
-          <t>AbandonDialog</t>
+          <t>CustomerMirrorPanel</t>
         </is>
       </c>
       <c r="C104" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardDialogs.tsx</t>
+          <t>components/patterns/wizard/CustomerMirrorPanel.tsx</t>
         </is>
       </c>
       <c r="D104" s="20" t="inlineStr">
@@ -5609,11 +5579,11 @@
         </is>
       </c>
       <c r="E104" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F104" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G104" s="17" t="inlineStr"/>
@@ -5631,12 +5601,12 @@
       </c>
       <c r="B105" s="17" t="inlineStr">
         <is>
-          <t>CustomerMirrorPanel</t>
+          <t>StepSummaryPanel</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/CustomerMirrorPanel.tsx</t>
+          <t>components/patterns/wizard/StepSummaryPanel.tsx</t>
         </is>
       </c>
       <c r="D105" s="20" t="inlineStr">
@@ -5645,17 +5615,17 @@
         </is>
       </c>
       <c r="E105" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F105" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G105" s="17" t="inlineStr"/>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5667,31 +5637,35 @@
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
+          <t>StepSummarySection</t>
+        </is>
+      </c>
+      <c r="C106" s="17" t="inlineStr">
+        <is>
+          <t>components/patterns/wizard/StepSummarySection.tsx</t>
+        </is>
+      </c>
+      <c r="D106" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E106" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F106" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G106" s="17" t="inlineStr">
+        <is>
           <t>StepSummaryPanel</t>
         </is>
       </c>
-      <c r="C106" s="17" t="inlineStr">
-        <is>
-          <t>components/patterns/wizard/StepSummaryPanel.tsx</t>
-        </is>
-      </c>
-      <c r="D106" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
-        </is>
-      </c>
-      <c r="E106" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="F106" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
-        </is>
-      </c>
-      <c r="G106" s="17" t="inlineStr"/>
       <c r="H106" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5703,12 +5677,12 @@
       </c>
       <c r="B107" s="17" t="inlineStr">
         <is>
-          <t>StepSummarySection</t>
+          <t>SummaryFieldRow</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/StepSummarySection.tsx</t>
+          <t>components/patterns/wizard/SummaryFieldRow.tsx</t>
         </is>
       </c>
       <c r="D107" s="20" t="inlineStr">
@@ -5717,11 +5691,11 @@
         </is>
       </c>
       <c r="E107" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F107" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G107" s="17" t="inlineStr">
@@ -5731,7 +5705,7 @@
       </c>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5743,12 +5717,12 @@
       </c>
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>SummaryFieldRow</t>
+          <t>WizardFooter</t>
         </is>
       </c>
       <c r="C108" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/SummaryFieldRow.tsx</t>
+          <t>components/patterns/wizard/WizardFooter.tsx</t>
         </is>
       </c>
       <c r="D108" s="20" t="inlineStr">
@@ -5757,21 +5731,17 @@
         </is>
       </c>
       <c r="E108" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F108" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
-        </is>
-      </c>
-      <c r="G108" s="17" t="inlineStr">
-        <is>
-          <t>StepSummaryPanel</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G108" s="17" t="inlineStr"/>
       <c r="H108" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5783,12 +5753,12 @@
       </c>
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>WizardFooter</t>
+          <t>WizardStepHeader</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardFooter.tsx</t>
+          <t>components/patterns/wizard/WizardStepHeader.tsx</t>
         </is>
       </c>
       <c r="D109" s="20" t="inlineStr">
@@ -5797,11 +5767,11 @@
         </is>
       </c>
       <c r="E109" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F109" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G109" s="17" t="inlineStr"/>
@@ -5819,12 +5789,12 @@
       </c>
       <c r="B110" s="17" t="inlineStr">
         <is>
-          <t>WizardStepHeader</t>
+          <t>WizardTitleBand</t>
         </is>
       </c>
       <c r="C110" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardStepHeader.tsx</t>
+          <t>components/patterns/wizard/WizardTitleBand.tsx</t>
         </is>
       </c>
       <c r="D110" s="20" t="inlineStr">
@@ -5833,58 +5803,22 @@
         </is>
       </c>
       <c r="E110" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F110" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G110" s="17" t="inlineStr"/>
       <c r="H110" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
-        </is>
-      </c>
-    </row>
-    <row r="111">
-      <c r="A111" s="17" t="inlineStr">
-        <is>
-          <t>Wizard</t>
-        </is>
-      </c>
-      <c r="B111" s="17" t="inlineStr">
-        <is>
-          <t>WizardTitleBand</t>
-        </is>
-      </c>
-      <c r="C111" s="17" t="inlineStr">
-        <is>
-          <t>components/patterns/wizard/WizardTitleBand.tsx</t>
-        </is>
-      </c>
-      <c r="D111" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
-        </is>
-      </c>
-      <c r="E111" s="17" t="n">
-        <v>9</v>
-      </c>
-      <c r="F111" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
-        </is>
-      </c>
-      <c r="G111" s="17" t="inlineStr"/>
-      <c r="H111" s="17" t="inlineStr">
-        <is>
           <t>2026-10-18</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H111"/>
+  <autoFilter ref="A1:H110"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -7269,7 +7203,7 @@
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, configStore</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, AppointmentBookingStep, configStore</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
@@ -7300,11 +7234,11 @@
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, navigation</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
         </is>
       </c>
       <c r="G37" s="17" t="inlineStr">
@@ -7854,12 +7788,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>connectionType</t>
+          <t>taskId</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>lib/connectionType.ts</t>
+          <t>lib/taskId.ts</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
@@ -7868,16 +7802,16 @@
         </is>
       </c>
       <c r="E52" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G52" s="17" t="inlineStr">
         <is>
-          <t>ConnectionTypeTag</t>
+          <t>useWizardDraftActions</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
@@ -7894,12 +7828,12 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>taskId</t>
+          <t>connectionType</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>lib/taskId.ts</t>
+          <t>lib/connectionType.ts</t>
         </is>
       </c>
       <c r="D53" s="20" t="inlineStr">
@@ -7912,12 +7846,12 @@
       </c>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration, customer360</t>
         </is>
       </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
-          <t>useWizardDraftActions</t>
+          <t>ConnectionTypeTag</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">

</xml_diff>

<commit_message>
Wire the eligibility rule engine into the journeys
The Eligibility Gate asks src/domain/eligibility (through engines/connectionEligibility) for the line-count decision: a block is a hard stop, approvals are approval routing, Credit Control approval routes the order to Credit Control, orders keep the decision for the approver, MNP orders are held for engine approvals. Replaces BR-288/BR-347 for QID and Passport; other ID types keep the older check.

Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -14,8 +14,8 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Legend &amp; Method" sheetId="5" state="visible" r:id="rId5"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$111</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$57</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$114</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$60</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -667,10 +667,10 @@
         </is>
       </c>
       <c r="C5" s="17" t="n">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="D5" s="17" t="n">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="E5" s="17" t="n">
         <v>2</v>
@@ -691,10 +691,10 @@
         </is>
       </c>
       <c r="C6" s="17" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="D6" s="17" t="n">
-        <v>17</v>
+        <v>18</v>
       </c>
       <c r="E6" s="17" t="n">
         <v>3</v>
@@ -739,10 +739,10 @@
         </is>
       </c>
       <c r="C8" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="D8" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="E8" s="17" t="n">
         <v>0</v>
@@ -763,10 +763,10 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>4</v>
@@ -835,10 +835,10 @@
         </is>
       </c>
       <c r="C12" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="D12" s="17" t="n">
         <v>7</v>
-      </c>
-      <c r="D12" s="17" t="n">
-        <v>5</v>
       </c>
       <c r="E12" s="17" t="n">
         <v>2</v>
@@ -855,14 +855,14 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>110 UI components + 56 non-UI files</t>
+          <t>113 UI components + 59 non-UI files</t>
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>166</v>
+        <v>172</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>140</v>
+        <v>146</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>21</v>
@@ -1616,7 +1616,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H111"/>
+  <dimension ref="A1:H114"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="14.85" customWidth="1" min="1" max="1"/>
@@ -1702,7 +1702,7 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>CreditCheckPanel, MsisdnPicker, SimTypeStep, ActivationCompleteScreen, AppointmentBookingStep, BillingAccountStep, BulkOperationPortal, CafSignatureCapture, DonorAttachmentStep, IdLookupStep, LineSelectionStep, PrepaidCartStep, PrepaidCheckoutStep, SimSwapFormStep, TicketCreationModal, WinCashPaymentStep, ConnectionTypeTag, Tooltip</t>
+          <t>CreditCheckPanel, MsisdnPicker, SimTypeStep, ActivationCompleteScreen, AppointmentBookingStep, BillingAccountStep, BulkOperationPortal, CafSignatureCapture, DonorAttachmentStep, IdLookupStep, PrepaidCartStep, PrepaidCheckoutStep, SimSwapFormStep, TicketCreationModal, WinCashPaymentStep, ConnectionTypeTag, Tooltip</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
@@ -1742,7 +1742,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ValidationStatus, ZsbAddressStep, StepSummarySection, WizardFooter, WizardStepHeader, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, ScanFailureNotice, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ValidationStatus, ZsbAddressStep, CustomerViewButton, StepSummarySection, WizardFooter, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
@@ -1782,7 +1782,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>ErrorBoundary, AdditionalDocumentsUpload, BillLimitEditor, CafDocumentUpload, EligibilityRows, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, SimTypeStep, SupportingDocumentUpload, ActivationCompleteScreen, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CafSignatureCapture, CheckoutDefaultLayout, DemoFaultPanel, FixedPlanStep, IdLookupStatus, OrderConfirmationScreen, PostpaidDiscountsPanel, PostpaidPlanCard, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPackDetailsDrawer, PrepaidPlanCard, TicketCreationModal, ValidationStatus, VerificationGate, WinCashPaymentStep, ZsbAddressStep, StepSummarySection, SummaryFieldRow, WizardDialogs, WizardFooter, WizardStepHeader, WizardTitleBand, SignaturePad</t>
+          <t>ErrorBoundary, AdditionalDocumentsUpload, BillLimitEditor, CafDocumentUpload, EligibilityRows, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, SimTypeStep, SupportingDocumentUpload, ActivationCompleteScreen, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CafSignatureCapture, CheckoutDefaultLayout, DemoFaultPanel, FixedPlanStep, IdLookupStatus, OrderConfirmationScreen, PostpaidDiscountsPanel, PostpaidPlanCard, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPackDetailsDrawer, PrepaidPlanCard, TicketCreationModal, ValidationStatus, VerificationGate, WinCashPaymentStep, ZsbAddressStep, CustomerViewButton, StepSummarySection, SummaryFieldRow, WizardDialogs, WizardFooter, WizardTitleBand, SignaturePad</t>
         </is>
       </c>
       <c r="H4" s="17" t="inlineStr">
@@ -1822,7 +1822,7 @@
       </c>
       <c r="G5" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, DonorAttachmentStep, DonorDetailsStep, GuidedContactStep, TicketCreationModal, ZsbAddressStep</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, DonorDetailsStep, GuidedContactStep, TicketCreationModal, ZsbAddressStep</t>
         </is>
       </c>
       <c r="H5" s="17" t="inlineStr">
@@ -1982,7 +1982,7 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>WizardStepHeader, CloseButton, Tabs</t>
+          <t>CustomerViewButton, CloseButton, Tabs</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
@@ -2262,12 +2262,12 @@
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
+          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2462,7 +2462,7 @@
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>ContactPhoneInput, GuidedContactStep</t>
+          <t>ContactPhoneInput, DonorDetailsStep, GuidedContactStep</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
@@ -2627,7 +2627,7 @@
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2679,12 +2679,12 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>ChoiceCards</t>
+          <t>ServiceTypeTag</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/ChoiceCards.tsx</t>
+          <t>components/primitives/ServiceTypeTag.tsx</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
@@ -2693,17 +2693,21 @@
         </is>
       </c>
       <c r="E27" s="17" t="n">
-        <v>6</v>
+        <v>10</v>
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
-        </is>
-      </c>
-      <c r="G27" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G27" s="17" t="inlineStr">
+        <is>
+          <t>LineSelectionStep, ConnectionTypeTag</t>
+        </is>
+      </c>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2715,12 +2719,12 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>PanelIcon</t>
+          <t>ChoiceCards</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/PanelIcon.tsx</t>
+          <t>components/primitives/ChoiceCards.tsx</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -2733,17 +2737,13 @@
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, navigation, administration, customer360, orders, support</t>
-        </is>
-      </c>
-      <c r="G28" s="17" t="inlineStr">
-        <is>
-          <t>Tabs</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr"/>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2755,12 +2755,12 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>PanelIcon</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/Radio.tsx</t>
+          <t>components/primitives/PanelIcon.tsx</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
@@ -2773,10 +2773,14 @@
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr"/>
+          <t>trouble-ticketing-complaints, navigation, administration, customer360, orders, support</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr">
+        <is>
+          <t>Tabs</t>
+        </is>
+      </c>
       <c r="H29" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -2791,12 +2795,12 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Tabs</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/Tabs.tsx</t>
+          <t>components/primitives/Radio.tsx</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
@@ -2805,17 +2809,17 @@
         </is>
       </c>
       <c r="E30" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, administration, customer360, orders, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G30" s="17" t="inlineStr"/>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2827,31 +2831,31 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>VodafoneMark</t>
+          <t>Tabs</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/VodafoneMark.tsx</t>
-        </is>
-      </c>
-      <c r="D31" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/primitives/Tabs.tsx</t>
+        </is>
+      </c>
+      <c r="D31" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E31" s="17" t="n">
-        <v>1</v>
+        <v>5</v>
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>trouble-ticketing-complaints, administration, customer360, orders, support</t>
         </is>
       </c>
       <c r="G31" s="17" t="inlineStr"/>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2863,12 +2867,12 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>VodafoneWordmark</t>
+          <t>VodafoneMark</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/VodafoneWordmark.tsx</t>
+          <t>components/primitives/VodafoneMark.tsx</t>
         </is>
       </c>
       <c r="D32" s="21" t="inlineStr">
@@ -2899,27 +2903,31 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>LocationInput</t>
+          <t>VodafoneWordmark</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/LocationInput.tsx</t>
-        </is>
-      </c>
-      <c r="D33" s="22" t="inlineStr">
-        <is>
-          <t>No consumer</t>
+          <t>components/primitives/VodafoneWordmark.tsx</t>
+        </is>
+      </c>
+      <c r="D33" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E33" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F33" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F33" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G33" s="17" t="inlineStr"/>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2931,17 +2939,17 @@
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>OoredooMark</t>
+          <t>LocationInput</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/OoredooMark.tsx</t>
-        </is>
-      </c>
-      <c r="D34" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>components/primitives/LocationInput.tsx</t>
+        </is>
+      </c>
+      <c r="D34" s="22" t="inlineStr">
+        <is>
+          <t>No consumer</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
@@ -2951,44 +2959,36 @@
       <c r="G34" s="17" t="inlineStr"/>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" s="17" t="inlineStr">
         <is>
-          <t>Domain</t>
+          <t>Primitive</t>
         </is>
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>ScannedIdPreview</t>
+          <t>OoredooMark</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>components/domain/ScannedIdPreview.tsx</t>
-        </is>
-      </c>
-      <c r="D35" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/primitives/OoredooMark.tsx</t>
+        </is>
+      </c>
+      <c r="D35" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>13</v>
-      </c>
-      <c r="F35" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G35" s="17" t="inlineStr">
-        <is>
-          <t>PassportScanSections, QidImageUpload, qidImageUploadModel, IdScannerPanel, useIdLookup</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F35" s="17" t="inlineStr"/>
+      <c r="G35" s="17" t="inlineStr"/>
       <c r="H35" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -3003,12 +3003,12 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>PassportScanSections</t>
+          <t>ScannedIdPreview</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>components/domain/PassportScanSections.tsx</t>
+          <t>components/domain/ScannedIdPreview.tsx</t>
         </is>
       </c>
       <c r="D36" s="20" t="inlineStr">
@@ -3017,16 +3017,16 @@
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>QidImageUpload</t>
+          <t>PassportScanSections, QidImageUpload, qidImageUploadModel, IdScannerPanel, useIdLookup</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
@@ -3043,12 +3043,12 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>QidImageUpload</t>
+          <t>PassportScanSections</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>components/domain/QidImageUpload.tsx</t>
+          <t>components/domain/PassportScanSections.tsx</t>
         </is>
       </c>
       <c r="D37" s="20" t="inlineStr">
@@ -3066,12 +3066,12 @@
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>IdScannerPanel</t>
+          <t>QidImageUpload</t>
         </is>
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3083,12 +3083,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>QidTypeSelector</t>
+          <t>QidImageUpload</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>components/domain/QidInput.tsx</t>
+          <t>components/domain/QidImageUpload.tsx</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
@@ -3106,12 +3106,12 @@
       </c>
       <c r="G38" s="17" t="inlineStr">
         <is>
-          <t>GuidedContactStep, IdLookupStep, IdScannerPanel, MoiResultPanel, guidedContactModel, idLookupModel, useIdLookup</t>
+          <t>IdScannerPanel</t>
         </is>
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3123,12 +3123,12 @@
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>SimSerialScanner</t>
+          <t>QidTypeSelector</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>components/domain/SimSerialScanner.tsx</t>
+          <t>components/domain/QidInput.tsx</t>
         </is>
       </c>
       <c r="D39" s="20" t="inlineStr">
@@ -3137,21 +3137,21 @@
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>10</v>
+        <v>12</v>
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>SimTypeStep</t>
+          <t>GuidedContactStep, IdLookupStep, IdScannerPanel, MoiResultPanel, guidedContactModel, idLookupModel, useIdLookup</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3163,12 +3163,12 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload</t>
+          <t>ScanFailureNotice</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>components/domain/AdditionalDocumentsUpload.tsx</t>
+          <t>components/domain/ScanFailureNotice.tsx</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
@@ -3177,21 +3177,21 @@
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture</t>
+          <t>PassportScanSections, QidImageUpload</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3203,12 +3203,12 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>BillLimitEditor</t>
+          <t>SimSerialScanner</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>components/domain/BillLimitEditor.tsx</t>
+          <t>components/domain/SimSerialScanner.tsx</t>
         </is>
       </c>
       <c r="D41" s="20" t="inlineStr">
@@ -3217,21 +3217,21 @@
         </is>
       </c>
       <c r="E41" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>PostpaidAddonsPanel, PostpaidPlanAddonsStep</t>
+          <t>SimTypeStep</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -3243,12 +3243,12 @@
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>CafDocumentUpload</t>
+          <t>AdditionalDocumentsUpload</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>components/domain/CafDocumentUpload.tsx</t>
+          <t>components/domain/AdditionalDocumentsUpload.tsx</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
@@ -3283,12 +3283,12 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput</t>
+          <t>BillLimitEditor</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>components/domain/CompanySearchInput.tsx</t>
+          <t>components/domain/BillLimitEditor.tsx</t>
         </is>
       </c>
       <c r="D43" s="20" t="inlineStr">
@@ -3304,7 +3304,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G43" s="17" t="inlineStr"/>
+      <c r="G43" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidAddonsPanel, PostpaidPlanAddonsStep</t>
+        </is>
+      </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -3319,12 +3323,12 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>CreditCheckPanel</t>
+          <t>CafDocumentUpload</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>components/domain/CreditCheckPanel.tsx</t>
+          <t>components/domain/CafDocumentUpload.tsx</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
@@ -3342,7 +3346,7 @@
       </c>
       <c r="G44" s="17" t="inlineStr">
         <is>
-          <t>FixedPlanStep</t>
+          <t>CafSignatureCapture</t>
         </is>
       </c>
       <c r="H44" s="17" t="inlineStr">
@@ -3359,12 +3363,12 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>EligibilityChecksList</t>
+          <t>CompanySearchInput</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>components/domain/EligibilityRows.tsx</t>
+          <t>components/domain/CompanySearchInput.tsx</t>
         </is>
       </c>
       <c r="D45" s="20" t="inlineStr">
@@ -3395,12 +3399,12 @@
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>EsimActivationPanel</t>
+          <t>CreditCheckPanel</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>components/domain/EsimActivationPanel.tsx</t>
+          <t>components/domain/CreditCheckPanel.tsx</t>
         </is>
       </c>
       <c r="D46" s="20" t="inlineStr">
@@ -3418,12 +3422,12 @@
       </c>
       <c r="G46" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>FixedPlanStep</t>
         </is>
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -3435,12 +3439,12 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker</t>
+          <t>EligibilityChecksList</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>components/domain/MsisdnPicker.tsx</t>
+          <t>components/domain/EligibilityRows.tsx</t>
         </is>
       </c>
       <c r="D47" s="20" t="inlineStr">
@@ -3453,7 +3457,7 @@
       </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr"/>
@@ -3471,12 +3475,12 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>SimTypeStep</t>
+          <t>EsimActivationPanel</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>components/domain/SimTypeStep.tsx</t>
+          <t>components/domain/EsimActivationPanel.tsx</t>
         </is>
       </c>
       <c r="D48" s="20" t="inlineStr">
@@ -3494,7 +3498,7 @@
       </c>
       <c r="G48" s="17" t="inlineStr">
         <is>
-          <t>CheckoutSummaryStep, checkoutDetailedTables, checkoutSummaryRows, prepaidCartModel, useCheckoutSummary</t>
+          <t>ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="H48" s="17" t="inlineStr">
@@ -3511,12 +3515,12 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>StarStat</t>
+          <t>MsisdnPicker</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>components/domain/StarStat.tsx</t>
+          <t>components/domain/MsisdnPicker.tsx</t>
         </is>
       </c>
       <c r="D49" s="20" t="inlineStr">
@@ -3532,11 +3536,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
-      <c r="G49" s="17" t="inlineStr">
-        <is>
-          <t>MsisdnPicker</t>
-        </is>
-      </c>
+      <c r="G49" s="17" t="inlineStr"/>
       <c r="H49" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -3551,12 +3551,12 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>SupportingDocumentUpload</t>
+          <t>SimTypeStep</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>components/domain/SupportingDocumentUpload.tsx</t>
+          <t>components/domain/SimTypeStep.tsx</t>
         </is>
       </c>
       <c r="D50" s="20" t="inlineStr">
@@ -3572,10 +3572,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G50" s="17" t="inlineStr"/>
+      <c r="G50" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep, checkoutDetailedTables, checkoutSummaryRows, prepaidCartModel, useCheckoutSummary</t>
+        </is>
+      </c>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3587,12 +3591,12 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>FibreReadinessBanner</t>
+          <t>StarStat</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>components/domain/FibreReadinessBanner.tsx</t>
+          <t>components/domain/StarStat.tsx</t>
         </is>
       </c>
       <c r="D51" s="20" t="inlineStr">
@@ -3601,16 +3605,16 @@
         </is>
       </c>
       <c r="E51" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F51" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G51" s="17" t="inlineStr">
         <is>
-          <t>ZsbAddressStep</t>
+          <t>MsisdnPicker</t>
         </is>
       </c>
       <c r="H51" s="17" t="inlineStr">
@@ -3627,31 +3631,31 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>ContactPhoneInput</t>
+          <t>SupportingDocumentUpload</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>components/domain/ContactPhoneInput.tsx</t>
-        </is>
-      </c>
-      <c r="D52" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/domain/SupportingDocumentUpload.tsx</t>
+        </is>
+      </c>
+      <c r="D52" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E52" s="17" t="n">
-        <v>1</v>
+        <v>9</v>
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G52" s="17" t="inlineStr"/>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -3663,35 +3667,35 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>CpeSerialScanner</t>
+          <t>FibreReadinessBanner</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>components/domain/CpeSerialScanner.tsx</t>
-        </is>
-      </c>
-      <c r="D53" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/domain/FibreReadinessBanner.tsx</t>
+        </is>
+      </c>
+      <c r="D53" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E53" s="17" t="n">
-        <v>1</v>
+        <v>8</v>
       </c>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>fwa-5g-home</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
-          <t>DualPlaySerialCheckStep</t>
+          <t>ZsbAddressStep</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3703,12 +3707,12 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>OsmEmbed</t>
+          <t>ContactPhoneInput</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>components/domain/OsmEmbed.tsx</t>
+          <t>components/domain/ContactPhoneInput.tsx</t>
         </is>
       </c>
       <c r="D54" s="21" t="inlineStr">
@@ -3727,79 +3731,83 @@
       <c r="G54" s="17" t="inlineStr"/>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
     <row r="55">
       <c r="A55" s="17" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>PageHeader</t>
+          <t>CpeSerialScanner</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PageHeader.tsx</t>
-        </is>
-      </c>
-      <c r="D55" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/domain/CpeSerialScanner.tsx</t>
+        </is>
+      </c>
+      <c r="D55" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E55" s="17" t="n">
-        <v>18</v>
+        <v>1</v>
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fwa-5g-home, lead-management, mnp-fnp-porting, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G55" s="17" t="inlineStr"/>
+          <t>fwa-5g-home</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>DualPlaySerialCheckStep</t>
+        </is>
+      </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
     <row r="56">
       <c r="A56" s="17" t="inlineStr">
         <is>
-          <t>Pattern</t>
+          <t>Domain</t>
         </is>
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>GuidedContactStep</t>
+          <t>OsmEmbed</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/GuidedContactStep.tsx</t>
-        </is>
-      </c>
-      <c r="D56" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/domain/OsmEmbed.tsx</t>
+        </is>
+      </c>
+      <c r="D56" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
-        <v>12</v>
+        <v>1</v>
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G56" s="17" t="inlineStr"/>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -3811,12 +3819,12 @@
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStatus</t>
+          <t>PageHeader</t>
         </is>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/IdLookupStatus.tsx</t>
+          <t>components/patterns/PageHeader.tsx</t>
         </is>
       </c>
       <c r="D57" s="20" t="inlineStr">
@@ -3825,21 +3833,17 @@
         </is>
       </c>
       <c r="E57" s="17" t="n">
-        <v>12</v>
+        <v>18</v>
       </c>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G57" s="17" t="inlineStr">
-        <is>
-          <t>IdLookupStep</t>
-        </is>
-      </c>
+          <t>enterprise-iot-b2b, fwa-5g-home, lead-management, mnp-fnp-porting, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr"/>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3851,12 +3855,12 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStep</t>
+          <t>GuidedContactStep</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/IdLookupStep.tsx</t>
+          <t>components/patterns/GuidedContactStep.tsx</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
@@ -3872,14 +3876,10 @@
           <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
-      <c r="G58" s="17" t="inlineStr">
-        <is>
-          <t>GuidedContactStep</t>
-        </is>
-      </c>
+      <c r="G58" s="17" t="inlineStr"/>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -3891,12 +3891,12 @@
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>IdScannerPanel</t>
+          <t>IdLookupStatus</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/IdScannerPanel.tsx</t>
+          <t>components/patterns/IdLookupStatus.tsx</t>
         </is>
       </c>
       <c r="D59" s="20" t="inlineStr">
@@ -3931,12 +3931,12 @@
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>MoiResultPanel</t>
+          <t>IdLookupStep</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/MoiResultPanel.tsx</t>
+          <t>components/patterns/IdLookupStep.tsx</t>
         </is>
       </c>
       <c r="D60" s="20" t="inlineStr">
@@ -3954,12 +3954,12 @@
       </c>
       <c r="G60" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStep</t>
+          <t>GuidedContactStep</t>
         </is>
       </c>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -3971,12 +3971,12 @@
       </c>
       <c r="B61" s="17" t="inlineStr">
         <is>
-          <t>ValidationStatus</t>
+          <t>IdScannerPanel</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ValidationStatus.tsx</t>
+          <t>components/patterns/IdScannerPanel.tsx</t>
         </is>
       </c>
       <c r="D61" s="20" t="inlineStr">
@@ -3994,12 +3994,12 @@
       </c>
       <c r="G61" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStatus</t>
+          <t>IdLookupStep</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4011,12 +4011,12 @@
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>SignatureCapture</t>
+          <t>MoiResultPanel</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/SignatureCapture.tsx</t>
+          <t>components/patterns/MoiResultPanel.tsx</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr">
@@ -4025,21 +4025,21 @@
         </is>
       </c>
       <c r="E62" s="17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G62" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture, DonorAttachmentStep, SimSwapFormStep</t>
+          <t>IdLookupStep</t>
         </is>
       </c>
       <c r="H62" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4051,12 +4051,12 @@
       </c>
       <c r="B63" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>ValidationStatus</t>
         </is>
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ActivationCompleteScreen.tsx</t>
+          <t>components/patterns/ValidationStatus.tsx</t>
         </is>
       </c>
       <c r="D63" s="20" t="inlineStr">
@@ -4065,17 +4065,21 @@
         </is>
       </c>
       <c r="E63" s="17" t="n">
-        <v>9</v>
+        <v>12</v>
       </c>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G63" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G63" s="17" t="inlineStr">
+        <is>
+          <t>IdLookupStatus</t>
+        </is>
+      </c>
       <c r="H63" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4087,12 +4091,12 @@
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountAutoResolver</t>
+          <t>SignatureCapture</t>
         </is>
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingAccountAutoResolver.tsx</t>
+          <t>components/patterns/SignatureCapture.tsx</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr">
@@ -4101,17 +4105,21 @@
         </is>
       </c>
       <c r="E64" s="17" t="n">
-        <v>9</v>
+        <v>11</v>
       </c>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G64" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>CafSignatureCapture, DonorAttachmentStep, SimSwapFormStep</t>
+        </is>
+      </c>
       <c r="H64" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4123,12 +4131,12 @@
       </c>
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture</t>
+          <t>ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafSignatureCapture.tsx</t>
+          <t>components/patterns/ActivationCompleteScreen.tsx</t>
         </is>
       </c>
       <c r="D65" s="20" t="inlineStr">
@@ -4159,12 +4167,12 @@
       </c>
       <c r="B66" s="17" t="inlineStr">
         <is>
-          <t>CheckoutDefaultLayout</t>
+          <t>BillingAccountAutoResolver</t>
         </is>
       </c>
       <c r="C66" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
+          <t>components/patterns/BillingAccountAutoResolver.tsx</t>
         </is>
       </c>
       <c r="D66" s="20" t="inlineStr">
@@ -4180,14 +4188,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G66" s="17" t="inlineStr">
-        <is>
-          <t>CheckoutSummaryStep</t>
-        </is>
-      </c>
+      <c r="G66" s="17" t="inlineStr"/>
       <c r="H66" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4199,12 +4203,12 @@
       </c>
       <c r="B67" s="17" t="inlineStr">
         <is>
-          <t>CheckoutSummaryStep</t>
+          <t>CafSignatureCapture</t>
         </is>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryStep.tsx</t>
+          <t>components/patterns/CafSignatureCapture.tsx</t>
         </is>
       </c>
       <c r="D67" s="20" t="inlineStr">
@@ -4223,7 +4227,7 @@
       <c r="G67" s="17" t="inlineStr"/>
       <c r="H67" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4235,12 +4239,12 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>DiscountCard</t>
+          <t>CheckoutDefaultLayout</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DiscountCard.tsx</t>
+          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
         </is>
       </c>
       <c r="D68" s="20" t="inlineStr">
@@ -4258,12 +4262,12 @@
       </c>
       <c r="G68" s="17" t="inlineStr">
         <is>
-          <t>PostpaidDiscountsPanel</t>
+          <t>CheckoutSummaryStep</t>
         </is>
       </c>
       <c r="H68" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4275,12 +4279,12 @@
       </c>
       <c r="B69" s="17" t="inlineStr">
         <is>
-          <t>FixedPlanStep</t>
+          <t>CheckoutSummaryStep</t>
         </is>
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/FixedPlanStep.tsx</t>
+          <t>components/patterns/CheckoutSummaryStep.tsx</t>
         </is>
       </c>
       <c r="D69" s="20" t="inlineStr">
@@ -4299,7 +4303,7 @@
       <c r="G69" s="17" t="inlineStr"/>
       <c r="H69" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4311,12 +4315,12 @@
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>FullTerms</t>
+          <t>DiscountCard</t>
         </is>
       </c>
       <c r="C70" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafTerms.tsx</t>
+          <t>components/patterns/DiscountCard.tsx</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
@@ -4334,7 +4338,7 @@
       </c>
       <c r="G70" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture</t>
+          <t>PostpaidDiscountsPanel</t>
         </is>
       </c>
       <c r="H70" s="17" t="inlineStr">
@@ -4351,12 +4355,12 @@
       </c>
       <c r="B71" s="17" t="inlineStr">
         <is>
-          <t>KeyInformationPanel</t>
+          <t>FixedPlanStep</t>
         </is>
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/KeyInformationPanel.tsx</t>
+          <t>components/patterns/FixedPlanStep.tsx</t>
         </is>
       </c>
       <c r="D71" s="20" t="inlineStr">
@@ -4375,7 +4379,7 @@
       <c r="G71" s="17" t="inlineStr"/>
       <c r="H71" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4387,12 +4391,12 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>OrderConfirmationScreen</t>
+          <t>FullTerms</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/OrderConfirmationScreen.tsx</t>
+          <t>components/patterns/CafTerms.tsx</t>
         </is>
       </c>
       <c r="D72" s="20" t="inlineStr">
@@ -4410,12 +4414,12 @@
       </c>
       <c r="G72" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>CafSignatureCapture</t>
         </is>
       </c>
       <c r="H72" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4427,12 +4431,12 @@
       </c>
       <c r="B73" s="17" t="inlineStr">
         <is>
-          <t>PlanDetailsDrawer</t>
+          <t>KeyInformationPanel</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanDetailsDrawer.tsx</t>
+          <t>components/patterns/KeyInformationPanel.tsx</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
@@ -4448,11 +4452,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G73" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidPlanAddonsStep</t>
-        </is>
-      </c>
+      <c r="G73" s="17" t="inlineStr"/>
       <c r="H73" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -4467,12 +4467,12 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>PlanGroupPanel</t>
+          <t>OrderConfirmationScreen</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanGroupPanel.tsx</t>
+          <t>components/patterns/OrderConfirmationScreen.tsx</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
@@ -4490,12 +4490,12 @@
       </c>
       <c r="G74" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanAddonsStep</t>
+          <t>ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="H74" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4507,12 +4507,12 @@
       </c>
       <c r="B75" s="17" t="inlineStr">
         <is>
-          <t>PlanSearchBox</t>
+          <t>PlanDetailsDrawer</t>
         </is>
       </c>
       <c r="C75" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanSearchBox.tsx</t>
+          <t>components/patterns/PlanDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D75" s="20" t="inlineStr">
@@ -4547,12 +4547,12 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>PlanTabStrip</t>
+          <t>PlanGroupPanel</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanTabStrip.tsx</t>
+          <t>components/patterns/PlanGroupPanel.tsx</t>
         </is>
       </c>
       <c r="D76" s="20" t="inlineStr">
@@ -4575,7 +4575,7 @@
       </c>
       <c r="H76" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4587,12 +4587,12 @@
       </c>
       <c r="B77" s="17" t="inlineStr">
         <is>
-          <t>PostpaidAddonsPanel</t>
+          <t>PlanSearchBox</t>
         </is>
       </c>
       <c r="C77" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
+          <t>components/patterns/PlanSearchBox.tsx</t>
         </is>
       </c>
       <c r="D77" s="20" t="inlineStr">
@@ -4615,7 +4615,7 @@
       </c>
       <c r="H77" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4627,12 +4627,12 @@
       </c>
       <c r="B78" s="17" t="inlineStr">
         <is>
-          <t>PostpaidDiscountsPanel</t>
+          <t>PlanTabStrip</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
+          <t>components/patterns/PlanTabStrip.tsx</t>
         </is>
       </c>
       <c r="D78" s="20" t="inlineStr">
@@ -4655,7 +4655,7 @@
       </c>
       <c r="H78" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4667,12 +4667,12 @@
       </c>
       <c r="B79" s="17" t="inlineStr">
         <is>
-          <t>PostpaidMonthlySummary</t>
+          <t>PostpaidAddonsPanel</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
+          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
         </is>
       </c>
       <c r="D79" s="20" t="inlineStr">
@@ -4707,12 +4707,12 @@
       </c>
       <c r="B80" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanAddonsStep</t>
+          <t>PostpaidDiscountsPanel</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
+          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
         </is>
       </c>
       <c r="D80" s="20" t="inlineStr">
@@ -4728,10 +4728,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G80" s="17" t="inlineStr"/>
+      <c r="G80" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidPlanAddonsStep</t>
+        </is>
+      </c>
       <c r="H80" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4743,12 +4747,12 @@
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanCard</t>
+          <t>PostpaidMonthlySummary</t>
         </is>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanCard.tsx</t>
+          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
         </is>
       </c>
       <c r="D81" s="20" t="inlineStr">
@@ -4766,7 +4770,7 @@
       </c>
       <c r="G81" s="17" t="inlineStr">
         <is>
-          <t>PlanGroupPanel</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="H81" s="17" t="inlineStr">
@@ -4783,12 +4787,12 @@
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCartStep</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCartStep.tsx</t>
+          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
         </is>
       </c>
       <c r="D82" s="20" t="inlineStr">
@@ -4807,7 +4811,7 @@
       <c r="G82" s="17" t="inlineStr"/>
       <c r="H82" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -4819,12 +4823,12 @@
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCheckoutStep</t>
+          <t>PostpaidPlanCard</t>
         </is>
       </c>
       <c r="C83" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
+          <t>components/patterns/PostpaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D83" s="20" t="inlineStr">
@@ -4840,7 +4844,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G83" s="17" t="inlineStr"/>
+      <c r="G83" s="17" t="inlineStr">
+        <is>
+          <t>PlanGroupPanel</t>
+        </is>
+      </c>
       <c r="H83" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4855,12 +4863,12 @@
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPackDetailsDrawer</t>
+          <t>PrepaidCartStep</t>
         </is>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
+          <t>components/patterns/PrepaidCartStep.tsx</t>
         </is>
       </c>
       <c r="D84" s="20" t="inlineStr">
@@ -4876,14 +4884,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G84" s="17" t="inlineStr">
-        <is>
-          <t>PrepaidPlanStep</t>
-        </is>
-      </c>
+      <c r="G84" s="17" t="inlineStr"/>
       <c r="H84" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4895,12 +4899,12 @@
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanCard</t>
+          <t>PrepaidCheckoutStep</t>
         </is>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanCard.tsx</t>
+          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
         </is>
       </c>
       <c r="D85" s="20" t="inlineStr">
@@ -4916,11 +4920,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G85" s="17" t="inlineStr">
-        <is>
-          <t>PrepaidPlanStep</t>
-        </is>
-      </c>
+      <c r="G85" s="17" t="inlineStr"/>
       <c r="H85" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4935,12 +4935,12 @@
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanStep</t>
+          <t>PrepaidPackDetailsDrawer</t>
         </is>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanStep.tsx</t>
+          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D86" s="20" t="inlineStr">
@@ -4956,7 +4956,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G86" s="17" t="inlineStr"/>
+      <c r="G86" s="17" t="inlineStr">
+        <is>
+          <t>PrepaidPlanStep</t>
+        </is>
+      </c>
       <c r="H86" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -4971,12 +4975,12 @@
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>SummaryTables</t>
+          <t>PrepaidPlanCard</t>
         </is>
       </c>
       <c r="C87" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryTables.tsx</t>
+          <t>components/patterns/PrepaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D87" s="20" t="inlineStr">
@@ -4994,12 +4998,12 @@
       </c>
       <c r="G87" s="17" t="inlineStr">
         <is>
-          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
+          <t>PrepaidPlanStep</t>
         </is>
       </c>
       <c r="H87" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5011,12 +5015,12 @@
       </c>
       <c r="B88" s="17" t="inlineStr">
         <is>
-          <t>WinCashPaymentStep</t>
+          <t>PrepaidPlanStep</t>
         </is>
       </c>
       <c r="C88" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/WinCashPaymentStep.tsx</t>
+          <t>components/patterns/PrepaidPlanStep.tsx</t>
         </is>
       </c>
       <c r="D88" s="20" t="inlineStr">
@@ -5035,7 +5039,7 @@
       <c r="G88" s="17" t="inlineStr"/>
       <c r="H88" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5047,12 +5051,12 @@
       </c>
       <c r="B89" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep</t>
+          <t>SummaryTables</t>
         </is>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingAccountStep.tsx</t>
+          <t>components/patterns/CheckoutSummaryTables.tsx</t>
         </is>
       </c>
       <c r="D89" s="20" t="inlineStr">
@@ -5061,17 +5065,21 @@
         </is>
       </c>
       <c r="E89" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F89" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G89" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G89" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
+        </is>
+      </c>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5083,12 +5091,12 @@
       </c>
       <c r="B90" s="17" t="inlineStr">
         <is>
-          <t>BillingProfileSetupDrawer</t>
+          <t>WinCashPaymentStep</t>
         </is>
       </c>
       <c r="C90" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingProfileSetupDrawer.tsx</t>
+          <t>components/patterns/WinCashPaymentStep.tsx</t>
         </is>
       </c>
       <c r="D90" s="20" t="inlineStr">
@@ -5097,18 +5105,14 @@
         </is>
       </c>
       <c r="E90" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F90" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G90" s="17" t="inlineStr">
-        <is>
-          <t>BillingAccountStep</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G90" s="17" t="inlineStr"/>
       <c r="H90" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5123,12 +5127,12 @@
       </c>
       <c r="B91" s="17" t="inlineStr">
         <is>
-          <t>ZsbAddressStep</t>
+          <t>BillingAccountStep</t>
         </is>
       </c>
       <c r="C91" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ZsbAddressStep.tsx</t>
+          <t>components/patterns/BillingAccountStep.tsx</t>
         </is>
       </c>
       <c r="D91" s="20" t="inlineStr">
@@ -5159,12 +5163,12 @@
       </c>
       <c r="B92" s="17" t="inlineStr">
         <is>
-          <t>AppointmentBookingStep</t>
+          <t>BillingProfileSetupDrawer</t>
         </is>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/AppointmentBookingStep.tsx</t>
+          <t>components/patterns/BillingProfileSetupDrawer.tsx</t>
         </is>
       </c>
       <c r="D92" s="20" t="inlineStr">
@@ -5173,17 +5177,21 @@
         </is>
       </c>
       <c r="E92" s="17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F92" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
-        </is>
-      </c>
-      <c r="G92" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G92" s="17" t="inlineStr">
+        <is>
+          <t>BillingAccountStep</t>
+        </is>
+      </c>
       <c r="H92" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5195,12 +5203,12 @@
       </c>
       <c r="B93" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel</t>
+          <t>ZsbAddressStep</t>
         </is>
       </c>
       <c r="C93" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DemoFaultPanel.tsx</t>
+          <t>components/patterns/ZsbAddressStep.tsx</t>
         </is>
       </c>
       <c r="D93" s="20" t="inlineStr">
@@ -5209,17 +5217,17 @@
         </is>
       </c>
       <c r="E93" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F93" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G93" s="17" t="inlineStr"/>
       <c r="H93" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5231,12 +5239,12 @@
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>DonorAttachmentStep</t>
+          <t>AppointmentBookingStep</t>
         </is>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorAttachmentStep.tsx</t>
+          <t>components/patterns/AppointmentBookingStep.tsx</t>
         </is>
       </c>
       <c r="D94" s="20" t="inlineStr">
@@ -5245,17 +5253,17 @@
         </is>
       </c>
       <c r="E94" s="17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F94" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
         </is>
       </c>
       <c r="G94" s="17" t="inlineStr"/>
       <c r="H94" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5267,12 +5275,12 @@
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>DonorDetailsStep</t>
+          <t>DemoFaultPanel</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorDetailsStep.tsx</t>
+          <t>components/patterns/DemoFaultPanel.tsx</t>
         </is>
       </c>
       <c r="D95" s="20" t="inlineStr">
@@ -5288,14 +5296,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
-      <c r="G95" s="17" t="inlineStr">
-        <is>
-          <t>DonorAttachmentStep</t>
-        </is>
-      </c>
+      <c r="G95" s="17" t="inlineStr"/>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5307,12 +5311,12 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>EntityMissing</t>
+          <t>DonorAttachmentStep</t>
         </is>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/EntityMissing.tsx</t>
+          <t>components/patterns/DonorAttachmentStep.tsx</t>
         </is>
       </c>
       <c r="D96" s="20" t="inlineStr">
@@ -5325,13 +5329,13 @@
       </c>
       <c r="F96" s="17" t="inlineStr">
         <is>
-          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G96" s="17" t="inlineStr"/>
       <c r="H96" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5343,12 +5347,12 @@
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>ActivityCommentsStep</t>
+          <t>DonorDetailsStep</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ActivityCommentsStep.tsx</t>
+          <t>components/patterns/DonorDetailsStep.tsx</t>
         </is>
       </c>
       <c r="D97" s="20" t="inlineStr">
@@ -5357,17 +5361,21 @@
         </is>
       </c>
       <c r="E97" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F97" s="17" t="inlineStr">
         <is>
-          <t>pre-to-post-migration, sim-number-management, administration</t>
-        </is>
-      </c>
-      <c r="G97" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+        </is>
+      </c>
+      <c r="G97" s="17" t="inlineStr">
+        <is>
+          <t>DonorAttachmentStep</t>
+        </is>
+      </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5379,12 +5387,12 @@
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>LineSelectionStep</t>
+          <t>EntityMissing</t>
         </is>
       </c>
       <c r="C98" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/LineSelectionStep.tsx</t>
+          <t>components/patterns/EntityMissing.tsx</t>
         </is>
       </c>
       <c r="D98" s="20" t="inlineStr">
@@ -5393,17 +5401,17 @@
         </is>
       </c>
       <c r="E98" s="17" t="n">
-        <v>3</v>
+        <v>6</v>
       </c>
       <c r="F98" s="17" t="inlineStr">
         <is>
-          <t>mobile-service-changes, pre-to-post-migration, administration</t>
+          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
         </is>
       </c>
       <c r="G98" s="17" t="inlineStr"/>
       <c r="H98" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5415,12 +5423,12 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>TicketCreationModal</t>
+          <t>ActivityCommentsStep</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/TicketCreationModal.tsx</t>
+          <t>components/patterns/ActivityCommentsStep.tsx</t>
         </is>
       </c>
       <c r="D99" s="20" t="inlineStr">
@@ -5433,13 +5441,13 @@
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, customer360, support</t>
+          <t>pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G99" s="17" t="inlineStr"/>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5451,31 +5459,31 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>BulkOperationPortal</t>
+          <t>LineSelectionStep</t>
         </is>
       </c>
       <c r="C100" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BulkOperationPortal.tsx</t>
-        </is>
-      </c>
-      <c r="D100" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/patterns/LineSelectionStep.tsx</t>
+        </is>
+      </c>
+      <c r="D100" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E100" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F100" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b</t>
+          <t>mobile-service-changes, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G100" s="17" t="inlineStr"/>
       <c r="H100" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5487,25 +5495,25 @@
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>DualPlaySerialCheckStep</t>
+          <t>TicketCreationModal</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
-        </is>
-      </c>
-      <c r="D101" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/patterns/TicketCreationModal.tsx</t>
+        </is>
+      </c>
+      <c r="D101" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E101" s="17" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="F101" s="17" t="inlineStr">
         <is>
-          <t>fwa-5g-home</t>
+          <t>trouble-ticketing-complaints, customer360, support</t>
         </is>
       </c>
       <c r="G101" s="17" t="inlineStr"/>
@@ -5523,12 +5531,12 @@
       </c>
       <c r="B102" s="17" t="inlineStr">
         <is>
-          <t>SimSwapFormStep</t>
+          <t>BulkOperationPortal</t>
         </is>
       </c>
       <c r="C102" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/SimSwapFormStep.tsx</t>
+          <t>components/patterns/BulkOperationPortal.tsx</t>
         </is>
       </c>
       <c r="D102" s="21" t="inlineStr">
@@ -5541,7 +5549,7 @@
       </c>
       <c r="F102" s="17" t="inlineStr">
         <is>
-          <t>sim-number-management</t>
+          <t>enterprise-iot-b2b</t>
         </is>
       </c>
       <c r="G102" s="17" t="inlineStr"/>
@@ -5559,12 +5567,12 @@
       </c>
       <c r="B103" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>DualPlaySerialCheckStep</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/VerificationGate.tsx</t>
+          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
         </is>
       </c>
       <c r="D103" s="21" t="inlineStr">
@@ -5577,7 +5585,7 @@
       </c>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fwa-5g-home</t>
         </is>
       </c>
       <c r="G103" s="17" t="inlineStr"/>
@@ -5590,30 +5598,30 @@
     <row r="104">
       <c r="A104" s="17" t="inlineStr">
         <is>
-          <t>Wizard</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="B104" s="17" t="inlineStr">
         <is>
-          <t>AbandonDialog</t>
+          <t>SimSwapFormStep</t>
         </is>
       </c>
       <c r="C104" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardDialogs.tsx</t>
-        </is>
-      </c>
-      <c r="D104" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/patterns/SimSwapFormStep.tsx</t>
+        </is>
+      </c>
+      <c r="D104" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E104" s="17" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F104" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>sim-number-management</t>
         </is>
       </c>
       <c r="G104" s="17" t="inlineStr"/>
@@ -5626,30 +5634,30 @@
     <row r="105">
       <c r="A105" s="17" t="inlineStr">
         <is>
-          <t>Wizard</t>
+          <t>Pattern</t>
         </is>
       </c>
       <c r="B105" s="17" t="inlineStr">
         <is>
-          <t>CustomerMirrorPanel</t>
+          <t>VerificationGate</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/CustomerMirrorPanel.tsx</t>
-        </is>
-      </c>
-      <c r="D105" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/patterns/VerificationGate.tsx</t>
+        </is>
+      </c>
+      <c r="D105" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E105" s="17" t="n">
-        <v>11</v>
+        <v>1</v>
       </c>
       <c r="F105" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G105" s="17" t="inlineStr"/>
@@ -5667,12 +5675,12 @@
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
-          <t>StepSummaryPanel</t>
+          <t>AbandonDialog</t>
         </is>
       </c>
       <c r="C106" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/StepSummaryPanel.tsx</t>
+          <t>components/patterns/wizard/WizardDialogs.tsx</t>
         </is>
       </c>
       <c r="D106" s="20" t="inlineStr">
@@ -5691,7 +5699,7 @@
       <c r="G106" s="17" t="inlineStr"/>
       <c r="H106" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5703,12 +5711,12 @@
       </c>
       <c r="B107" s="17" t="inlineStr">
         <is>
-          <t>StepSummarySection</t>
+          <t>CustomerMirrorPanel</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/StepSummarySection.tsx</t>
+          <t>components/patterns/wizard/CustomerMirrorPanel.tsx</t>
         </is>
       </c>
       <c r="D107" s="20" t="inlineStr">
@@ -5724,11 +5732,7 @@
           <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
-      <c r="G107" s="17" t="inlineStr">
-        <is>
-          <t>StepSummaryPanel</t>
-        </is>
-      </c>
+      <c r="G107" s="17" t="inlineStr"/>
       <c r="H107" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5743,12 +5747,12 @@
       </c>
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>SummaryFieldRow</t>
+          <t>CustomerViewButton</t>
         </is>
       </c>
       <c r="C108" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/SummaryFieldRow.tsx</t>
+          <t>components/patterns/wizard/CustomerViewButton.tsx</t>
         </is>
       </c>
       <c r="D108" s="20" t="inlineStr">
@@ -5766,12 +5770,12 @@
       </c>
       <c r="G108" s="17" t="inlineStr">
         <is>
-          <t>StepSummaryPanel</t>
+          <t>WizardStepHeader</t>
         </is>
       </c>
       <c r="H108" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -5783,12 +5787,12 @@
       </c>
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>WizardFooter</t>
+          <t>StepSummaryPanel</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardFooter.tsx</t>
+          <t>components/patterns/wizard/StepSummaryPanel.tsx</t>
         </is>
       </c>
       <c r="D109" s="20" t="inlineStr">
@@ -5807,7 +5811,7 @@
       <c r="G109" s="17" t="inlineStr"/>
       <c r="H109" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -5819,12 +5823,12 @@
       </c>
       <c r="B110" s="17" t="inlineStr">
         <is>
-          <t>WizardStepHeader</t>
+          <t>StepSummarySection</t>
         </is>
       </c>
       <c r="C110" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardStepHeader.tsx</t>
+          <t>components/patterns/wizard/StepSummarySection.tsx</t>
         </is>
       </c>
       <c r="D110" s="20" t="inlineStr">
@@ -5840,7 +5844,11 @@
           <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
-      <c r="G110" s="17" t="inlineStr"/>
+      <c r="G110" s="17" t="inlineStr">
+        <is>
+          <t>StepSummaryPanel</t>
+        </is>
+      </c>
       <c r="H110" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -5855,12 +5863,12 @@
       </c>
       <c r="B111" s="17" t="inlineStr">
         <is>
-          <t>WizardTitleBand</t>
+          <t>SummaryFieldRow</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/wizard/WizardTitleBand.tsx</t>
+          <t>components/patterns/wizard/SummaryFieldRow.tsx</t>
         </is>
       </c>
       <c r="D111" s="20" t="inlineStr">
@@ -5876,15 +5884,127 @@
           <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
-      <c r="G111" s="17" t="inlineStr"/>
+      <c r="G111" s="17" t="inlineStr">
+        <is>
+          <t>StepSummaryPanel</t>
+        </is>
+      </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
         </is>
       </c>
     </row>
+    <row r="112">
+      <c r="A112" s="17" t="inlineStr">
+        <is>
+          <t>Wizard</t>
+        </is>
+      </c>
+      <c r="B112" s="17" t="inlineStr">
+        <is>
+          <t>WizardFooter</t>
+        </is>
+      </c>
+      <c r="C112" s="17" t="inlineStr">
+        <is>
+          <t>components/patterns/wizard/WizardFooter.tsx</t>
+        </is>
+      </c>
+      <c r="D112" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E112" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F112" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G112" s="17" t="inlineStr"/>
+      <c r="H112" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="113">
+      <c r="A113" s="17" t="inlineStr">
+        <is>
+          <t>Wizard</t>
+        </is>
+      </c>
+      <c r="B113" s="17" t="inlineStr">
+        <is>
+          <t>WizardStepHeader</t>
+        </is>
+      </c>
+      <c r="C113" s="17" t="inlineStr">
+        <is>
+          <t>components/patterns/wizard/WizardStepHeader.tsx</t>
+        </is>
+      </c>
+      <c r="D113" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E113" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F113" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G113" s="17" t="inlineStr"/>
+      <c r="H113" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="114">
+      <c r="A114" s="17" t="inlineStr">
+        <is>
+          <t>Wizard</t>
+        </is>
+      </c>
+      <c r="B114" s="17" t="inlineStr">
+        <is>
+          <t>WizardTitleBand</t>
+        </is>
+      </c>
+      <c r="C114" s="17" t="inlineStr">
+        <is>
+          <t>components/patterns/wizard/WizardTitleBand.tsx</t>
+        </is>
+      </c>
+      <c r="D114" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E114" s="17" t="n">
+        <v>11</v>
+      </c>
+      <c r="F114" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G114" s="17" t="inlineStr"/>
+      <c r="H114" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-18</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
-  <autoFilter ref="A1:H111"/>
+  <autoFilter ref="A1:H114"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -5895,7 +6015,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H57"/>
+  <dimension ref="A1:H60"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.50" customWidth="1" min="1" max="1"/>
@@ -5981,7 +6101,7 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, VerificationGate, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, customer360Engine, fibreServiceability, serviceLocationLookup, useAreaOptions, configStore, entityStore</t>
+          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, VerificationGate, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, connectionEligibility, customer360Engine, fibreServiceability, serviceLocationLookup, useAreaOptions, configStore, entityStore</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
@@ -6026,7 +6146,7 @@
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6221,7 +6341,7 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>lineSelectionModel, customer360Demo, customer360Engine</t>
+          <t>lineSelectionModel, customer360Demo, connectionEligibility, customer360Engine</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
@@ -6306,7 +6426,7 @@
       </c>
       <c r="H10" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6434,12 +6554,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>eligibilityEngine</t>
+          <t>connectionEligibility</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityEngine.ts</t>
+          <t>engines/connectionEligibility.ts</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -6455,14 +6575,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G14" s="17" t="inlineStr">
-        <is>
-          <t>eligibilityRowsModel, eligibilityTypes</t>
-        </is>
-      </c>
+      <c r="G14" s="17" t="inlineStr"/>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>uncommitted</t>
         </is>
       </c>
     </row>
@@ -6474,12 +6590,12 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>fibreServiceability</t>
+          <t>eligibilityEngine</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>engines/fibreServiceability.ts</t>
+          <t>engines/eligibilityEngine.ts</t>
         </is>
       </c>
       <c r="D15" s="20" t="inlineStr">
@@ -6497,12 +6613,12 @@
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
+          <t>eligibilityRowsModel, eligibilityTypes</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6514,12 +6630,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>personaEngine</t>
+          <t>fibreServiceability</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>engines/personaEngine.ts</t>
+          <t>engines/fibreServiceability.ts</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -6532,17 +6648,17 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>approvalAuthority, navigationEngine</t>
+          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -6554,12 +6670,12 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>eligibilityGuard</t>
+          <t>personaEngine</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityGuard.ts</t>
+          <t>engines/personaEngine.ts</t>
         </is>
       </c>
       <c r="D17" s="20" t="inlineStr">
@@ -6568,17 +6684,21 @@
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr"/>
+          <t>dashboard, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>approvalAuthority, navigationEngine</t>
+        </is>
+      </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -6590,12 +6710,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>serviceLocationLookup</t>
+          <t>eligibilityGuard</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceLocationLookup.ts</t>
+          <t>engines/eligibilityGuard.ts</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -6608,14 +6728,10 @@
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>ZsbAddressStep</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
+        </is>
+      </c>
+      <c r="G18" s="17" t="inlineStr"/>
       <c r="H18" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -6630,12 +6746,12 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>agentPrivilegeEngine</t>
+          <t>serviceLocationLookup</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>engines/agentPrivilegeEngine.ts</t>
+          <t>engines/serviceLocationLookup.ts</t>
         </is>
       </c>
       <c r="D19" s="20" t="inlineStr">
@@ -6644,17 +6760,21 @@
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, navigation, administration, customer360, profile, tasks</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>ZsbAddressStep</t>
+        </is>
+      </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6666,12 +6786,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>agentTaskEngine</t>
+          <t>agentPrivilegeEngine</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>engines/agentTaskEngine.ts</t>
+          <t>engines/agentPrivilegeEngine.ts</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -6684,13 +6804,13 @@
       </c>
       <c r="F20" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, trouble-ticketing-complaints, orders, support, tasks</t>
+          <t>trouble-ticketing-complaints, navigation, administration, customer360, profile, tasks</t>
         </is>
       </c>
       <c r="G20" s="17" t="inlineStr"/>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6702,12 +6822,12 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>approvalAuthority</t>
+          <t>agentTaskEngine</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>engines/approvalAuthority.ts</t>
+          <t>engines/agentTaskEngine.ts</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -6720,13 +6840,13 @@
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, sim-number-management, navigation, customer360, orders</t>
+          <t>dashboard, order-management, trouble-ticketing-complaints, orders, support, tasks</t>
         </is>
       </c>
       <c r="G21" s="17" t="inlineStr"/>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -6738,12 +6858,12 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>portInEngine</t>
+          <t>approvalAuthority</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>engines/portInEngine.ts</t>
+          <t>engines/approvalAuthority.ts</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -6756,13 +6876,13 @@
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+          <t>dashboard, order-management, sim-number-management, navigation, customer360, orders</t>
         </is>
       </c>
       <c r="G22" s="17" t="inlineStr"/>
       <c r="H22" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6774,12 +6894,12 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>csvExport</t>
+          <t>portInEngine</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>engines/csvExport.ts</t>
+          <t>engines/portInEngine.ts</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
@@ -6788,17 +6908,17 @@
         </is>
       </c>
       <c r="E23" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, customer360, profile, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G23" s="17" t="inlineStr"/>
       <c r="H23" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6810,12 +6930,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>bellNotificationExpiry</t>
+          <t>csvExport</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>engines/bellNotificationExpiry.ts</t>
+          <t>engines/csvExport.ts</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -6824,11 +6944,11 @@
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>administration, customer360</t>
+          <t>trouble-ticketing-complaints, customer360, profile, support</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr"/>
@@ -6846,12 +6966,12 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>businessAccountEngine</t>
+          <t>bellNotificationExpiry</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>engines/businessAccountEngine.ts</t>
+          <t>engines/bellNotificationExpiry.ts</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
@@ -6864,13 +6984,13 @@
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>customer-search, customer360</t>
+          <t>administration, customer360</t>
         </is>
       </c>
       <c r="G25" s="17" t="inlineStr"/>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -6882,12 +7002,12 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>navigationEngine</t>
+          <t>businessAccountEngine</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>engines/navigationEngine.ts</t>
+          <t>engines/businessAccountEngine.ts</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -6900,13 +7020,13 @@
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>navigation, customer360</t>
+          <t>customer-search, customer360</t>
         </is>
       </c>
       <c r="G26" s="17" t="inlineStr"/>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -6918,12 +7038,12 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>qnomyQueueEngine</t>
+          <t>navigationEngine</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>engines/qnomyQueueEngine.ts</t>
+          <t>engines/navigationEngine.ts</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
@@ -6936,13 +7056,13 @@
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>navigation, tickets</t>
+          <t>navigation, customer360</t>
         </is>
       </c>
       <c r="G27" s="17" t="inlineStr"/>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6954,31 +7074,31 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>agentProfileEngine</t>
+          <t>qnomyQueueEngine</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>engines/agentProfileEngine.ts</t>
-        </is>
-      </c>
-      <c r="D28" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>engines/qnomyQueueEngine.ts</t>
+        </is>
+      </c>
+      <c r="D28" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E28" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>navigation, tickets</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr"/>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -6990,12 +7110,12 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>customer360VisibilityEngine</t>
+          <t>agentProfileEngine</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>engines/customer360VisibilityEngine.ts</t>
+          <t>engines/agentProfileEngine.ts</t>
         </is>
       </c>
       <c r="D29" s="21" t="inlineStr">
@@ -7008,13 +7128,13 @@
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>navigation</t>
         </is>
       </c>
       <c r="G29" s="17" t="inlineStr"/>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7026,12 +7146,12 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>profileChangeTicket</t>
+          <t>customer360VisibilityEngine</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>engines/profileChangeTicket.ts</t>
+          <t>engines/customer360VisibilityEngine.ts</t>
         </is>
       </c>
       <c r="D30" s="21" t="inlineStr">
@@ -7062,12 +7182,12 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>searchScopeEngine</t>
+          <t>profileChangeTicket</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>engines/searchScopeEngine.ts</t>
+          <t>engines/profileChangeTicket.ts</t>
         </is>
       </c>
       <c r="D31" s="21" t="inlineStr">
@@ -7080,13 +7200,13 @@
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G31" s="17" t="inlineStr"/>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7098,27 +7218,31 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>moduleDescriptions</t>
+          <t>searchScopeEngine</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>engines/moduleDescriptions.ts</t>
-        </is>
-      </c>
-      <c r="D32" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>engines/searchScopeEngine.ts</t>
+        </is>
+      </c>
+      <c r="D32" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E32" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F32" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F32" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G32" s="17" t="inlineStr"/>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7130,12 +7254,12 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>screenGrouping</t>
+          <t>moduleDescriptions</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>engines/screenGrouping.ts</t>
+          <t>engines/moduleDescriptions.ts</t>
         </is>
       </c>
       <c r="D33" s="23" t="inlineStr">
@@ -7157,40 +7281,32 @@
     <row r="34">
       <c r="A34" s="17" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>entityStore</t>
+          <t>screenGrouping</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>stores/entityStore.ts</t>
-        </is>
-      </c>
-      <c r="D34" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>engines/screenGrouping.ts</t>
+        </is>
+      </c>
+      <c r="D34" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="F34" s="17" t="inlineStr">
-        <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G34" s="17" t="inlineStr">
-        <is>
-          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F34" s="17" t="inlineStr"/>
+      <c r="G34" s="17" t="inlineStr"/>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7202,12 +7318,12 @@
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>customerContextStore</t>
+          <t>entityStore</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>stores/customerContextStore.ts</t>
+          <t>stores/entityStore.ts</t>
         </is>
       </c>
       <c r="D35" s="20" t="inlineStr">
@@ -7216,21 +7332,21 @@
         </is>
       </c>
       <c r="E35" s="17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G35" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, useWizardDraftActions, authStore</t>
+          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
         </is>
       </c>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7242,12 +7358,12 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>authStore</t>
+          <t>customerContextStore</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>stores/authStore.ts</t>
+          <t>stores/customerContextStore.ts</t>
         </is>
       </c>
       <c r="D36" s="20" t="inlineStr">
@@ -7256,16 +7372,16 @@
         </is>
       </c>
       <c r="E36" s="17" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F36" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, support, tasks, tickets</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G36" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore</t>
+          <t>ActivationCompleteScreen, useActedForCustomer, useWizardDraftActions, authStore</t>
         </is>
       </c>
       <c r="H36" s="17" t="inlineStr">
@@ -7282,12 +7398,12 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>notificationStore</t>
+          <t>authStore</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>stores/notificationStore.ts</t>
+          <t>stores/authStore.ts</t>
         </is>
       </c>
       <c r="D37" s="20" t="inlineStr">
@@ -7296,21 +7412,21 @@
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G37" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, useSubmit</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore</t>
         </is>
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7322,12 +7438,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>personaStore</t>
+          <t>notificationStore</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>stores/personaStore.ts</t>
+          <t>stores/notificationStore.ts</t>
         </is>
       </c>
       <c r="D38" s="20" t="inlineStr">
@@ -7336,21 +7452,21 @@
         </is>
       </c>
       <c r="E38" s="17" t="n">
-        <v>19</v>
+        <v>20</v>
       </c>
       <c r="F38" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, tasks</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
         </is>
       </c>
       <c r="G38" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, AppointmentBookingStep, configStore</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, useSubmit</t>
         </is>
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7362,12 +7478,12 @@
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>workflowStore</t>
+          <t>personaStore</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>stores/workflowStore.ts</t>
+          <t>stores/personaStore.ts</t>
         </is>
       </c>
       <c r="D39" s="20" t="inlineStr">
@@ -7376,16 +7492,16 @@
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>12</v>
+        <v>19</v>
       </c>
       <c r="F39" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, tasks</t>
         </is>
       </c>
       <c r="G39" s="17" t="inlineStr">
         <is>
-          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, AppointmentBookingStep, configStore</t>
         </is>
       </c>
       <c r="H39" s="17" t="inlineStr">
@@ -7402,35 +7518,35 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>customerVerificationStore</t>
+          <t>workflowStore</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>stores/customerVerificationStore.ts</t>
-        </is>
-      </c>
-      <c r="D40" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>stores/workflowStore.ts</t>
+        </is>
+      </c>
+      <c r="D40" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
         </is>
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7442,12 +7558,12 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>qnomyQueueStore</t>
+          <t>customerVerificationStore</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>stores/qnomyQueueStore.ts</t>
+          <t>stores/customerVerificationStore.ts</t>
         </is>
       </c>
       <c r="D41" s="21" t="inlineStr">
@@ -7460,13 +7576,17 @@
       </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G41" s="17" t="inlineStr"/>
+          <t>customer360</t>
+        </is>
+      </c>
+      <c r="G41" s="17" t="inlineStr">
+        <is>
+          <t>VerificationGate</t>
+        </is>
+      </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7478,12 +7598,12 @@
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>regionStore</t>
+          <t>qnomyQueueStore</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>stores/regionStore.ts</t>
+          <t>stores/qnomyQueueStore.ts</t>
         </is>
       </c>
       <c r="D42" s="21" t="inlineStr">
@@ -7502,7 +7622,7 @@
       <c r="G42" s="17" t="inlineStr"/>
       <c r="H42" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7514,12 +7634,12 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>sidebarStore</t>
+          <t>regionStore</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>stores/sidebarStore.ts</t>
+          <t>stores/regionStore.ts</t>
         </is>
       </c>
       <c r="D43" s="21" t="inlineStr">
@@ -7538,7 +7658,7 @@
       <c r="G43" s="17" t="inlineStr"/>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7550,12 +7670,12 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>themeStore</t>
+          <t>sidebarStore</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>stores/themeStore.ts</t>
+          <t>stores/sidebarStore.ts</t>
         </is>
       </c>
       <c r="D44" s="21" t="inlineStr">
@@ -7574,7 +7694,7 @@
       <c r="G44" s="17" t="inlineStr"/>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7586,67 +7706,63 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>configStore</t>
+          <t>themeStore</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>stores/configStore.ts</t>
-        </is>
-      </c>
-      <c r="D45" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>stores/themeStore.ts</t>
+        </is>
+      </c>
+      <c r="D45" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F45" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F45" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G45" s="17" t="inlineStr"/>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="17" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>useEnterToSubmit</t>
+          <t>configStore</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>hooks/useEnterToSubmit.ts</t>
-        </is>
-      </c>
-      <c r="D46" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>stores/configStore.ts</t>
+        </is>
+      </c>
+      <c r="D46" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E46" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="F46" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G46" s="17" t="inlineStr">
-        <is>
-          <t>VerificationGate, useIdLookup</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F46" s="17" t="inlineStr"/>
+      <c r="G46" s="17" t="inlineStr"/>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7658,12 +7774,12 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>useSearchListNav</t>
+          <t>useEnterToSubmit</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSearchListNav.ts</t>
+          <t>hooks/useEnterToSubmit.ts</t>
         </is>
       </c>
       <c r="D47" s="20" t="inlineStr">
@@ -7672,21 +7788,21 @@
         </is>
       </c>
       <c r="E47" s="17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
+          <t>VerificationGate, useIdLookup</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7698,12 +7814,12 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>useAreaOptions</t>
+          <t>useSearchListNav</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>hooks/useAreaOptions.ts</t>
+          <t>hooks/useSearchListNav.ts</t>
         </is>
       </c>
       <c r="D48" s="20" t="inlineStr">
@@ -7712,21 +7828,21 @@
         </is>
       </c>
       <c r="E48" s="17" t="n">
-        <v>8</v>
+        <v>11</v>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G48" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep, ZsbAddressStep</t>
+          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
         </is>
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7738,12 +7854,12 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>useSubmit</t>
+          <t>useAreaOptions</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSubmit.ts</t>
+          <t>hooks/useAreaOptions.ts</t>
         </is>
       </c>
       <c r="D49" s="20" t="inlineStr">
@@ -7752,17 +7868,21 @@
         </is>
       </c>
       <c r="E49" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
-        </is>
-      </c>
-      <c r="G49" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>BillingAccountStep, ZsbAddressStep</t>
+        </is>
+      </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7774,68 +7894,64 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>useMinWidth</t>
+          <t>useSubmit</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>hooks/useMinWidth.ts</t>
-        </is>
-      </c>
-      <c r="D50" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>hooks/useSubmit.ts</t>
+        </is>
+      </c>
+      <c r="D50" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E50" s="17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F50" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
         </is>
       </c>
       <c r="G50" s="17" t="inlineStr"/>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
         <is>
-          <t>Helper</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>statusTone</t>
+          <t>useMinWidth</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>lib/statusTone.ts</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>hooks/useMinWidth.ts</t>
+        </is>
+      </c>
+      <c r="D51" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E51" s="17" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="F51" s="17" t="inlineStr">
         <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G51" s="17" t="inlineStr">
-        <is>
-          <t>ruleEngine</t>
-        </is>
-      </c>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G51" s="17" t="inlineStr"/>
       <c r="H51" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -7850,12 +7966,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>format</t>
+          <t>statusTone</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>lib/format.ts</t>
+          <t>lib/statusTone.ts</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
@@ -7864,21 +7980,21 @@
         </is>
       </c>
       <c r="E52" s="17" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, support, tasks</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G52" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, SupportingDocumentUpload, GuidedContactStep, IdLookupStep, postpaidPlanModel, StepSummaryPanel, stepSummary, postpaidPricing</t>
+          <t>ruleEngine</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7890,12 +8006,12 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>deviceType</t>
+          <t>format</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>lib/deviceType.ts</t>
+          <t>lib/format.ts</t>
         </is>
       </c>
       <c r="D53" s="20" t="inlineStr">
@@ -7904,16 +8020,16 @@
         </is>
       </c>
       <c r="E53" s="17" t="n">
-        <v>11</v>
+        <v>19</v>
       </c>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, support, tasks</t>
         </is>
       </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
-          <t>SimSerialScanner, SimTypeStep, cafTypes</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, SupportingDocumentUpload, GuidedContactStep, IdLookupStep, postpaidPlanModel, StepSummaryPanel, stepSummary, postpaidPricing</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
@@ -7930,12 +8046,12 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>taskId</t>
+          <t>buildEnv</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>lib/taskId.ts</t>
+          <t>lib/buildEnv.ts</t>
         </is>
       </c>
       <c r="D54" s="20" t="inlineStr">
@@ -7944,21 +8060,21 @@
         </is>
       </c>
       <c r="E54" s="17" t="n">
-        <v>11</v>
+        <v>16</v>
       </c>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G54" s="17" t="inlineStr">
         <is>
-          <t>useWizardDraftActions</t>
+          <t>syntheticMarker, navigationEngine</t>
         </is>
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7970,12 +8086,12 @@
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>connectionType</t>
+          <t>deviceType</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>lib/connectionType.ts</t>
+          <t>lib/deviceType.ts</t>
         </is>
       </c>
       <c r="D55" s="20" t="inlineStr">
@@ -7984,21 +8100,21 @@
         </is>
       </c>
       <c r="E55" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
         </is>
       </c>
       <c r="G55" s="17" t="inlineStr">
         <is>
-          <t>ConnectionTypeTag</t>
+          <t>SimSerialScanner, SimTypeStep, cafTypes</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8010,28 +8126,32 @@
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>screenName</t>
+          <t>taskId</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>lib/screenName.ts</t>
-        </is>
-      </c>
-      <c r="D56" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>lib/taskId.ts</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
-        <v>1</v>
+        <v>11</v>
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G56" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G56" s="17" t="inlineStr">
+        <is>
+          <t>useWizardDraftActions</t>
+        </is>
+      </c>
       <c r="H56" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -8046,40 +8166,156 @@
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
+          <t>connectionType</t>
+        </is>
+      </c>
+      <c r="C57" s="17" t="inlineStr">
+        <is>
+          <t>lib/connectionType.ts</t>
+        </is>
+      </c>
+      <c r="D57" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E57" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F57" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr">
+        <is>
+          <t>ConnectionTypeTag</t>
+        </is>
+      </c>
+      <c r="H57" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="17" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="B58" s="17" t="inlineStr">
+        <is>
+          <t>serviceTypeTag</t>
+        </is>
+      </c>
+      <c r="C58" s="17" t="inlineStr">
+        <is>
+          <t>lib/serviceTypeTag.ts</t>
+        </is>
+      </c>
+      <c r="D58" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
+        </is>
+      </c>
+      <c r="E58" s="17" t="n">
+        <v>10</v>
+      </c>
+      <c r="F58" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>ServiceTypeTag</t>
+        </is>
+      </c>
+      <c r="H58" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-19</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="17" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="B59" s="17" t="inlineStr">
+        <is>
+          <t>screenName</t>
+        </is>
+      </c>
+      <c r="C59" s="17" t="inlineStr">
+        <is>
+          <t>lib/screenName.ts</t>
+        </is>
+      </c>
+      <c r="D59" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
+        </is>
+      </c>
+      <c r="E59" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F59" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G59" s="17" t="inlineStr"/>
+      <c r="H59" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="17" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="B60" s="17" t="inlineStr">
+        <is>
           <t>values</t>
         </is>
       </c>
-      <c r="C57" s="17" t="inlineStr">
+      <c r="C60" s="17" t="inlineStr">
         <is>
           <t>lib/values.ts</t>
         </is>
       </c>
-      <c r="D57" s="21" t="inlineStr">
+      <c r="D60" s="21" t="inlineStr">
         <is>
           <t>Single area</t>
         </is>
       </c>
-      <c r="E57" s="17" t="n">
+      <c r="E60" s="17" t="n">
         <v>1</v>
       </c>
-      <c r="F57" s="17" t="inlineStr">
+      <c r="F60" s="17" t="inlineStr">
         <is>
           <t>customer360</t>
         </is>
       </c>
-      <c r="G57" s="17" t="inlineStr">
+      <c r="G60" s="17" t="inlineStr">
         <is>
           <t>customer360Demo</t>
         </is>
       </c>
-      <c r="H57" s="17" t="inlineStr">
+      <c r="H60" s="17" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H57"/>
+  <autoFilter ref="A1:H60"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
MNP plan-type eligibility, shared SIM serial read-back, additional documents, docked web nav, cross-sell sections
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -6578,7 +6578,7 @@
       <c r="G14" s="17" t="inlineStr"/>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -6618,7 +6618,7 @@
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Actual User capability for New Postpaid (under-18 secondary contact, no eligibility checks), Supplementary Form signing for primary and secondary contact, distinct demo reader identity, CUST-3090 test customer, offer category order
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -887,11 +887,11 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>23 named - see the Capabilities sheet</t>
+          <t>24 named - see the Capabilities sheet</t>
         </is>
       </c>
       <c r="C15" s="17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="D15" s="17" t="inlineStr"/>
       <c r="E15" s="17" t="inlineStr"/>
@@ -908,7 +908,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E24"/>
+  <dimension ref="A1:E25"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="37.80" customWidth="1" min="1" max="1"/>
@@ -1491,15 +1491,45 @@
     <row r="19">
       <c r="A19" s="17" t="inlineStr">
         <is>
+          <t>Actual User</t>
+        </is>
+      </c>
+      <c r="B19" s="17" t="inlineStr">
+        <is>
+          <t>Who will use the line when it is not the customer who owns it: the agent adds an actual user, who is identified like the primary customer (ID type, scan or upload, MOI, email, phone). The actual user is named on the Supplementary Form, which the one CAF signature also signs; an existing customer's changed email is written back to their record.</t>
+        </is>
+      </c>
+      <c r="C19" s="17" t="inlineStr">
+        <is>
+          <t>capabilities/ActualUser/ActualUser.tsx
+capabilities/ActualUser/actualUserModel.ts
+capabilities/ActualUser/index.ts
+capabilities/ActualUser/step.tsx
+capabilities/ActualUser/submit.ts
+capabilities/ActualUser/summary.ts</t>
+        </is>
+      </c>
+      <c r="D19" s="17" t="n">
+        <v>9</v>
+      </c>
+      <c r="E19" s="17" t="inlineStr">
+        <is>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="17" t="inlineStr">
+        <is>
           <t>Service Address</t>
         </is>
       </c>
-      <c r="B19" s="17" t="inlineStr">
+      <c r="B20" s="17" t="inlineStr">
         <is>
           <t>The address a service is activated at: one layout everywhere: Service Information (Kahramaa Meter ID / Vodafone Premise ID with Search), then Zone / Street / Building, then Additional Details, with Qatari-ID prefill.</t>
         </is>
       </c>
-      <c r="C19" s="17" t="inlineStr">
+      <c r="C20" s="17" t="inlineStr">
         <is>
           <t>capabilities/ServiceAddress/ServiceAddress.tsx
 capabilities/ServiceAddress/index.ts
@@ -1508,27 +1538,27 @@
 components/patterns/ZsbAddressStep.tsx</t>
         </is>
       </c>
-      <c r="D19" s="17" t="n">
+      <c r="D20" s="17" t="n">
         <v>8</v>
       </c>
-      <c r="E19" s="17" t="inlineStr">
+      <c r="E20" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
     </row>
-    <row r="20">
-      <c r="A20" s="17" t="inlineStr">
+    <row r="21">
+      <c r="A21" s="17" t="inlineStr">
         <is>
           <t>Appointment Booking</t>
         </is>
       </c>
-      <c r="B20" s="17" t="inlineStr">
+      <c r="B21" s="17" t="inlineStr">
         <is>
           <t>Book the installation visit: SLA cluster, the date strip (next working days from the earliest, with each day's open slots), the day's time slots and technicians free, the customer's request for a specific date and time (a later date makes the order future-dated), appointment notes and the documents the technician collects (defaulted from the persona).</t>
         </is>
       </c>
-      <c r="C20" s="17" t="inlineStr">
+      <c r="C21" s="17" t="inlineStr">
         <is>
           <t>capabilities/AppointmentBooking/AppointmentBooking.tsx
 capabilities/AppointmentBooking/index.ts
@@ -1537,27 +1567,27 @@
 components/patterns/appointmentModel.ts</t>
         </is>
       </c>
-      <c r="D20" s="17" t="n">
+      <c r="D21" s="17" t="n">
         <v>7</v>
       </c>
-      <c r="E20" s="17" t="inlineStr">
+      <c r="E21" s="17" t="inlineStr">
         <is>
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
         </is>
       </c>
     </row>
-    <row r="21">
-      <c r="A21" s="17" t="inlineStr">
+    <row r="22">
+      <c r="A22" s="17" t="inlineStr">
         <is>
           <t>Activity Comments</t>
         </is>
       </c>
-      <c r="B21" s="17" t="inlineStr">
+      <c r="B22" s="17" t="inlineStr">
         <is>
           <t>The closing note on the actions performed, with an optional channel.</t>
         </is>
       </c>
-      <c r="C21" s="17" t="inlineStr">
+      <c r="C22" s="17" t="inlineStr">
         <is>
           <t>capabilities/ActivityComments/ActivityComments.tsx
 capabilities/ActivityComments/index.ts
@@ -1565,27 +1595,27 @@
 components/patterns/ActivityCommentsStep.tsx</t>
         </is>
       </c>
-      <c r="D21" s="17" t="n">
+      <c r="D22" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="E21" s="17" t="inlineStr">
+      <c r="E22" s="17" t="inlineStr">
         <is>
           <t>pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
     </row>
-    <row r="22">
-      <c r="A22" s="17" t="inlineStr">
+    <row r="23">
+      <c r="A23" s="17" t="inlineStr">
         <is>
           <t>Line Selection</t>
         </is>
       </c>
-      <c r="B22" s="17" t="inlineStr">
+      <c r="B23" s="17" t="inlineStr">
         <is>
           <t>Choose which of the identified customer's existing mobile lines an order changes (Change Postpaid Plan, Change Prepaid Pack, Add Add-On): postpaid and / or prepaid lines with their current plan and price; a line that is not active, is barred or whose billing profile is in collections is shown with its reason and cannot be chosen.</t>
         </is>
       </c>
-      <c r="C22" s="17" t="inlineStr">
+      <c r="C23" s="17" t="inlineStr">
         <is>
           <t>capabilities/LineSelection/LineSelection.tsx
 capabilities/LineSelection/index.ts
@@ -1594,60 +1624,60 @@
 components/patterns/lineSelectionModel.ts</t>
         </is>
       </c>
-      <c r="D22" s="17" t="n">
+      <c r="D23" s="17" t="n">
         <v>3</v>
       </c>
-      <c r="E22" s="17" t="inlineStr">
+      <c r="E23" s="17" t="inlineStr">
         <is>
           <t>mobile-service-changes, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-    </row>
-    <row r="23">
-      <c r="A23" s="17" t="inlineStr">
-        <is>
-          <t>Selectable card styling</t>
-        </is>
-      </c>
-      <c r="B23" s="17" t="inlineStr">
-        <is>
-          <t>One selected / idle / highlighted surface for plans, offers, numbers, add-ons, discounts and ID/customer type.</t>
-        </is>
-      </c>
-      <c r="C23" s="17" t="inlineStr">
-        <is>
-          <t>capabilities/SelectableCard/index.ts</t>
-        </is>
-      </c>
-      <c r="D23" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="E23" s="17" t="inlineStr">
-        <is>
-          <t>administration</t>
         </is>
       </c>
     </row>
     <row r="24">
       <c r="A24" s="17" t="inlineStr">
         <is>
-          <t>Side drawer</t>
+          <t>Selectable card styling</t>
         </is>
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>Fixed 50%-width drawer for forms, details and multi-step flows: the title as a small uppercase label beside the close control, the body on the page tint, and a footer whose buttons share its width equally.</t>
+          <t>One selected / idle / highlighted surface for plans, offers, numbers, add-ons, discounts and ID/customer type.</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>capabilities/SideDrawer/index.ts</t>
+          <t>capabilities/SelectableCard/index.ts</t>
         </is>
       </c>
       <c r="D24" s="17" t="n">
         <v>1</v>
       </c>
       <c r="E24" s="17" t="inlineStr">
+        <is>
+          <t>administration</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="17" t="inlineStr">
+        <is>
+          <t>Side drawer</t>
+        </is>
+      </c>
+      <c r="B25" s="17" t="inlineStr">
+        <is>
+          <t>Fixed 50%-width drawer for forms, details and multi-step flows: the title as a small uppercase label beside the close control, the body on the page tint, and a footer whose buttons share its width equally.</t>
+        </is>
+      </c>
+      <c r="C25" s="17" t="inlineStr">
+        <is>
+          <t>capabilities/SideDrawer/index.ts</t>
+        </is>
+      </c>
+      <c r="D25" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="E25" s="17" t="inlineStr">
         <is>
           <t>administration</t>
         </is>
@@ -3115,7 +3145,7 @@
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3155,7 +3185,7 @@
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3195,7 +3225,7 @@
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3623,7 +3653,7 @@
       <c r="G50" s="17" t="inlineStr"/>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -3927,7 +3957,7 @@
       <c r="G58" s="17" t="inlineStr"/>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -4315,7 +4345,7 @@
       <c r="G68" s="17" t="inlineStr"/>
       <c r="H68" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -6394,7 +6424,7 @@
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8202,7 +8232,7 @@
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Secondary Contact must be 18+, pre-fill phone and write changes to contact record, line-count test; distinct solid Primary tag in services, contacts and profile header
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -1506,7 +1506,8 @@
 capabilities/ActualUser/index.ts
 capabilities/ActualUser/step.tsx
 capabilities/ActualUser/submit.ts
-capabilities/ActualUser/summary.ts</t>
+capabilities/ActualUser/summary.ts
+capabilities/ActualUser/useDemoReaderCustomer.ts</t>
         </is>
       </c>
       <c r="D19" s="17" t="n">
@@ -4037,7 +4038,7 @@
       </c>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -5929,7 +5930,7 @@
       <c r="G110" s="17" t="inlineStr"/>
       <c r="H110" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5969,7 +5970,7 @@
       </c>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6780,7 +6781,7 @@
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Protected-segment follow-ups: filter CSV export, task detail, bell inbox; block route-bound journeys; purge protected data on role switch
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$65</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$66</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -763,13 +763,13 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="D9" s="17" t="n">
         <v>31</v>
       </c>
       <c r="E9" s="17" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="F9" s="17" t="n">
         <v>2</v>
@@ -855,17 +855,17 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>118 UI components + 64 non-UI files</t>
+          <t>118 UI components + 65 non-UI files</t>
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>182</v>
+        <v>183</v>
       </c>
       <c r="D13" s="18" t="n">
         <v>156</v>
       </c>
       <c r="E13" s="18" t="n">
-        <v>21</v>
+        <v>22</v>
       </c>
       <c r="F13" s="18" t="n">
         <v>5</v>
@@ -3106,7 +3106,7 @@
       </c>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3226,7 +3226,7 @@
       </c>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3948,11 +3948,11 @@
         </is>
       </c>
       <c r="E58" s="17" t="n">
-        <v>16</v>
+        <v>17</v>
       </c>
       <c r="F58" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer-search, customer360, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer-search, customer360, support, tasks</t>
         </is>
       </c>
       <c r="G58" s="17" t="inlineStr">
@@ -3962,7 +3962,7 @@
       </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -3998,7 +3998,7 @@
       <c r="G59" s="17" t="inlineStr"/>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4078,7 +4078,7 @@
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4118,7 +4118,7 @@
       </c>
       <c r="H62" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4158,7 +4158,7 @@
       </c>
       <c r="H63" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -4502,7 +4502,7 @@
       <c r="G72" s="17" t="inlineStr"/>
       <c r="H72" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5426,7 +5426,7 @@
       <c r="G96" s="17" t="inlineStr"/>
       <c r="H96" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5682,7 +5682,7 @@
       <c r="G103" s="17" t="inlineStr"/>
       <c r="H103" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5790,7 +5790,7 @@
       <c r="G106" s="17" t="inlineStr"/>
       <c r="H106" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6286,7 +6286,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H65"/>
+  <dimension ref="A1:H66"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.50" customWidth="1" min="1" max="1"/>
@@ -6372,12 +6372,12 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, connectionEligibility, customer360Engine, fibreServiceability, serviceLocationLookup, useAreaOptions, useRestrictedCustomers, configStore, entityStore</t>
+          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, connectionEligibility, customer360Engine, fibreServiceability, roleSwitchPurge, serviceLocationLookup, useAreaOptions, useRestrictedCustomers, configStore, entityStore</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6452,12 +6452,12 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>TicketCreationModal, useIdLookup, useRestrictedCustomers</t>
+          <t>TicketCreationModal, useIdLookup, roleSwitchPurge, useRestrictedCustomers</t>
         </is>
       </c>
       <c r="H4" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6497,7 +6497,7 @@
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6509,12 +6509,12 @@
       </c>
       <c r="B6" s="17" t="inlineStr">
         <is>
-          <t>ruleEngine</t>
+          <t>restrictedCustomers</t>
         </is>
       </c>
       <c r="C6" s="17" t="inlineStr">
         <is>
-          <t>engines/ruleEngine.ts</t>
+          <t>engines/restrictedCustomers.ts</t>
         </is>
       </c>
       <c r="D6" s="20" t="inlineStr">
@@ -6527,17 +6527,17 @@
       </c>
       <c r="F6" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>BillLimitEditor, CreditCheckPanel, eligibilityRowsModel, FixedPlanStep, TicketCreationModal</t>
+          <t>useRestrictedCustomers</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6549,12 +6549,12 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>billingBalance</t>
+          <t>ruleEngine</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>engines/billingBalance.ts</t>
+          <t>engines/ruleEngine.ts</t>
         </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
@@ -6563,21 +6563,21 @@
         </is>
       </c>
       <c r="E7" s="17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, product-lines, navigation, administration, customer-search, customer360, orders</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, support</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>customer360Demo, customer360Engine</t>
+          <t>BillLimitEditor, CreditCheckPanel, eligibilityRowsModel, FixedPlanStep, TicketCreationModal</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6589,12 +6589,12 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>customer360Engine</t>
+          <t>billingBalance</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>engines/customer360Engine.ts</t>
+          <t>engines/billingBalance.ts</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -6612,12 +6612,12 @@
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>customer360Demo, customerServicesEngine</t>
+          <t>customer360Demo, customer360Engine</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6629,12 +6629,12 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>customerServicesEngine</t>
+          <t>customer360Engine</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>engines/customerServicesEngine.ts</t>
+          <t>engines/customer360Engine.ts</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -6652,12 +6652,12 @@
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>lineSelectionModel, customer360Demo, connectionEligibility, customer360Engine</t>
+          <t>customer360Demo, customerServicesEngine</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6669,12 +6669,12 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>serviceCall</t>
+          <t>customerServicesEngine</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceCall.ts</t>
+          <t>engines/customerServicesEngine.ts</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -6683,21 +6683,21 @@
         </is>
       </c>
       <c r="E10" s="17" t="n">
-        <v>13</v>
+        <v>14</v>
       </c>
       <c r="F10" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, product-lines, navigation, administration, customer-search, customer360, orders</t>
         </is>
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
+          <t>lineSelectionModel, customer360Demo, connectionEligibility, customer360Engine</t>
         </is>
       </c>
       <c r="H10" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6709,12 +6709,12 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>eligibilityEngine</t>
+          <t>serviceCall</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityEngine.ts</t>
+          <t>engines/serviceCall.ts</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -6723,21 +6723,21 @@
         </is>
       </c>
       <c r="E11" s="17" t="n">
-        <v>12</v>
+        <v>13</v>
       </c>
       <c r="F11" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>eligibilityRowsModel, eligibilityTypes, useIdLookup</t>
+          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -6749,12 +6749,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>milestoneEngine</t>
+          <t>eligibilityEngine</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>engines/milestoneEngine.ts</t>
+          <t>engines/eligibilityEngine.ts</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -6772,12 +6772,12 @@
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>guidedWizardTypes, useJourneyMilestones</t>
+          <t>eligibilityRowsModel, eligibilityTypes, useIdLookup</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6789,12 +6789,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>activityEngine</t>
+          <t>milestoneEngine</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>engines/activityEngine.ts</t>
+          <t>engines/milestoneEngine.ts</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
@@ -6803,16 +6803,16 @@
         </is>
       </c>
       <c r="E13" s="17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F13" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, useWizardDraftActions</t>
+          <t>guidedWizardTypes, useJourneyMilestones</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
@@ -6829,12 +6829,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>businessSegment</t>
+          <t>activityEngine</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>engines/businessSegment.ts</t>
+          <t>engines/activityEngine.ts</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -6847,12 +6847,12 @@
       </c>
       <c r="F14" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, navigation, administration, customer-search, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep, customer360Demo, businessAccountEngine</t>
+          <t>ActivationCompleteScreen, useWizardDraftActions</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
@@ -6869,12 +6869,12 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>creditLimit</t>
+          <t>businessSegment</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>engines/creditLimit.ts</t>
+          <t>engines/businessSegment.ts</t>
         </is>
       </c>
       <c r="D15" s="20" t="inlineStr">
@@ -6887,17 +6887,17 @@
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, navigation, administration, customer-search, customer360</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>CreditLimitCard, billingAccountModel</t>
+          <t>BillingAccountStep, customer360Demo, businessAccountEngine</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6909,12 +6909,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>postpaidPricing</t>
+          <t>creditLimit</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>engines/postpaidPricing.ts</t>
+          <t>engines/creditLimit.ts</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -6927,17 +6927,17 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, administration, customer360</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, CheckoutDefaultLayout, PostpaidMonthlySummary, checkoutDetailedTables, checkoutSummaryRows, useCheckoutSummary, usePostpaidPlanAddons</t>
+          <t>CreditLimitCard, billingAccountModel</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6949,12 +6949,12 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>connectionEligibility</t>
+          <t>postpaidPricing</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>engines/connectionEligibility.ts</t>
+          <t>engines/postpaidPricing.ts</t>
         </is>
       </c>
       <c r="D17" s="20" t="inlineStr">
@@ -6963,17 +6963,21 @@
         </is>
       </c>
       <c r="E17" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G17" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G17" s="17" t="inlineStr">
+        <is>
+          <t>MsisdnPicker, CheckoutDefaultLayout, PostpaidMonthlySummary, checkoutDetailedTables, checkoutSummaryRows, useCheckoutSummary, usePostpaidPlanAddons</t>
+        </is>
+      </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6985,12 +6989,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>customerBenefitEngine</t>
+          <t>connectionEligibility</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>engines/customerBenefitEngine.ts</t>
+          <t>engines/connectionEligibility.ts</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -7006,14 +7010,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
         </is>
       </c>
-      <c r="G18" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidPlanAddonsStep, usePostpaidPlanAddons</t>
-        </is>
-      </c>
+      <c r="G18" s="17" t="inlineStr"/>
       <c r="H18" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7025,12 +7025,12 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>addonEligibility</t>
+          <t>customerBenefitEngine</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>engines/addonEligibility.ts</t>
+          <t>engines/customerBenefitEngine.ts</t>
         </is>
       </c>
       <c r="D19" s="20" t="inlineStr">
@@ -7039,17 +7039,21 @@
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidPlanAddonsStep, usePostpaidPlanAddons</t>
+        </is>
+      </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7061,12 +7065,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>fibreServiceability</t>
+          <t>addonEligibility</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>engines/fibreServiceability.ts</t>
+          <t>engines/addonEligibility.ts</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -7082,11 +7086,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
-        </is>
-      </c>
+      <c r="G20" s="17" t="inlineStr"/>
       <c r="H20" s="17" t="inlineStr">
         <is>
           <t>2026-10-05</t>
@@ -7101,12 +7101,12 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>personaEngine</t>
+          <t>fibreServiceability</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>engines/personaEngine.ts</t>
+          <t>engines/fibreServiceability.ts</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -7119,17 +7119,17 @@
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G21" s="17" t="inlineStr">
         <is>
-          <t>approvalAuthority, navigationEngine</t>
+          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7141,12 +7141,12 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>eligibilityGuard</t>
+          <t>personaEngine</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityGuard.ts</t>
+          <t>engines/personaEngine.ts</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -7155,17 +7155,21 @@
         </is>
       </c>
       <c r="E22" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F22" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
-        </is>
-      </c>
-      <c r="G22" s="17" t="inlineStr"/>
+          <t>dashboard, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
+        </is>
+      </c>
+      <c r="G22" s="17" t="inlineStr">
+        <is>
+          <t>approvalAuthority, navigationEngine</t>
+        </is>
+      </c>
       <c r="H22" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -7177,12 +7181,12 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>serviceLocationLookup</t>
+          <t>eligibilityGuard</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceLocationLookup.ts</t>
+          <t>engines/eligibilityGuard.ts</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
@@ -7195,14 +7199,10 @@
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>ZsbAddressStep</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr"/>
       <c r="H23" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -7217,12 +7217,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>restrictedCustomers</t>
+          <t>serviceLocationLookup</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>engines/restrictedCustomers.ts</t>
+          <t>engines/serviceLocationLookup.ts</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -7231,21 +7231,21 @@
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>7</v>
+        <v>8</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>order-management, trouble-ticketing-complaints, customer360, orders, support, tasks, tickets</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G24" s="17" t="inlineStr">
         <is>
-          <t>useRestrictedCustomers</t>
+          <t>ZsbAddressStep</t>
         </is>
       </c>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7653,12 +7653,12 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>searchScopeEngine</t>
+          <t>roleSwitchPurge</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>engines/searchScopeEngine.ts</t>
+          <t>engines/roleSwitchPurge.ts</t>
         </is>
       </c>
       <c r="D36" s="21" t="inlineStr">
@@ -7677,7 +7677,7 @@
       <c r="G36" s="17" t="inlineStr"/>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>uncommitted</t>
         </is>
       </c>
     </row>
@@ -7689,27 +7689,31 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>moduleDescriptions</t>
+          <t>searchScopeEngine</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>engines/moduleDescriptions.ts</t>
-        </is>
-      </c>
-      <c r="D37" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>engines/searchScopeEngine.ts</t>
+        </is>
+      </c>
+      <c r="D37" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E37" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F37" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F37" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G37" s="17" t="inlineStr"/>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7721,12 +7725,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>screenGrouping</t>
+          <t>moduleDescriptions</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>engines/screenGrouping.ts</t>
+          <t>engines/moduleDescriptions.ts</t>
         </is>
       </c>
       <c r="D38" s="23" t="inlineStr">
@@ -7748,40 +7752,32 @@
     <row r="39">
       <c r="A39" s="17" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>entityStore</t>
+          <t>screenGrouping</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>stores/entityStore.ts</t>
-        </is>
-      </c>
-      <c r="D39" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>engines/screenGrouping.ts</t>
+        </is>
+      </c>
+      <c r="D39" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E39" s="17" t="n">
-        <v>24</v>
-      </c>
-      <c r="F39" s="17" t="inlineStr">
-        <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G39" s="17" t="inlineStr">
-        <is>
-          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F39" s="17" t="inlineStr"/>
+      <c r="G39" s="17" t="inlineStr"/>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7793,12 +7789,12 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>customerContextStore</t>
+          <t>entityStore</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>stores/customerContextStore.ts</t>
+          <t>stores/entityStore.ts</t>
         </is>
       </c>
       <c r="D40" s="20" t="inlineStr">
@@ -7807,21 +7803,21 @@
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F40" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G40" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, useActedForCustomer, useWizardDraftActions, authStore</t>
+          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
         </is>
       </c>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7833,12 +7829,12 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>personaStore</t>
+          <t>customerContextStore</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>stores/personaStore.ts</t>
+          <t>stores/customerContextStore.ts</t>
         </is>
       </c>
       <c r="D41" s="20" t="inlineStr">
@@ -7851,17 +7847,17 @@
       </c>
       <c r="F41" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, support, tasks, tickets</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G41" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, eligibilityRowsModel, ActivationCompleteScreen, AppointmentBookingStep, PostpaidPlanAddonsStep, TicketCreationModal, useCheckoutSummary, useIdLookup, useRestrictedCustomers, configStore</t>
+          <t>ActivationCompleteScreen, useActedForCustomer, useWizardDraftActions, roleSwitchPurge, authStore</t>
         </is>
       </c>
       <c r="H41" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7873,12 +7869,12 @@
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>authStore</t>
+          <t>personaStore</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>stores/authStore.ts</t>
+          <t>stores/personaStore.ts</t>
         </is>
       </c>
       <c r="D42" s="20" t="inlineStr">
@@ -7887,16 +7883,16 @@
         </is>
       </c>
       <c r="E42" s="17" t="n">
-        <v>21</v>
+        <v>23</v>
       </c>
       <c r="F42" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, support, tasks, tickets</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G42" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore</t>
+          <t>MsisdnPicker, eligibilityRowsModel, ActivationCompleteScreen, AppointmentBookingStep, PostpaidPlanAddonsStep, TicketCreationModal, useCheckoutSummary, useIdLookup, useRestrictedCustomers, configStore</t>
         </is>
       </c>
       <c r="H42" s="17" t="inlineStr">
@@ -7913,12 +7909,12 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>notificationStore</t>
+          <t>authStore</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>stores/notificationStore.ts</t>
+          <t>stores/authStore.ts</t>
         </is>
       </c>
       <c r="D43" s="20" t="inlineStr">
@@ -7927,21 +7923,21 @@
         </is>
       </c>
       <c r="E43" s="17" t="n">
-        <v>20</v>
+        <v>21</v>
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G43" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useJourneyMilestones, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, useSubmit</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore</t>
         </is>
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7953,12 +7949,12 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>workflowStore</t>
+          <t>notificationStore</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>stores/workflowStore.ts</t>
+          <t>stores/notificationStore.ts</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
@@ -7967,21 +7963,21 @@
         </is>
       </c>
       <c r="E44" s="17" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F44" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
         </is>
       </c>
       <c r="G44" s="17" t="inlineStr">
         <is>
-          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useJourneyMilestones, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, roleSwitchPurge, useSubmit</t>
         </is>
       </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7993,35 +7989,35 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>customerVerificationStore</t>
+          <t>workflowStore</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>stores/customerVerificationStore.ts</t>
-        </is>
-      </c>
-      <c r="D45" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>stores/workflowStore.ts</t>
+        </is>
+      </c>
+      <c r="D45" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E45" s="17" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F45" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
         </is>
       </c>
       <c r="G45" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation, roleSwitchPurge</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8033,12 +8029,12 @@
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>qnomyQueueStore</t>
+          <t>customerVerificationStore</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>stores/qnomyQueueStore.ts</t>
+          <t>stores/customerVerificationStore.ts</t>
         </is>
       </c>
       <c r="D46" s="21" t="inlineStr">
@@ -8051,13 +8047,17 @@
       </c>
       <c r="F46" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G46" s="17" t="inlineStr"/>
+          <t>customer360</t>
+        </is>
+      </c>
+      <c r="G46" s="17" t="inlineStr">
+        <is>
+          <t>VerificationGate</t>
+        </is>
+      </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8069,12 +8069,12 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>regionStore</t>
+          <t>qnomyQueueStore</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>stores/regionStore.ts</t>
+          <t>stores/qnomyQueueStore.ts</t>
         </is>
       </c>
       <c r="D47" s="21" t="inlineStr">
@@ -8093,7 +8093,7 @@
       <c r="G47" s="17" t="inlineStr"/>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -8105,12 +8105,12 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>sidebarStore</t>
+          <t>regionStore</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>stores/sidebarStore.ts</t>
+          <t>stores/regionStore.ts</t>
         </is>
       </c>
       <c r="D48" s="21" t="inlineStr">
@@ -8129,7 +8129,7 @@
       <c r="G48" s="17" t="inlineStr"/>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8141,12 +8141,12 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>themeStore</t>
+          <t>sidebarStore</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>stores/themeStore.ts</t>
+          <t>stores/sidebarStore.ts</t>
         </is>
       </c>
       <c r="D49" s="21" t="inlineStr">
@@ -8165,7 +8165,7 @@
       <c r="G49" s="17" t="inlineStr"/>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8177,67 +8177,63 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>configStore</t>
+          <t>themeStore</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>stores/configStore.ts</t>
-        </is>
-      </c>
-      <c r="D50" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>stores/themeStore.ts</t>
+        </is>
+      </c>
+      <c r="D50" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E50" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F50" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F50" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G50" s="17" t="inlineStr"/>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="17" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>useEnterToSubmit</t>
+          <t>configStore</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>hooks/useEnterToSubmit.ts</t>
-        </is>
-      </c>
-      <c r="D51" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>stores/configStore.ts</t>
+        </is>
+      </c>
+      <c r="D51" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E51" s="17" t="n">
-        <v>12</v>
-      </c>
-      <c r="F51" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G51" s="17" t="inlineStr">
-        <is>
-          <t>VerificationGate, useIdLookup</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F51" s="17" t="inlineStr"/>
+      <c r="G51" s="17" t="inlineStr"/>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8249,12 +8245,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>useSearchListNav</t>
+          <t>useRestrictedCustomers</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSearchListNav.ts</t>
+          <t>hooks/useRestrictedCustomers.ts</t>
         </is>
       </c>
       <c r="D52" s="20" t="inlineStr">
@@ -8263,21 +8259,21 @@
         </is>
       </c>
       <c r="E52" s="17" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F52" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G52" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
+          <t>TicketCreationModal</t>
         </is>
       </c>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8289,12 +8285,12 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>useAreaOptions</t>
+          <t>useEnterToSubmit</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>hooks/useAreaOptions.ts</t>
+          <t>hooks/useEnterToSubmit.ts</t>
         </is>
       </c>
       <c r="D53" s="20" t="inlineStr">
@@ -8303,21 +8299,21 @@
         </is>
       </c>
       <c r="E53" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F53" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G53" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep, ZsbAddressStep</t>
+          <t>VerificationGate, useIdLookup</t>
         </is>
       </c>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8329,12 +8325,12 @@
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>useRestrictedCustomers</t>
+          <t>useSearchListNav</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>hooks/useRestrictedCustomers.ts</t>
+          <t>hooks/useSearchListNav.ts</t>
         </is>
       </c>
       <c r="D54" s="20" t="inlineStr">
@@ -8343,21 +8339,21 @@
         </is>
       </c>
       <c r="E54" s="17" t="n">
-        <v>7</v>
+        <v>12</v>
       </c>
       <c r="F54" s="17" t="inlineStr">
         <is>
-          <t>order-management, trouble-ticketing-complaints, customer360, orders, support, tasks, tickets</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G54" s="17" t="inlineStr">
         <is>
-          <t>TicketCreationModal</t>
+          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
         </is>
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -8369,12 +8365,12 @@
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>useSubmit</t>
+          <t>useAreaOptions</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSubmit.ts</t>
+          <t>hooks/useAreaOptions.ts</t>
         </is>
       </c>
       <c r="D55" s="20" t="inlineStr">
@@ -8383,17 +8379,21 @@
         </is>
       </c>
       <c r="E55" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
-        </is>
-      </c>
-      <c r="G55" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G55" s="17" t="inlineStr">
+        <is>
+          <t>BillingAccountStep, ZsbAddressStep</t>
+        </is>
+      </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -8405,68 +8405,64 @@
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>useMinWidth</t>
+          <t>useSubmit</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>hooks/useMinWidth.ts</t>
-        </is>
-      </c>
-      <c r="D56" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>hooks/useSubmit.ts</t>
+        </is>
+      </c>
+      <c r="D56" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E56" s="17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
         </is>
       </c>
       <c r="G56" s="17" t="inlineStr"/>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="57">
       <c r="A57" s="17" t="inlineStr">
         <is>
-          <t>Helper</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
-          <t>statusTone</t>
+          <t>useMinWidth</t>
         </is>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>lib/statusTone.ts</t>
-        </is>
-      </c>
-      <c r="D57" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>hooks/useMinWidth.ts</t>
+        </is>
+      </c>
+      <c r="D57" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E57" s="17" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G57" s="17" t="inlineStr">
-        <is>
-          <t>ruleEngine</t>
-        </is>
-      </c>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G57" s="17" t="inlineStr"/>
       <c r="H57" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -8481,12 +8477,12 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>format</t>
+          <t>statusTone</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>lib/format.ts</t>
+          <t>lib/statusTone.ts</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
@@ -8495,21 +8491,21 @@
         </is>
       </c>
       <c r="E58" s="17" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F58" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, tasks</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G58" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, GuidedContactStep, IdLookupStep, postpaidPlanModel, StepSummaryPanel, stepSummary, customer360Engine, postpaidPricing</t>
+          <t>ruleEngine</t>
         </is>
       </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -8521,12 +8517,12 @@
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>buildEnv</t>
+          <t>format</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>lib/buildEnv.ts</t>
+          <t>lib/format.ts</t>
         </is>
       </c>
       <c r="D59" s="20" t="inlineStr">
@@ -8535,21 +8531,21 @@
         </is>
       </c>
       <c r="E59" s="17" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F59" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, tasks</t>
         </is>
       </c>
       <c r="G59" s="17" t="inlineStr">
         <is>
-          <t>syntheticMarker, navigationEngine</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, GuidedContactStep, IdLookupStep, postpaidPlanModel, StepSummaryPanel, stepSummary, customer360Engine, postpaidPricing</t>
         </is>
       </c>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8561,12 +8557,12 @@
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>deviceType</t>
+          <t>buildEnv</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>lib/deviceType.ts</t>
+          <t>lib/buildEnv.ts</t>
         </is>
       </c>
       <c r="D60" s="20" t="inlineStr">
@@ -8575,21 +8571,21 @@
         </is>
       </c>
       <c r="E60" s="17" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F60" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G60" s="17" t="inlineStr">
         <is>
-          <t>IdFileUpload, PassportScanSections, SimSerialScanner, SimTypeStep, cafTypes</t>
+          <t>syntheticMarker, navigationEngine</t>
         </is>
       </c>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8601,12 +8597,12 @@
       </c>
       <c r="B61" s="17" t="inlineStr">
         <is>
-          <t>taskId</t>
+          <t>deviceType</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>lib/taskId.ts</t>
+          <t>lib/deviceType.ts</t>
         </is>
       </c>
       <c r="D61" s="20" t="inlineStr">
@@ -8615,16 +8611,16 @@
         </is>
       </c>
       <c r="E61" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G61" s="17" t="inlineStr">
         <is>
-          <t>useWizardDraftActions</t>
+          <t>IdFileUpload, PassportScanSections, SimSerialScanner, SimTypeStep, cafTypes</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr">
@@ -8641,12 +8637,12 @@
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>connectionType</t>
+          <t>taskId</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>lib/connectionType.ts</t>
+          <t>lib/taskId.ts</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr">
@@ -8655,21 +8651,21 @@
         </is>
       </c>
       <c r="E62" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G62" s="17" t="inlineStr">
         <is>
-          <t>ConnectionTypeTag</t>
+          <t>useWizardDraftActions</t>
         </is>
       </c>
       <c r="H62" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8681,12 +8677,12 @@
       </c>
       <c r="B63" s="17" t="inlineStr">
         <is>
-          <t>serviceTypeTag</t>
+          <t>connectionType</t>
         </is>
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>lib/serviceTypeTag.ts</t>
+          <t>lib/connectionType.ts</t>
         </is>
       </c>
       <c r="D63" s="20" t="inlineStr">
@@ -8704,7 +8700,7 @@
       </c>
       <c r="G63" s="17" t="inlineStr">
         <is>
-          <t>ServiceTypeTag</t>
+          <t>ConnectionTypeTag</t>
         </is>
       </c>
       <c r="H63" s="17" t="inlineStr">
@@ -8721,31 +8717,35 @@
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>screenName</t>
+          <t>serviceTypeTag</t>
         </is>
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
-          <t>lib/screenName.ts</t>
-        </is>
-      </c>
-      <c r="D64" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>lib/serviceTypeTag.ts</t>
+        </is>
+      </c>
+      <c r="D64" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E64" s="17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G64" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G64" s="17" t="inlineStr">
+        <is>
+          <t>ServiceTypeTag</t>
+        </is>
+      </c>
       <c r="H64" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8757,12 +8757,12 @@
       </c>
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>values</t>
+          <t>screenName</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>lib/values.ts</t>
+          <t>lib/screenName.ts</t>
         </is>
       </c>
       <c r="D65" s="21" t="inlineStr">
@@ -8775,22 +8775,58 @@
       </c>
       <c r="F65" s="17" t="inlineStr">
         <is>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G65" s="17" t="inlineStr"/>
+      <c r="H65" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="66">
+      <c r="A66" s="17" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="B66" s="17" t="inlineStr">
+        <is>
+          <t>values</t>
+        </is>
+      </c>
+      <c r="C66" s="17" t="inlineStr">
+        <is>
+          <t>lib/values.ts</t>
+        </is>
+      </c>
+      <c r="D66" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
+        </is>
+      </c>
+      <c r="E66" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F66" s="17" t="inlineStr">
+        <is>
           <t>customer360</t>
         </is>
       </c>
-      <c r="G65" s="17" t="inlineStr">
+      <c r="G66" s="17" t="inlineStr">
         <is>
           <t>customer360Demo</t>
         </is>
       </c>
-      <c r="H65" s="17" t="inlineStr">
+      <c r="H66" s="17" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H65"/>
+  <autoFilter ref="A1:H66"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Retiree no longer validated with a government system; milestone toasts not displayed (code kept)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -1932,7 +1932,7 @@
       </c>
       <c r="H5" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -1972,7 +1972,7 @@
       </c>
       <c r="H6" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2012,7 +2012,7 @@
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2092,7 +2092,7 @@
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2332,7 +2332,7 @@
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2372,7 +2372,7 @@
       </c>
       <c r="H16" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2920,7 +2920,7 @@
       <c r="G30" s="17" t="inlineStr"/>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3168,7 +3168,7 @@
       </c>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3208,7 +3208,7 @@
       </c>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3404,7 +3404,7 @@
       <c r="G43" s="17" t="inlineStr"/>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3440,7 +3440,7 @@
       <c r="G44" s="17" t="inlineStr"/>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3520,7 +3520,7 @@
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3600,7 +3600,7 @@
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3640,7 +3640,7 @@
       </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -3716,7 +3716,7 @@
       <c r="G51" s="17" t="inlineStr"/>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4060,7 +4060,7 @@
       <c r="G60" s="17" t="inlineStr"/>
       <c r="H60" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4300,7 +4300,7 @@
       </c>
       <c r="H66" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4376,7 +4376,7 @@
       <c r="G68" s="17" t="inlineStr"/>
       <c r="H68" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4448,7 +4448,7 @@
       <c r="G70" s="17" t="inlineStr"/>
       <c r="H70" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4488,7 +4488,7 @@
       </c>
       <c r="H71" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4916,7 +4916,7 @@
       </c>
       <c r="H82" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4996,7 +4996,7 @@
       </c>
       <c r="H84" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5072,7 +5072,7 @@
       </c>
       <c r="H86" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5108,7 +5108,7 @@
       <c r="G87" s="17" t="inlineStr"/>
       <c r="H87" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5144,7 +5144,7 @@
       <c r="G88" s="17" t="inlineStr"/>
       <c r="H88" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5260,7 +5260,7 @@
       <c r="G91" s="17" t="inlineStr"/>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5336,7 +5336,7 @@
       <c r="G93" s="17" t="inlineStr"/>
       <c r="H93" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5372,7 +5372,7 @@
       <c r="G94" s="17" t="inlineStr"/>
       <c r="H94" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5448,7 +5448,7 @@
       <c r="G96" s="17" t="inlineStr"/>
       <c r="H96" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5488,7 +5488,7 @@
       </c>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5524,7 +5524,7 @@
       <c r="G98" s="17" t="inlineStr"/>
       <c r="H98" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5560,7 +5560,7 @@
       <c r="G99" s="17" t="inlineStr"/>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5596,7 +5596,7 @@
       <c r="G100" s="17" t="inlineStr"/>
       <c r="H100" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5636,7 +5636,7 @@
       </c>
       <c r="H101" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5672,7 +5672,7 @@
       <c r="G102" s="17" t="inlineStr"/>
       <c r="H102" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5816,7 +5816,7 @@
       <c r="G106" s="17" t="inlineStr"/>
       <c r="H106" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5960,7 +5960,7 @@
       <c r="G110" s="17" t="inlineStr"/>
       <c r="H110" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5996,7 +5996,7 @@
       <c r="G111" s="17" t="inlineStr"/>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6775,12 +6775,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>serviceCall</t>
+          <t>eligibilityEngine</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceCall.ts</t>
+          <t>engines/eligibilityEngine.ts</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -6789,21 +6789,21 @@
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>13</v>
+        <v>12</v>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
+          <t>eligibilityRowsModel, eligibilityTypes, idLookupModel, useIdLookup</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6815,12 +6815,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>eligibilityEngine</t>
+          <t>milestoneEngine</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityEngine.ts</t>
+          <t>engines/milestoneEngine.ts</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
@@ -6838,12 +6838,12 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>eligibilityRowsModel, eligibilityTypes, idLookupModel, useIdLookup</t>
+          <t>guidedWizardTypes, useJourneyMilestones</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6855,12 +6855,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>milestoneEngine</t>
+          <t>serviceCall</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>engines/milestoneEngine.ts</t>
+          <t>engines/serviceCall.ts</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>guidedWizardTypes, useJourneyMilestones</t>
+          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -7271,7 +7271,7 @@
       <c r="G24" s="17" t="inlineStr"/>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -8811,7 +8811,7 @@
       </c>
       <c r="H65" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Mobile Postpaid audit: High-severity fixes (access, protected data, customer window, plans and discounts, eligibility scope, B2B2C, billing, bill limit, reserved numbers)
Co-Authored-By: Claude Sonnet 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -15,7 +15,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'UI Components'!$A$1:$H$119</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$68</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="3" hidden="1">'Shared Code'!$A$1:$H$69</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -763,10 +763,10 @@
         </is>
       </c>
       <c r="C9" s="17" t="n">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D9" s="17" t="n">
-        <v>32</v>
+        <v>33</v>
       </c>
       <c r="E9" s="17" t="n">
         <v>6</v>
@@ -855,14 +855,14 @@
       </c>
       <c r="B13" s="18" t="inlineStr">
         <is>
-          <t>118 UI components + 67 non-UI files</t>
+          <t>118 UI components + 68 non-UI files</t>
         </is>
       </c>
       <c r="C13" s="18" t="n">
-        <v>185</v>
+        <v>186</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>157</v>
+        <v>158</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>23</v>
@@ -1847,7 +1847,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, ScanFailureNotice, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, RestrictedCustomerNotice, RestrictedRowsNotice, ValidationStatus, ZsbAddressStep, CustomerViewButton, StepSummarySection, WizardFooter, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, ScanFailureNotice, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, RestrictedCustomerNotice, RestrictedRowsNotice, ValidationStatus, ZsbAddressStep, CustomerViewButton, StepSummarySection, WizardFooter, ChoiceCards, DataTable, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
@@ -2407,7 +2407,7 @@
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanAddonsStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
+          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
@@ -2660,12 +2660,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>SignaturePad</t>
+          <t>SegmentedTabs</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/SignaturePad.tsx</t>
+          <t>components/primitives/SegmentedTabs.tsx</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -2678,14 +2678,10 @@
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
-        </is>
-      </c>
-      <c r="G24" s="17" t="inlineStr">
-        <is>
-          <t>SignatureCapture</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360, tickets</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr"/>
       <c r="H24" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -2700,12 +2696,12 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>ConnectionTypeTag</t>
+          <t>SignaturePad</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/ConnectionTypeTag.tsx</t>
+          <t>components/primitives/SignaturePad.tsx</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
@@ -2714,21 +2710,21 @@
         </is>
       </c>
       <c r="E25" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G25" s="17" t="inlineStr">
         <is>
-          <t>FixedPlanStep, PostpaidPlanCard, PrepaidPlanCard</t>
+          <t>SignatureCapture</t>
         </is>
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -2740,12 +2736,12 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>IconButton</t>
+          <t>ConnectionTypeTag</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/IconButton.tsx</t>
+          <t>components/primitives/ConnectionTypeTag.tsx</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -2763,12 +2759,12 @@
       </c>
       <c r="G26" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload</t>
+          <t>FixedPlanStep, PostpaidPlanCard, PrepaidPlanCard</t>
         </is>
       </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2780,12 +2776,12 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>ServiceTypeTag</t>
+          <t>IconButton</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/ServiceTypeTag.tsx</t>
+          <t>components/primitives/IconButton.tsx</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
@@ -2803,12 +2799,12 @@
       </c>
       <c r="G27" s="17" t="inlineStr">
         <is>
-          <t>LineSelectionStep, ConnectionTypeTag</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload</t>
         </is>
       </c>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2820,12 +2816,12 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>ChoiceCards</t>
+          <t>ServiceTypeTag</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/ChoiceCards.tsx</t>
+          <t>components/primitives/ServiceTypeTag.tsx</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -2834,17 +2830,21 @@
         </is>
       </c>
       <c r="E28" s="17" t="n">
-        <v>7</v>
+        <v>10</v>
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, customer360</t>
-        </is>
-      </c>
-      <c r="G28" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G28" s="17" t="inlineStr">
+        <is>
+          <t>LineSelectionStep, ConnectionTypeTag</t>
+        </is>
+      </c>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -2856,12 +2856,12 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>PanelIcon</t>
+          <t>ChoiceCards</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/PanelIcon.tsx</t>
+          <t>components/primitives/ChoiceCards.tsx</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
@@ -2870,21 +2870,17 @@
         </is>
       </c>
       <c r="E29" s="17" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, navigation, administration, customer360, orders, support</t>
-        </is>
-      </c>
-      <c r="G29" s="17" t="inlineStr">
-        <is>
-          <t>Tabs</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, customer360</t>
+        </is>
+      </c>
+      <c r="G29" s="17" t="inlineStr"/>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -2896,12 +2892,12 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>Radio</t>
+          <t>PanelIcon</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/Radio.tsx</t>
+          <t>components/primitives/PanelIcon.tsx</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
@@ -2914,13 +2910,17 @@
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
-        </is>
-      </c>
-      <c r="G30" s="17" t="inlineStr"/>
+          <t>trouble-ticketing-complaints, navigation, administration, customer360, orders, support</t>
+        </is>
+      </c>
+      <c r="G30" s="17" t="inlineStr">
+        <is>
+          <t>Tabs</t>
+        </is>
+      </c>
       <c r="H30" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -2932,12 +2932,12 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>Tabs</t>
+          <t>Radio</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/Tabs.tsx</t>
+          <t>components/primitives/Radio.tsx</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">
@@ -2946,17 +2946,17 @@
         </is>
       </c>
       <c r="E31" s="17" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, administration, customer360, orders, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G31" s="17" t="inlineStr"/>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -2968,12 +2968,12 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>SegmentedTabs</t>
+          <t>Tabs</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>components/primitives/SegmentedTabs.tsx</t>
+          <t>components/primitives/Tabs.tsx</t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
@@ -2982,11 +2982,11 @@
         </is>
       </c>
       <c r="E32" s="17" t="n">
-        <v>3</v>
+        <v>5</v>
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>administration, customer360, tickets</t>
+          <t>trouble-ticketing-complaints, administration, customer360, orders, support</t>
         </is>
       </c>
       <c r="G32" s="17" t="inlineStr"/>
@@ -6312,7 +6312,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H69"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13.50" customWidth="1" min="1" max="1"/>
@@ -6438,7 +6438,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, agentPrivilegeEngine, agentProfileEngine, approvalAuthority, customer360VisibilityEngine, navigationEngine, personaEngine, qnomyQueueEngine, screenGrouping, configStore</t>
+          <t>agentPrivilegeEngine, agentProfileEngine, approvalAuthority, customer360VisibilityEngine, navigationEngine, personaEngine, qnomyQueueEngine, screenGrouping, configStore</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
@@ -6575,12 +6575,12 @@
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>restrictedCustomers</t>
+          <t>personaEngine</t>
         </is>
       </c>
       <c r="C7" s="17" t="inlineStr">
         <is>
-          <t>engines/restrictedCustomers.ts</t>
+          <t>engines/personaEngine.ts</t>
         </is>
       </c>
       <c r="D7" s="20" t="inlineStr">
@@ -6593,17 +6593,17 @@
       </c>
       <c r="F7" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
         </is>
       </c>
       <c r="G7" s="17" t="inlineStr">
         <is>
-          <t>useRestrictedCustomers</t>
+          <t>approvalAuthority, navigationEngine</t>
         </is>
       </c>
       <c r="H7" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -6615,12 +6615,12 @@
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>ruleEngine</t>
+          <t>restrictedCustomers</t>
         </is>
       </c>
       <c r="C8" s="17" t="inlineStr">
         <is>
-          <t>engines/ruleEngine.ts</t>
+          <t>engines/restrictedCustomers.ts</t>
         </is>
       </c>
       <c r="D8" s="20" t="inlineStr">
@@ -6633,12 +6633,12 @@
       </c>
       <c r="F8" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G8" s="17" t="inlineStr">
         <is>
-          <t>BillLimitEditor, CreditCheckPanel, eligibilityRowsModel, FixedPlanStep, TicketCreationModal</t>
+          <t>useRestrictedCustomers</t>
         </is>
       </c>
       <c r="H8" s="17" t="inlineStr">
@@ -6655,12 +6655,12 @@
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>billingBalance</t>
+          <t>ruleEngine</t>
         </is>
       </c>
       <c r="C9" s="17" t="inlineStr">
         <is>
-          <t>engines/billingBalance.ts</t>
+          <t>engines/ruleEngine.ts</t>
         </is>
       </c>
       <c r="D9" s="20" t="inlineStr">
@@ -6669,21 +6669,21 @@
         </is>
       </c>
       <c r="E9" s="17" t="n">
-        <v>14</v>
+        <v>15</v>
       </c>
       <c r="F9" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, product-lines, navigation, administration, customer-search, customer360, orders</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, support</t>
         </is>
       </c>
       <c r="G9" s="17" t="inlineStr">
         <is>
-          <t>customer360Demo, customer360Engine</t>
+          <t>BillLimitEditor, CreditCheckPanel, eligibilityRowsModel, FixedPlanStep, TicketCreationModal</t>
         </is>
       </c>
       <c r="H9" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6695,12 +6695,12 @@
       </c>
       <c r="B10" s="17" t="inlineStr">
         <is>
-          <t>customer360Engine</t>
+          <t>billingBalance</t>
         </is>
       </c>
       <c r="C10" s="17" t="inlineStr">
         <is>
-          <t>engines/customer360Engine.ts</t>
+          <t>engines/billingBalance.ts</t>
         </is>
       </c>
       <c r="D10" s="20" t="inlineStr">
@@ -6718,12 +6718,12 @@
       </c>
       <c r="G10" s="17" t="inlineStr">
         <is>
-          <t>customer360Demo, customerServicesEngine</t>
+          <t>customer360Demo, customer360Engine</t>
         </is>
       </c>
       <c r="H10" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6735,12 +6735,12 @@
       </c>
       <c r="B11" s="17" t="inlineStr">
         <is>
-          <t>customerServicesEngine</t>
+          <t>customer360Engine</t>
         </is>
       </c>
       <c r="C11" s="17" t="inlineStr">
         <is>
-          <t>engines/customerServicesEngine.ts</t>
+          <t>engines/customer360Engine.ts</t>
         </is>
       </c>
       <c r="D11" s="20" t="inlineStr">
@@ -6758,12 +6758,12 @@
       </c>
       <c r="G11" s="17" t="inlineStr">
         <is>
-          <t>lineSelectionModel, customer360Demo, connectionEligibility, customer360Engine</t>
+          <t>customer360Demo, customerServicesEngine</t>
         </is>
       </c>
       <c r="H11" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -6775,12 +6775,12 @@
       </c>
       <c r="B12" s="17" t="inlineStr">
         <is>
-          <t>eligibilityEngine</t>
+          <t>customerServicesEngine</t>
         </is>
       </c>
       <c r="C12" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityEngine.ts</t>
+          <t>engines/customerServicesEngine.ts</t>
         </is>
       </c>
       <c r="D12" s="20" t="inlineStr">
@@ -6789,21 +6789,21 @@
         </is>
       </c>
       <c r="E12" s="17" t="n">
-        <v>12</v>
+        <v>14</v>
       </c>
       <c r="F12" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, product-lines, navigation, administration, customer-search, customer360, orders</t>
         </is>
       </c>
       <c r="G12" s="17" t="inlineStr">
         <is>
-          <t>eligibilityRowsModel, eligibilityTypes, idLookupModel, useIdLookup</t>
+          <t>lineSelectionModel, customer360Demo, connectionEligibility, customer360Engine</t>
         </is>
       </c>
       <c r="H12" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -6815,12 +6815,12 @@
       </c>
       <c r="B13" s="17" t="inlineStr">
         <is>
-          <t>milestoneEngine</t>
+          <t>eligibilityEngine</t>
         </is>
       </c>
       <c r="C13" s="17" t="inlineStr">
         <is>
-          <t>engines/milestoneEngine.ts</t>
+          <t>engines/eligibilityEngine.ts</t>
         </is>
       </c>
       <c r="D13" s="20" t="inlineStr">
@@ -6838,12 +6838,12 @@
       </c>
       <c r="G13" s="17" t="inlineStr">
         <is>
-          <t>guidedWizardTypes, useJourneyMilestones</t>
+          <t>eligibilityRowsModel, eligibilityTypes, idLookupModel, useIdLookup</t>
         </is>
       </c>
       <c r="H13" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6855,12 +6855,12 @@
       </c>
       <c r="B14" s="17" t="inlineStr">
         <is>
-          <t>serviceCall</t>
+          <t>milestoneEngine</t>
         </is>
       </c>
       <c r="C14" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceCall.ts</t>
+          <t>engines/milestoneEngine.ts</t>
         </is>
       </c>
       <c r="D14" s="20" t="inlineStr">
@@ -6878,12 +6878,12 @@
       </c>
       <c r="G14" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
+          <t>guidedWizardTypes, useJourneyMilestones</t>
         </is>
       </c>
       <c r="H14" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6895,12 +6895,12 @@
       </c>
       <c r="B15" s="17" t="inlineStr">
         <is>
-          <t>activityEngine</t>
+          <t>serviceCall</t>
         </is>
       </c>
       <c r="C15" s="17" t="inlineStr">
         <is>
-          <t>engines/activityEngine.ts</t>
+          <t>engines/serviceCall.ts</t>
         </is>
       </c>
       <c r="D15" s="20" t="inlineStr">
@@ -6909,21 +6909,21 @@
         </is>
       </c>
       <c r="E15" s="17" t="n">
-        <v>11</v>
+        <v>12</v>
       </c>
       <c r="F15" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G15" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, useWizardDraftActions</t>
+          <t>DemoFaultPanel, ValidationStatus, useIdLookup</t>
         </is>
       </c>
       <c r="H15" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6935,12 +6935,12 @@
       </c>
       <c r="B16" s="17" t="inlineStr">
         <is>
-          <t>businessSegment</t>
+          <t>activityEngine</t>
         </is>
       </c>
       <c r="C16" s="17" t="inlineStr">
         <is>
-          <t>engines/businessSegment.ts</t>
+          <t>engines/activityEngine.ts</t>
         </is>
       </c>
       <c r="D16" s="20" t="inlineStr">
@@ -6953,12 +6953,12 @@
       </c>
       <c r="F16" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, navigation, administration, customer-search, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G16" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep, customer360Demo, businessAccountEngine</t>
+          <t>ActivationCompleteScreen, useWizardDraftActions</t>
         </is>
       </c>
       <c r="H16" s="17" t="inlineStr">
@@ -6975,12 +6975,12 @@
       </c>
       <c r="B17" s="17" t="inlineStr">
         <is>
-          <t>creditLimit</t>
+          <t>businessSegment</t>
         </is>
       </c>
       <c r="C17" s="17" t="inlineStr">
         <is>
-          <t>engines/creditLimit.ts</t>
+          <t>engines/businessSegment.ts</t>
         </is>
       </c>
       <c r="D17" s="20" t="inlineStr">
@@ -6993,17 +6993,17 @@
       </c>
       <c r="F17" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, navigation, administration, customer-search, customer360</t>
         </is>
       </c>
       <c r="G17" s="17" t="inlineStr">
         <is>
-          <t>CreditLimitCard, billingAccountModel</t>
+          <t>BillingAccountStep, customer360Demo, businessAccountEngine</t>
         </is>
       </c>
       <c r="H17" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7015,12 +7015,12 @@
       </c>
       <c r="B18" s="17" t="inlineStr">
         <is>
-          <t>postpaidPricing</t>
+          <t>creditLimit</t>
         </is>
       </c>
       <c r="C18" s="17" t="inlineStr">
         <is>
-          <t>engines/postpaidPricing.ts</t>
+          <t>engines/creditLimit.ts</t>
         </is>
       </c>
       <c r="D18" s="20" t="inlineStr">
@@ -7033,17 +7033,17 @@
       </c>
       <c r="F18" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, administration, customer360</t>
         </is>
       </c>
       <c r="G18" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, CheckoutDefaultLayout, PostpaidMonthlySummary, checkoutDetailedTables, checkoutSummaryRows, useCheckoutSummary, usePostpaidPlanAddons</t>
+          <t>CreditLimitCard, billingAccountModel</t>
         </is>
       </c>
       <c r="H18" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -7055,12 +7055,12 @@
       </c>
       <c r="B19" s="17" t="inlineStr">
         <is>
-          <t>connectionEligibility</t>
+          <t>postpaidPricing</t>
         </is>
       </c>
       <c r="C19" s="17" t="inlineStr">
         <is>
-          <t>engines/connectionEligibility.ts</t>
+          <t>engines/postpaidPricing.ts</t>
         </is>
       </c>
       <c r="D19" s="20" t="inlineStr">
@@ -7069,17 +7069,21 @@
         </is>
       </c>
       <c r="E19" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F19" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
-        </is>
-      </c>
-      <c r="G19" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, administration</t>
+        </is>
+      </c>
+      <c r="G19" s="17" t="inlineStr">
+        <is>
+          <t>MsisdnPicker, CheckoutDefaultLayout, PostpaidMonthlySummary, checkoutDetailedTables, checkoutSummaryRows, useCheckoutSummary, usePostpaidPlanAddons</t>
+        </is>
+      </c>
       <c r="H19" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7091,12 +7095,12 @@
       </c>
       <c r="B20" s="17" t="inlineStr">
         <is>
-          <t>customerBenefitEngine</t>
+          <t>connectionEligibility</t>
         </is>
       </c>
       <c r="C20" s="17" t="inlineStr">
         <is>
-          <t>engines/customerBenefitEngine.ts</t>
+          <t>engines/connectionEligibility.ts</t>
         </is>
       </c>
       <c r="D20" s="20" t="inlineStr">
@@ -7112,14 +7116,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
         </is>
       </c>
-      <c r="G20" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidPlanAddonsStep, usePostpaidPlanAddons</t>
-        </is>
-      </c>
+      <c r="G20" s="17" t="inlineStr"/>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7131,12 +7131,12 @@
       </c>
       <c r="B21" s="17" t="inlineStr">
         <is>
-          <t>addonEligibility</t>
+          <t>customerBenefitEngine</t>
         </is>
       </c>
       <c r="C21" s="17" t="inlineStr">
         <is>
-          <t>engines/addonEligibility.ts</t>
+          <t>engines/customerBenefitEngine.ts</t>
         </is>
       </c>
       <c r="D21" s="20" t="inlineStr">
@@ -7145,17 +7145,21 @@
         </is>
       </c>
       <c r="E21" s="17" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="F21" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G21" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G21" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidPlanAddonsStep, usePostpaidPlanAddons</t>
+        </is>
+      </c>
       <c r="H21" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7167,12 +7171,12 @@
       </c>
       <c r="B22" s="17" t="inlineStr">
         <is>
-          <t>fibreServiceability</t>
+          <t>addonCategories</t>
         </is>
       </c>
       <c r="C22" s="17" t="inlineStr">
         <is>
-          <t>engines/fibreServiceability.ts</t>
+          <t>engines/addonCategories.ts</t>
         </is>
       </c>
       <c r="D22" s="20" t="inlineStr">
@@ -7188,14 +7192,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G22" s="17" t="inlineStr">
-        <is>
-          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
-        </is>
-      </c>
+      <c r="G22" s="17" t="inlineStr"/>
       <c r="H22" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>uncommitted</t>
         </is>
       </c>
     </row>
@@ -7207,12 +7207,12 @@
       </c>
       <c r="B23" s="17" t="inlineStr">
         <is>
-          <t>personaEngine</t>
+          <t>addonEligibility</t>
         </is>
       </c>
       <c r="C23" s="17" t="inlineStr">
         <is>
-          <t>engines/personaEngine.ts</t>
+          <t>engines/addonEligibility.ts</t>
         </is>
       </c>
       <c r="D23" s="20" t="inlineStr">
@@ -7225,17 +7225,13 @@
       </c>
       <c r="F23" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, product-lines, sim-number-management, navigation, administration, customer360, orders, profile</t>
-        </is>
-      </c>
-      <c r="G23" s="17" t="inlineStr">
-        <is>
-          <t>approvalAuthority, navigationEngine</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G23" s="17" t="inlineStr"/>
       <c r="H23" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7247,12 +7243,12 @@
       </c>
       <c r="B24" s="17" t="inlineStr">
         <is>
-          <t>eligibilityGuard</t>
+          <t>fibreServiceability</t>
         </is>
       </c>
       <c r="C24" s="17" t="inlineStr">
         <is>
-          <t>engines/eligibilityGuard.ts</t>
+          <t>engines/fibreServiceability.ts</t>
         </is>
       </c>
       <c r="D24" s="20" t="inlineStr">
@@ -7261,17 +7257,21 @@
         </is>
       </c>
       <c r="E24" s="17" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="F24" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
-        </is>
-      </c>
-      <c r="G24" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G24" s="17" t="inlineStr">
+        <is>
+          <t>FibreReadinessBanner, ActivationCompleteScreen</t>
+        </is>
+      </c>
       <c r="H24" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7283,12 +7283,12 @@
       </c>
       <c r="B25" s="17" t="inlineStr">
         <is>
-          <t>serviceLocationLookup</t>
+          <t>eligibilityGuard</t>
         </is>
       </c>
       <c r="C25" s="17" t="inlineStr">
         <is>
-          <t>engines/serviceLocationLookup.ts</t>
+          <t>engines/eligibilityGuard.ts</t>
         </is>
       </c>
       <c r="D25" s="20" t="inlineStr">
@@ -7301,17 +7301,13 @@
       </c>
       <c r="F25" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G25" s="17" t="inlineStr">
-        <is>
-          <t>ZsbAddressStep</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration</t>
+        </is>
+      </c>
+      <c r="G25" s="17" t="inlineStr"/>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -7323,12 +7319,12 @@
       </c>
       <c r="B26" s="17" t="inlineStr">
         <is>
-          <t>agentTaskEngine</t>
+          <t>serviceLocationLookup</t>
         </is>
       </c>
       <c r="C26" s="17" t="inlineStr">
         <is>
-          <t>engines/agentTaskEngine.ts</t>
+          <t>engines/serviceLocationLookup.ts</t>
         </is>
       </c>
       <c r="D26" s="20" t="inlineStr">
@@ -7337,17 +7333,21 @@
         </is>
       </c>
       <c r="E26" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F26" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, trouble-ticketing-complaints, orders, support, tasks</t>
-        </is>
-      </c>
-      <c r="G26" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G26" s="17" t="inlineStr">
+        <is>
+          <t>ZsbAddressStep</t>
+        </is>
+      </c>
       <c r="H26" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7359,12 +7359,12 @@
       </c>
       <c r="B27" s="17" t="inlineStr">
         <is>
-          <t>approvalAuthority</t>
+          <t>agentTaskEngine</t>
         </is>
       </c>
       <c r="C27" s="17" t="inlineStr">
         <is>
-          <t>engines/approvalAuthority.ts</t>
+          <t>engines/agentTaskEngine.ts</t>
         </is>
       </c>
       <c r="D27" s="20" t="inlineStr">
@@ -7377,13 +7377,13 @@
       </c>
       <c r="F27" s="17" t="inlineStr">
         <is>
-          <t>dashboard, order-management, sim-number-management, navigation, customer360, orders</t>
+          <t>dashboard, order-management, trouble-ticketing-complaints, orders, support, tasks</t>
         </is>
       </c>
       <c r="G27" s="17" t="inlineStr"/>
       <c r="H27" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7395,12 +7395,12 @@
       </c>
       <c r="B28" s="17" t="inlineStr">
         <is>
-          <t>portInEngine</t>
+          <t>approvalAuthority</t>
         </is>
       </c>
       <c r="C28" s="17" t="inlineStr">
         <is>
-          <t>engines/portInEngine.ts</t>
+          <t>engines/approvalAuthority.ts</t>
         </is>
       </c>
       <c r="D28" s="20" t="inlineStr">
@@ -7413,13 +7413,13 @@
       </c>
       <c r="F28" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
+          <t>dashboard, order-management, sim-number-management, navigation, customer360, orders</t>
         </is>
       </c>
       <c r="G28" s="17" t="inlineStr"/>
       <c r="H28" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7431,12 +7431,12 @@
       </c>
       <c r="B29" s="17" t="inlineStr">
         <is>
-          <t>csvExport</t>
+          <t>portInEngine</t>
         </is>
       </c>
       <c r="C29" s="17" t="inlineStr">
         <is>
-          <t>engines/csvExport.ts</t>
+          <t>engines/portInEngine.ts</t>
         </is>
       </c>
       <c r="D29" s="20" t="inlineStr">
@@ -7445,17 +7445,17 @@
         </is>
       </c>
       <c r="E29" s="17" t="n">
-        <v>4</v>
+        <v>6</v>
       </c>
       <c r="F29" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, customer360, profile, support</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G29" s="17" t="inlineStr"/>
       <c r="H29" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7467,12 +7467,12 @@
       </c>
       <c r="B30" s="17" t="inlineStr">
         <is>
-          <t>bellNotificationExpiry</t>
+          <t>csvExport</t>
         </is>
       </c>
       <c r="C30" s="17" t="inlineStr">
         <is>
-          <t>engines/bellNotificationExpiry.ts</t>
+          <t>engines/csvExport.ts</t>
         </is>
       </c>
       <c r="D30" s="20" t="inlineStr">
@@ -7481,11 +7481,11 @@
         </is>
       </c>
       <c r="E30" s="17" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="F30" s="17" t="inlineStr">
         <is>
-          <t>administration, customer360</t>
+          <t>trouble-ticketing-complaints, customer360, profile, support</t>
         </is>
       </c>
       <c r="G30" s="17" t="inlineStr"/>
@@ -7503,12 +7503,12 @@
       </c>
       <c r="B31" s="17" t="inlineStr">
         <is>
-          <t>businessAccountEngine</t>
+          <t>bellNotificationExpiry</t>
         </is>
       </c>
       <c r="C31" s="17" t="inlineStr">
         <is>
-          <t>engines/businessAccountEngine.ts</t>
+          <t>engines/bellNotificationExpiry.ts</t>
         </is>
       </c>
       <c r="D31" s="20" t="inlineStr">
@@ -7521,13 +7521,13 @@
       </c>
       <c r="F31" s="17" t="inlineStr">
         <is>
-          <t>customer-search, customer360</t>
+          <t>administration, customer360</t>
         </is>
       </c>
       <c r="G31" s="17" t="inlineStr"/>
       <c r="H31" s="17" t="inlineStr">
         <is>
-          <t>2026-10-06</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7539,12 +7539,12 @@
       </c>
       <c r="B32" s="17" t="inlineStr">
         <is>
-          <t>navigationEngine</t>
+          <t>businessAccountEngine</t>
         </is>
       </c>
       <c r="C32" s="17" t="inlineStr">
         <is>
-          <t>engines/navigationEngine.ts</t>
+          <t>engines/businessAccountEngine.ts</t>
         </is>
       </c>
       <c r="D32" s="20" t="inlineStr">
@@ -7557,13 +7557,13 @@
       </c>
       <c r="F32" s="17" t="inlineStr">
         <is>
-          <t>navigation, customer360</t>
+          <t>customer-search, customer360</t>
         </is>
       </c>
       <c r="G32" s="17" t="inlineStr"/>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-06</t>
         </is>
       </c>
     </row>
@@ -7575,12 +7575,12 @@
       </c>
       <c r="B33" s="17" t="inlineStr">
         <is>
-          <t>qnomyQueueEngine</t>
+          <t>navigationEngine</t>
         </is>
       </c>
       <c r="C33" s="17" t="inlineStr">
         <is>
-          <t>engines/qnomyQueueEngine.ts</t>
+          <t>engines/navigationEngine.ts</t>
         </is>
       </c>
       <c r="D33" s="20" t="inlineStr">
@@ -7593,17 +7593,13 @@
       </c>
       <c r="F33" s="17" t="inlineStr">
         <is>
-          <t>navigation, tickets</t>
-        </is>
-      </c>
-      <c r="G33" s="17" t="inlineStr">
-        <is>
-          <t>qnomyWalkIns</t>
-        </is>
-      </c>
+          <t>navigation, customer360</t>
+        </is>
+      </c>
+      <c r="G33" s="17" t="inlineStr"/>
       <c r="H33" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -7615,31 +7611,35 @@
       </c>
       <c r="B34" s="17" t="inlineStr">
         <is>
-          <t>agentProfileEngine</t>
+          <t>qnomyQueueEngine</t>
         </is>
       </c>
       <c r="C34" s="17" t="inlineStr">
         <is>
-          <t>engines/agentProfileEngine.ts</t>
-        </is>
-      </c>
-      <c r="D34" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>engines/qnomyQueueEngine.ts</t>
+        </is>
+      </c>
+      <c r="D34" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E34" s="17" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="F34" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G34" s="17" t="inlineStr"/>
+          <t>navigation, tickets</t>
+        </is>
+      </c>
+      <c r="G34" s="17" t="inlineStr">
+        <is>
+          <t>qnomyWalkIns</t>
+        </is>
+      </c>
       <c r="H34" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7651,12 +7651,12 @@
       </c>
       <c r="B35" s="17" t="inlineStr">
         <is>
-          <t>customer360VisibilityEngine</t>
+          <t>agentProfileEngine</t>
         </is>
       </c>
       <c r="C35" s="17" t="inlineStr">
         <is>
-          <t>engines/customer360VisibilityEngine.ts</t>
+          <t>engines/agentProfileEngine.ts</t>
         </is>
       </c>
       <c r="D35" s="21" t="inlineStr">
@@ -7669,13 +7669,13 @@
       </c>
       <c r="F35" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>navigation</t>
         </is>
       </c>
       <c r="G35" s="17" t="inlineStr"/>
       <c r="H35" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -7687,12 +7687,12 @@
       </c>
       <c r="B36" s="17" t="inlineStr">
         <is>
-          <t>profileChangeTicket</t>
+          <t>customer360VisibilityEngine</t>
         </is>
       </c>
       <c r="C36" s="17" t="inlineStr">
         <is>
-          <t>engines/profileChangeTicket.ts</t>
+          <t>engines/customer360VisibilityEngine.ts</t>
         </is>
       </c>
       <c r="D36" s="21" t="inlineStr">
@@ -7711,7 +7711,7 @@
       <c r="G36" s="17" t="inlineStr"/>
       <c r="H36" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -7723,12 +7723,12 @@
       </c>
       <c r="B37" s="17" t="inlineStr">
         <is>
-          <t>qnomyWalkIns</t>
+          <t>profileChangeTicket</t>
         </is>
       </c>
       <c r="C37" s="17" t="inlineStr">
         <is>
-          <t>engines/qnomyWalkIns.ts</t>
+          <t>engines/profileChangeTicket.ts</t>
         </is>
       </c>
       <c r="D37" s="21" t="inlineStr">
@@ -7741,13 +7741,13 @@
       </c>
       <c r="F37" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G37" s="17" t="inlineStr"/>
       <c r="H37" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -7759,12 +7759,12 @@
       </c>
       <c r="B38" s="17" t="inlineStr">
         <is>
-          <t>roleSwitchPurge</t>
+          <t>qnomyWalkIns</t>
         </is>
       </c>
       <c r="C38" s="17" t="inlineStr">
         <is>
-          <t>engines/roleSwitchPurge.ts</t>
+          <t>engines/qnomyWalkIns.ts</t>
         </is>
       </c>
       <c r="D38" s="21" t="inlineStr">
@@ -7783,7 +7783,7 @@
       <c r="G38" s="17" t="inlineStr"/>
       <c r="H38" s="17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -7795,12 +7795,12 @@
       </c>
       <c r="B39" s="17" t="inlineStr">
         <is>
-          <t>searchScopeEngine</t>
+          <t>roleSwitchPurge</t>
         </is>
       </c>
       <c r="C39" s="17" t="inlineStr">
         <is>
-          <t>engines/searchScopeEngine.ts</t>
+          <t>engines/roleSwitchPurge.ts</t>
         </is>
       </c>
       <c r="D39" s="21" t="inlineStr">
@@ -7819,7 +7819,7 @@
       <c r="G39" s="17" t="inlineStr"/>
       <c r="H39" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -7831,27 +7831,31 @@
       </c>
       <c r="B40" s="17" t="inlineStr">
         <is>
-          <t>moduleDescriptions</t>
+          <t>searchScopeEngine</t>
         </is>
       </c>
       <c r="C40" s="17" t="inlineStr">
         <is>
-          <t>engines/moduleDescriptions.ts</t>
-        </is>
-      </c>
-      <c r="D40" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>engines/searchScopeEngine.ts</t>
+        </is>
+      </c>
+      <c r="D40" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E40" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F40" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F40" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G40" s="17" t="inlineStr"/>
       <c r="H40" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -7863,12 +7867,12 @@
       </c>
       <c r="B41" s="17" t="inlineStr">
         <is>
-          <t>screenGrouping</t>
+          <t>moduleDescriptions</t>
         </is>
       </c>
       <c r="C41" s="17" t="inlineStr">
         <is>
-          <t>engines/screenGrouping.ts</t>
+          <t>engines/moduleDescriptions.ts</t>
         </is>
       </c>
       <c r="D41" s="23" t="inlineStr">
@@ -7890,40 +7894,32 @@
     <row r="42">
       <c r="A42" s="17" t="inlineStr">
         <is>
-          <t>Store</t>
+          <t>Engine</t>
         </is>
       </c>
       <c r="B42" s="17" t="inlineStr">
         <is>
-          <t>customerContextStore</t>
+          <t>screenGrouping</t>
         </is>
       </c>
       <c r="C42" s="17" t="inlineStr">
         <is>
-          <t>stores/customerContextStore.ts</t>
-        </is>
-      </c>
-      <c r="D42" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>engines/screenGrouping.ts</t>
+        </is>
+      </c>
+      <c r="D42" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E42" s="17" t="n">
-        <v>25</v>
-      </c>
-      <c r="F42" s="17" t="inlineStr">
-        <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G42" s="17" t="inlineStr">
-        <is>
-          <t>ActivationCompleteScreen, useActedForCustomer, useWizardDraftActions, roleSwitchPurge, authStore</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F42" s="17" t="inlineStr"/>
+      <c r="G42" s="17" t="inlineStr"/>
       <c r="H42" s="17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -7935,12 +7931,12 @@
       </c>
       <c r="B43" s="17" t="inlineStr">
         <is>
-          <t>authStore</t>
+          <t>customerContextStore</t>
         </is>
       </c>
       <c r="C43" s="17" t="inlineStr">
         <is>
-          <t>stores/authStore.ts</t>
+          <t>stores/customerContextStore.ts</t>
         </is>
       </c>
       <c r="D43" s="20" t="inlineStr">
@@ -7949,21 +7945,21 @@
         </is>
       </c>
       <c r="E43" s="17" t="n">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="F43" s="17" t="inlineStr">
         <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G43" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore, entityStore</t>
+          <t>ActivationCompleteScreen, useActedForCustomer, useWizardDraftActions, roleSwitchPurge, authStore</t>
         </is>
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -7975,12 +7971,12 @@
       </c>
       <c r="B44" s="17" t="inlineStr">
         <is>
-          <t>entityStore</t>
+          <t>authStore</t>
         </is>
       </c>
       <c r="C44" s="17" t="inlineStr">
         <is>
-          <t>stores/entityStore.ts</t>
+          <t>stores/authStore.ts</t>
         </is>
       </c>
       <c r="D44" s="20" t="inlineStr">
@@ -7998,12 +7994,12 @@
       </c>
       <c r="G44" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useIdLookup, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, useWizardDraftActions, activityEngine, agentProfileEngine, profileChangeTicket, configStore, entityStore</t>
         </is>
       </c>
       <c r="H44" s="17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8015,12 +8011,12 @@
       </c>
       <c r="B45" s="17" t="inlineStr">
         <is>
-          <t>personaStore</t>
+          <t>entityStore</t>
         </is>
       </c>
       <c r="C45" s="17" t="inlineStr">
         <is>
-          <t>stores/personaStore.ts</t>
+          <t>stores/entityStore.ts</t>
         </is>
       </c>
       <c r="D45" s="20" t="inlineStr">
@@ -8029,21 +8025,21 @@
         </is>
       </c>
       <c r="E45" s="17" t="n">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="F45" s="17" t="inlineStr">
         <is>
-          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, support, tasks, tickets</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, orders, profile, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G45" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, eligibilityRowsModel, ActivationCompleteScreen, AppointmentBookingStep, TicketCreationModal, useCheckoutSummary, useIdLookup, useRestrictedCustomers, configStore</t>
+          <t>ActivationCompleteScreen, DonorAttachmentStep, DonorDetailsStep, useIdLookup, useDraftStepSync, useWizardDraftActions, activityEngine, bellNotificationExpiry, profileChangeTicket</t>
         </is>
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -8055,12 +8051,12 @@
       </c>
       <c r="B46" s="17" t="inlineStr">
         <is>
-          <t>notificationStore</t>
+          <t>personaStore</t>
         </is>
       </c>
       <c r="C46" s="17" t="inlineStr">
         <is>
-          <t>stores/notificationStore.ts</t>
+          <t>stores/personaStore.ts</t>
         </is>
       </c>
       <c r="D46" s="20" t="inlineStr">
@@ -8069,21 +8065,21 @@
         </is>
       </c>
       <c r="E46" s="17" t="n">
-        <v>20</v>
+        <v>23</v>
       </c>
       <c r="F46" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
+          <t>dashboard, fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G46" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useJourneyMilestones, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, roleSwitchPurge, useSubmit</t>
+          <t>MsisdnPicker, eligibilityRowsModel, AppointmentBookingStep, TicketCreationModal, useCheckoutSummary, useIdLookup, useRestrictedCustomers, configStore</t>
         </is>
       </c>
       <c r="H46" s="17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8095,12 +8091,12 @@
       </c>
       <c r="B47" s="17" t="inlineStr">
         <is>
-          <t>workflowStore</t>
+          <t>notificationStore</t>
         </is>
       </c>
       <c r="C47" s="17" t="inlineStr">
         <is>
-          <t>stores/workflowStore.ts</t>
+          <t>stores/notificationStore.ts</t>
         </is>
       </c>
       <c r="D47" s="20" t="inlineStr">
@@ -8109,21 +8105,21 @@
         </is>
       </c>
       <c r="E47" s="17" t="n">
-        <v>12</v>
+        <v>20</v>
       </c>
       <c r="F47" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
+          <t>enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, identity-customer-management, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360, profile, support, tasks</t>
         </is>
       </c>
       <c r="G47" s="17" t="inlineStr">
         <is>
-          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation, roleSwitchPurge</t>
+          <t>MsisdnPicker, ActivationCompleteScreen, TicketCreationModal, useJourneyMilestones, useWizardDraftActions, useWizardStepNavigation, profileChangeTicket, roleSwitchPurge, useSubmit</t>
         </is>
       </c>
       <c r="H47" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-23</t>
         </is>
       </c>
     </row>
@@ -8135,35 +8131,35 @@
       </c>
       <c r="B48" s="17" t="inlineStr">
         <is>
-          <t>customerVerificationStore</t>
+          <t>workflowStore</t>
         </is>
       </c>
       <c r="C48" s="17" t="inlineStr">
         <is>
-          <t>stores/customerVerificationStore.ts</t>
-        </is>
-      </c>
-      <c r="D48" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>stores/workflowStore.ts</t>
+        </is>
+      </c>
+      <c r="D48" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E48" s="17" t="n">
-        <v>1</v>
+        <v>12</v>
       </c>
       <c r="F48" s="17" t="inlineStr">
         <is>
-          <t>customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration</t>
         </is>
       </c>
       <c r="G48" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>useJourneyStartResume, useMirrorChannel, useWizardDraftActions, useWizardStepNavigation, roleSwitchPurge</t>
         </is>
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8175,12 +8171,12 @@
       </c>
       <c r="B49" s="17" t="inlineStr">
         <is>
-          <t>qnomyQueueStore</t>
+          <t>customerVerificationStore</t>
         </is>
       </c>
       <c r="C49" s="17" t="inlineStr">
         <is>
-          <t>stores/qnomyQueueStore.ts</t>
+          <t>stores/customerVerificationStore.ts</t>
         </is>
       </c>
       <c r="D49" s="21" t="inlineStr">
@@ -8193,13 +8189,17 @@
       </c>
       <c r="F49" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G49" s="17" t="inlineStr"/>
+          <t>customer360</t>
+        </is>
+      </c>
+      <c r="G49" s="17" t="inlineStr">
+        <is>
+          <t>VerificationGate</t>
+        </is>
+      </c>
       <c r="H49" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8211,12 +8211,12 @@
       </c>
       <c r="B50" s="17" t="inlineStr">
         <is>
-          <t>regionStore</t>
+          <t>qnomyQueueStore</t>
         </is>
       </c>
       <c r="C50" s="17" t="inlineStr">
         <is>
-          <t>stores/regionStore.ts</t>
+          <t>stores/qnomyQueueStore.ts</t>
         </is>
       </c>
       <c r="D50" s="21" t="inlineStr">
@@ -8235,7 +8235,7 @@
       <c r="G50" s="17" t="inlineStr"/>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -8247,12 +8247,12 @@
       </c>
       <c r="B51" s="17" t="inlineStr">
         <is>
-          <t>sidebarStore</t>
+          <t>regionStore</t>
         </is>
       </c>
       <c r="C51" s="17" t="inlineStr">
         <is>
-          <t>stores/sidebarStore.ts</t>
+          <t>stores/regionStore.ts</t>
         </is>
       </c>
       <c r="D51" s="21" t="inlineStr">
@@ -8271,7 +8271,7 @@
       <c r="G51" s="17" t="inlineStr"/>
       <c r="H51" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8283,12 +8283,12 @@
       </c>
       <c r="B52" s="17" t="inlineStr">
         <is>
-          <t>themeStore</t>
+          <t>sidebarStore</t>
         </is>
       </c>
       <c r="C52" s="17" t="inlineStr">
         <is>
-          <t>stores/themeStore.ts</t>
+          <t>stores/sidebarStore.ts</t>
         </is>
       </c>
       <c r="D52" s="21" t="inlineStr">
@@ -8307,7 +8307,7 @@
       <c r="G52" s="17" t="inlineStr"/>
       <c r="H52" s="17" t="inlineStr">
         <is>
-          <t>2026-08-24</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8319,67 +8319,63 @@
       </c>
       <c r="B53" s="17" t="inlineStr">
         <is>
-          <t>configStore</t>
+          <t>themeStore</t>
         </is>
       </c>
       <c r="C53" s="17" t="inlineStr">
         <is>
-          <t>stores/configStore.ts</t>
-        </is>
-      </c>
-      <c r="D53" s="23" t="inlineStr">
-        <is>
-          <t>App shell only</t>
+          <t>stores/themeStore.ts</t>
+        </is>
+      </c>
+      <c r="D53" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E53" s="17" t="n">
-        <v>0</v>
-      </c>
-      <c r="F53" s="17" t="inlineStr"/>
+        <v>1</v>
+      </c>
+      <c r="F53" s="17" t="inlineStr">
+        <is>
+          <t>navigation</t>
+        </is>
+      </c>
       <c r="G53" s="17" t="inlineStr"/>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-08-24</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" s="17" t="inlineStr">
         <is>
-          <t>Hook</t>
+          <t>Store</t>
         </is>
       </c>
       <c r="B54" s="17" t="inlineStr">
         <is>
-          <t>useRestrictedCustomers</t>
+          <t>configStore</t>
         </is>
       </c>
       <c r="C54" s="17" t="inlineStr">
         <is>
-          <t>hooks/useRestrictedCustomers.ts</t>
-        </is>
-      </c>
-      <c r="D54" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>stores/configStore.ts</t>
+        </is>
+      </c>
+      <c r="D54" s="23" t="inlineStr">
+        <is>
+          <t>App shell only</t>
         </is>
       </c>
       <c r="E54" s="17" t="n">
-        <v>15</v>
-      </c>
-      <c r="F54" s="17" t="inlineStr">
-        <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G54" s="17" t="inlineStr">
-        <is>
-          <t>TicketCreationModal</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F54" s="17" t="inlineStr"/>
+      <c r="G54" s="17" t="inlineStr"/>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8391,12 +8387,12 @@
       </c>
       <c r="B55" s="17" t="inlineStr">
         <is>
-          <t>useEnterToSubmit</t>
+          <t>useRestrictedCustomers</t>
         </is>
       </c>
       <c r="C55" s="17" t="inlineStr">
         <is>
-          <t>hooks/useEnterToSubmit.ts</t>
+          <t>hooks/useRestrictedCustomers.ts</t>
         </is>
       </c>
       <c r="D55" s="20" t="inlineStr">
@@ -8405,21 +8401,21 @@
         </is>
       </c>
       <c r="E55" s="17" t="n">
-        <v>12</v>
+        <v>15</v>
       </c>
       <c r="F55" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, order-management, trouble-ticketing-complaints, navigation, customer360, orders, profile, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G55" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate, useIdLookup</t>
+          <t>TicketCreationModal</t>
         </is>
       </c>
       <c r="H55" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -8431,12 +8427,12 @@
       </c>
       <c r="B56" s="17" t="inlineStr">
         <is>
-          <t>useSearchListNav</t>
+          <t>useEnterToSubmit</t>
         </is>
       </c>
       <c r="C56" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSearchListNav.ts</t>
+          <t>hooks/useEnterToSubmit.ts</t>
         </is>
       </c>
       <c r="D56" s="20" t="inlineStr">
@@ -8449,17 +8445,17 @@
       </c>
       <c r="F56" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
         </is>
       </c>
       <c r="G56" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
+          <t>VerificationGate, useIdLookup</t>
         </is>
       </c>
       <c r="H56" s="17" t="inlineStr">
         <is>
-          <t>2026-10-05</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -8471,12 +8467,12 @@
       </c>
       <c r="B57" s="17" t="inlineStr">
         <is>
-          <t>useAreaOptions</t>
+          <t>useSearchListNav</t>
         </is>
       </c>
       <c r="C57" s="17" t="inlineStr">
         <is>
-          <t>hooks/useAreaOptions.ts</t>
+          <t>hooks/useSearchListNav.ts</t>
         </is>
       </c>
       <c r="D57" s="20" t="inlineStr">
@@ -8485,21 +8481,21 @@
         </is>
       </c>
       <c r="E57" s="17" t="n">
-        <v>8</v>
+        <v>12</v>
       </c>
       <c r="F57" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G57" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep, ZsbAddressStep</t>
+          <t>CompanySearchInput, ContactPhoneInput, PlanSearchBox, LocationInput</t>
         </is>
       </c>
       <c r="H57" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-05</t>
         </is>
       </c>
     </row>
@@ -8511,12 +8507,12 @@
       </c>
       <c r="B58" s="17" t="inlineStr">
         <is>
-          <t>useSubmit</t>
+          <t>useAreaOptions</t>
         </is>
       </c>
       <c r="C58" s="17" t="inlineStr">
         <is>
-          <t>hooks/useSubmit.ts</t>
+          <t>hooks/useAreaOptions.ts</t>
         </is>
       </c>
       <c r="D58" s="20" t="inlineStr">
@@ -8525,17 +8521,21 @@
         </is>
       </c>
       <c r="E58" s="17" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="F58" s="17" t="inlineStr">
         <is>
-          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
-        </is>
-      </c>
-      <c r="G58" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G58" s="17" t="inlineStr">
+        <is>
+          <t>BillingAccountStep, ZsbAddressStep</t>
+        </is>
+      </c>
       <c r="H58" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -8547,68 +8547,64 @@
       </c>
       <c r="B59" s="17" t="inlineStr">
         <is>
-          <t>useMinWidth</t>
+          <t>useSubmit</t>
         </is>
       </c>
       <c r="C59" s="17" t="inlineStr">
         <is>
-          <t>hooks/useMinWidth.ts</t>
-        </is>
-      </c>
-      <c r="D59" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>hooks/useSubmit.ts</t>
+        </is>
+      </c>
+      <c r="D59" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E59" s="17" t="n">
-        <v>1</v>
+        <v>6</v>
       </c>
       <c r="F59" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
+          <t>lead-management, mnp-fnp-porting, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
         </is>
       </c>
       <c r="G59" s="17" t="inlineStr"/>
       <c r="H59" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="17" t="inlineStr">
         <is>
-          <t>Helper</t>
+          <t>Hook</t>
         </is>
       </c>
       <c r="B60" s="17" t="inlineStr">
         <is>
-          <t>statusTone</t>
+          <t>useMinWidth</t>
         </is>
       </c>
       <c r="C60" s="17" t="inlineStr">
         <is>
-          <t>lib/statusTone.ts</t>
-        </is>
-      </c>
-      <c r="D60" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>hooks/useMinWidth.ts</t>
+        </is>
+      </c>
+      <c r="D60" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E60" s="17" t="n">
-        <v>21</v>
+        <v>1</v>
       </c>
       <c r="F60" s="17" t="inlineStr">
         <is>
-          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
-        </is>
-      </c>
-      <c r="G60" s="17" t="inlineStr">
-        <is>
-          <t>ruleEngine</t>
-        </is>
-      </c>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G60" s="17" t="inlineStr"/>
       <c r="H60" s="17" t="inlineStr">
         <is>
           <t>2026-10-18</t>
@@ -8623,12 +8619,12 @@
       </c>
       <c r="B61" s="17" t="inlineStr">
         <is>
-          <t>format</t>
+          <t>statusTone</t>
         </is>
       </c>
       <c r="C61" s="17" t="inlineStr">
         <is>
-          <t>lib/format.ts</t>
+          <t>lib/statusTone.ts</t>
         </is>
       </c>
       <c r="D61" s="20" t="inlineStr">
@@ -8637,21 +8633,21 @@
         </is>
       </c>
       <c r="E61" s="17" t="n">
-        <v>19</v>
+        <v>21</v>
       </c>
       <c r="F61" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, tasks</t>
+          <t>dashboard, enterprise-iot-b2b, fixed-line-fibre, fwa-5g-home, lead-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, sim-number-management, trouble-ticketing-complaints, administration, customer360, orders, sales, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G61" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, GuidedContactStep, IdLookupStep, StepSummaryPanel, stepSummary, customer360Engine, postpaidPricing</t>
+          <t>ruleEngine</t>
         </is>
       </c>
       <c r="H61" s="17" t="inlineStr">
         <is>
-          <t>2026-10-21</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -8663,12 +8659,12 @@
       </c>
       <c r="B62" s="17" t="inlineStr">
         <is>
-          <t>buildEnv</t>
+          <t>format</t>
         </is>
       </c>
       <c r="C62" s="17" t="inlineStr">
         <is>
-          <t>lib/buildEnv.ts</t>
+          <t>lib/format.ts</t>
         </is>
       </c>
       <c r="D62" s="20" t="inlineStr">
@@ -8677,21 +8673,21 @@
         </is>
       </c>
       <c r="E62" s="17" t="n">
-        <v>16</v>
+        <v>19</v>
       </c>
       <c r="F62" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer-search, customer360, orders, tasks</t>
         </is>
       </c>
       <c r="G62" s="17" t="inlineStr">
         <is>
-          <t>syntheticMarker, navigationEngine</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, GuidedContactStep, IdLookupStep, StepSummaryPanel, stepSummary, customer360Engine, postpaidPricing</t>
         </is>
       </c>
       <c r="H62" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-21</t>
         </is>
       </c>
     </row>
@@ -8703,12 +8699,12 @@
       </c>
       <c r="B63" s="17" t="inlineStr">
         <is>
-          <t>deviceType</t>
+          <t>buildEnv</t>
         </is>
       </c>
       <c r="C63" s="17" t="inlineStr">
         <is>
-          <t>lib/deviceType.ts</t>
+          <t>lib/buildEnv.ts</t>
         </is>
       </c>
       <c r="D63" s="20" t="inlineStr">
@@ -8717,21 +8713,21 @@
         </is>
       </c>
       <c r="E63" s="17" t="n">
-        <v>13</v>
+        <v>16</v>
       </c>
       <c r="F63" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, order-management, pre-to-post-migration, product-lines, sim-number-management, trouble-ticketing-complaints, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G63" s="17" t="inlineStr">
         <is>
-          <t>IdFileUpload, PassportScanSections, SimSerialScanner, SimTypeStep, cafTypes</t>
+          <t>syntheticMarker, navigationEngine</t>
         </is>
       </c>
       <c r="H63" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8743,12 +8739,12 @@
       </c>
       <c r="B64" s="17" t="inlineStr">
         <is>
-          <t>taskId</t>
+          <t>deviceType</t>
         </is>
       </c>
       <c r="C64" s="17" t="inlineStr">
         <is>
-          <t>lib/taskId.ts</t>
+          <t>lib/deviceType.ts</t>
         </is>
       </c>
       <c r="D64" s="20" t="inlineStr">
@@ -8757,16 +8753,16 @@
         </is>
       </c>
       <c r="E64" s="17" t="n">
-        <v>11</v>
+        <v>13</v>
       </c>
       <c r="F64" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, navigation, administration, customer360</t>
         </is>
       </c>
       <c r="G64" s="17" t="inlineStr">
         <is>
-          <t>useWizardDraftActions</t>
+          <t>IdFileUpload, PassportScanSections, SimSerialScanner, SimTypeStep, cafTypes</t>
         </is>
       </c>
       <c r="H64" s="17" t="inlineStr">
@@ -8783,12 +8779,12 @@
       </c>
       <c r="B65" s="17" t="inlineStr">
         <is>
-          <t>connectionType</t>
+          <t>taskId</t>
         </is>
       </c>
       <c r="C65" s="17" t="inlineStr">
         <is>
-          <t>lib/connectionType.ts</t>
+          <t>lib/taskId.ts</t>
         </is>
       </c>
       <c r="D65" s="20" t="inlineStr">
@@ -8797,21 +8793,21 @@
         </is>
       </c>
       <c r="E65" s="17" t="n">
-        <v>10</v>
+        <v>11</v>
       </c>
       <c r="F65" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G65" s="17" t="inlineStr">
         <is>
-          <t>ConnectionTypeTag</t>
+          <t>useWizardDraftActions</t>
         </is>
       </c>
       <c r="H65" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -8823,12 +8819,12 @@
       </c>
       <c r="B66" s="17" t="inlineStr">
         <is>
-          <t>serviceTypeTag</t>
+          <t>connectionType</t>
         </is>
       </c>
       <c r="C66" s="17" t="inlineStr">
         <is>
-          <t>lib/serviceTypeTag.ts</t>
+          <t>lib/connectionType.ts</t>
         </is>
       </c>
       <c r="D66" s="20" t="inlineStr">
@@ -8846,12 +8842,12 @@
       </c>
       <c r="G66" s="17" t="inlineStr">
         <is>
-          <t>ServiceTypeTag</t>
+          <t>ConnectionTypeTag</t>
         </is>
       </c>
       <c r="H66" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -8863,31 +8859,35 @@
       </c>
       <c r="B67" s="17" t="inlineStr">
         <is>
-          <t>screenName</t>
+          <t>serviceTypeTag</t>
         </is>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>lib/screenName.ts</t>
-        </is>
-      </c>
-      <c r="D67" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>lib/serviceTypeTag.ts</t>
+        </is>
+      </c>
+      <c r="D67" s="20" t="inlineStr">
+        <is>
+          <t>Shared (2+ areas)</t>
         </is>
       </c>
       <c r="E67" s="17" t="n">
-        <v>1</v>
+        <v>10</v>
       </c>
       <c r="F67" s="17" t="inlineStr">
         <is>
-          <t>navigation</t>
-        </is>
-      </c>
-      <c r="G67" s="17" t="inlineStr"/>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration, customer360</t>
+        </is>
+      </c>
+      <c r="G67" s="17" t="inlineStr">
+        <is>
+          <t>ServiceTypeTag</t>
+        </is>
+      </c>
       <c r="H67" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-19</t>
         </is>
       </c>
     </row>
@@ -8899,12 +8899,12 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>values</t>
+          <t>screenName</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>lib/values.ts</t>
+          <t>lib/screenName.ts</t>
         </is>
       </c>
       <c r="D68" s="21" t="inlineStr">
@@ -8917,22 +8917,58 @@
       </c>
       <c r="F68" s="17" t="inlineStr">
         <is>
+          <t>navigation</t>
+        </is>
+      </c>
+      <c r="G68" s="17" t="inlineStr"/>
+      <c r="H68" s="17" t="inlineStr">
+        <is>
+          <t>2026-10-15</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" s="17" t="inlineStr">
+        <is>
+          <t>Helper</t>
+        </is>
+      </c>
+      <c r="B69" s="17" t="inlineStr">
+        <is>
+          <t>values</t>
+        </is>
+      </c>
+      <c r="C69" s="17" t="inlineStr">
+        <is>
+          <t>lib/values.ts</t>
+        </is>
+      </c>
+      <c r="D69" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
+        </is>
+      </c>
+      <c r="E69" s="17" t="n">
+        <v>1</v>
+      </c>
+      <c r="F69" s="17" t="inlineStr">
+        <is>
           <t>customer360</t>
         </is>
       </c>
-      <c r="G68" s="17" t="inlineStr">
+      <c r="G69" s="17" t="inlineStr">
         <is>
           <t>customer360Demo</t>
         </is>
       </c>
-      <c r="H68" s="17" t="inlineStr">
+      <c r="H69" s="17" t="inlineStr">
         <is>
           <t>2026-10-05</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H68"/>
+  <autoFilter ref="A1:H69"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Configurable document types and Additional Documents layout; Billing label; tooltip positioning fix
</commit_message>
<xml_diff>
--- a/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
+++ b/vfq-dxp-app/reference/outputs/Reusable_Capabilities_Inventory_Reference.xlsx
@@ -718,13 +718,13 @@
         <v>53</v>
       </c>
       <c r="D7" s="17" t="n">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="E7" s="17" t="n">
         <v>4</v>
       </c>
       <c r="F7" s="17" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
     </row>
     <row r="8">
@@ -862,13 +862,13 @@
         <v>191</v>
       </c>
       <c r="D13" s="18" t="n">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="E13" s="18" t="n">
         <v>23</v>
       </c>
       <c r="F13" s="18" t="n">
-        <v>5</v>
+        <v>6</v>
       </c>
     </row>
     <row r="14">
@@ -1902,7 +1902,7 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, ScanFailureNotice, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, RestrictedCustomerNotice, RestrictedRowsNotice, ValidationStatus, ZsbAddressStep, CustomerViewButton, StepSummarySection, WizardFooter, ChoiceCards, DataTable, EmptyState, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, CompanySearchInput, ContactPhoneInput, EligibilityRows, FibreReadinessBanner, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, ScanFailureNotice, SimSerialScanner, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, FixedPlanStep, OrderConfirmationScreen, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, RestrictedCustomerNotice, RestrictedRowsNotice, ValidationStatus, ZsbAddressStep, CustomerViewButton, StepSummarySection, WizardFooter, ChoiceCards, DataTable, EmptyState, IconButton, LocationInput, Pager, PhoneNumberInput, SearchField, Select, Tabs, offerCardParts</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
@@ -1942,7 +1942,7 @@
       </c>
       <c r="G4" s="17" t="inlineStr">
         <is>
-          <t>ErrorBoundary, AdditionalDocumentsUpload, BillLimitEditor, CafDocumentUpload, EligibilityRows, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, SimTypeStep, ActivationCompleteScreen, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CafSignatureCapture, CheckoutDefaultLayout, DemoFaultPanel, FixedPlanStep, IdLookupStatus, NewCustomerForm, OrderConfirmationScreen, PostpaidDiscountsPanel, PostpaidPlanCard, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPackDetailsDrawer, PrepaidPlanCard, TicketCreationModal, ValidationStatus, VerificationGate, WinCashPaymentStep, ZsbAddressStep, CustomerViewButton, StepSummarySection, SummaryFieldRow, WizardDialogs, WizardFooter, WizardTitleBand, SignaturePad</t>
+          <t>ErrorBoundary, AdditionalDocumentsUpload, BillLimitEditor, CafDocumentUpload, EligibilityRows, IdFileUpload, MsisdnPicker, PassportScanSections, QidImageUpload, QidInput, SimSerialScanner, SimTypeStep, ActivationCompleteScreen, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CafSignatureCapture, CheckoutDefaultLayout, DemoFaultPanel, FixedPlanStep, IdLookupStatus, NewCustomerForm, OrderConfirmationScreen, PostpaidDiscountsPanel, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPackDetailsDrawer, PrepaidPlanCard, TicketCreationModal, ValidationStatus, VerificationGate, WinCashPaymentStep, ZsbAddressStep, CustomerViewButton, StepSummarySection, SummaryFieldRow, WizardDialogs, WizardFooter, WizardTitleBand, SignaturePad</t>
         </is>
       </c>
       <c r="H4" s="17" t="inlineStr">
@@ -2022,7 +2022,7 @@
       </c>
       <c r="G6" s="17" t="inlineStr">
         <is>
-          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CreditLimitCard, DonorDetailsStep, GuidedContactStep, NewCustomerForm, TicketCreationModal, ZsbAddressStep</t>
+          <t>AdditionalDocumentsUpload, CafDocumentUpload, MsisdnPicker, BillingAccountStep, BillingProfileSetupDrawer, BulkOperationPortal, CreditLimitCard, DonorDetailsStep, GuidedContactStep, NewCustomerForm, PostpaidPlanAddonsStep, TicketCreationModal, ZsbAddressStep</t>
         </is>
       </c>
       <c r="H6" s="17" t="inlineStr">
@@ -2582,12 +2582,12 @@
       </c>
       <c r="G20" s="17" t="inlineStr">
         <is>
-          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
+          <t>MsisdnPicker, QidInput, AppointmentBookingStep, BillingAccountStep, CafSignatureCapture, DiscountCard, FixedPlanStep, LineSelectionStep, PostpaidPlanCard, PrepaidPlanCard, PrepaidPlanStep, ChoiceCards</t>
         </is>
       </c>
       <c r="H20" s="17" t="inlineStr">
         <is>
-          <t>2026-10-19</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3055,7 +3055,7 @@
       <c r="G32" s="17" t="inlineStr"/>
       <c r="H32" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3467,7 +3467,7 @@
       </c>
       <c r="H43" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3659,7 +3659,7 @@
       </c>
       <c r="H48" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3855,7 +3855,7 @@
       <c r="G53" s="17" t="inlineStr"/>
       <c r="H53" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -3895,7 +3895,7 @@
       </c>
       <c r="H54" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4199,7 +4199,7 @@
       <c r="G62" s="17" t="inlineStr"/>
       <c r="H62" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4371,12 +4371,12 @@
       </c>
       <c r="B67" s="17" t="inlineStr">
         <is>
-          <t>NewCustomerForm</t>
+          <t>ValidationStatus</t>
         </is>
       </c>
       <c r="C67" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/NewCustomerForm.tsx</t>
+          <t>components/patterns/ValidationStatus.tsx</t>
         </is>
       </c>
       <c r="D67" s="20" t="inlineStr">
@@ -4394,12 +4394,12 @@
       </c>
       <c r="G67" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStep</t>
+          <t>IdLookupStatus</t>
         </is>
       </c>
       <c r="H67" s="17" t="inlineStr">
         <is>
-          <t>2026-10-20</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4411,12 +4411,12 @@
       </c>
       <c r="B68" s="17" t="inlineStr">
         <is>
-          <t>ValidationStatus</t>
+          <t>SignatureCapture</t>
         </is>
       </c>
       <c r="C68" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ValidationStatus.tsx</t>
+          <t>components/patterns/SignatureCapture.tsx</t>
         </is>
       </c>
       <c r="D68" s="20" t="inlineStr">
@@ -4425,21 +4425,21 @@
         </is>
       </c>
       <c r="E68" s="17" t="n">
-        <v>12</v>
+        <v>11</v>
       </c>
       <c r="F68" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration, customer360</t>
+          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G68" s="17" t="inlineStr">
         <is>
-          <t>IdLookupStatus</t>
+          <t>CafSignatureCapture, DonorAttachmentStep, SimSwapFormStep</t>
         </is>
       </c>
       <c r="H68" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4451,12 +4451,12 @@
       </c>
       <c r="B69" s="17" t="inlineStr">
         <is>
-          <t>SignatureCapture</t>
+          <t>ActivationCompleteScreen</t>
         </is>
       </c>
       <c r="C69" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/SignatureCapture.tsx</t>
+          <t>components/patterns/ActivationCompleteScreen.tsx</t>
         </is>
       </c>
       <c r="D69" s="20" t="inlineStr">
@@ -4465,21 +4465,17 @@
         </is>
       </c>
       <c r="E69" s="17" t="n">
-        <v>11</v>
+        <v>9</v>
       </c>
       <c r="F69" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, identity-customer-management, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, sim-number-management, administration</t>
-        </is>
-      </c>
-      <c r="G69" s="17" t="inlineStr">
-        <is>
-          <t>CafSignatureCapture, DonorAttachmentStep, SimSwapFormStep</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+        </is>
+      </c>
+      <c r="G69" s="17" t="inlineStr"/>
       <c r="H69" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4491,12 +4487,12 @@
       </c>
       <c r="B70" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>BillingAccountAutoResolver</t>
         </is>
       </c>
       <c r="C70" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ActivationCompleteScreen.tsx</t>
+          <t>components/patterns/BillingAccountAutoResolver.tsx</t>
         </is>
       </c>
       <c r="D70" s="20" t="inlineStr">
@@ -4515,7 +4511,7 @@
       <c r="G70" s="17" t="inlineStr"/>
       <c r="H70" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -4527,12 +4523,12 @@
       </c>
       <c r="B71" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountAutoResolver</t>
+          <t>CafSignatureCapture</t>
         </is>
       </c>
       <c r="C71" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingAccountAutoResolver.tsx</t>
+          <t>components/patterns/CafSignatureCapture.tsx</t>
         </is>
       </c>
       <c r="D71" s="20" t="inlineStr">
@@ -4551,7 +4547,7 @@
       <c r="G71" s="17" t="inlineStr"/>
       <c r="H71" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4563,12 +4559,12 @@
       </c>
       <c r="B72" s="17" t="inlineStr">
         <is>
-          <t>CafSignatureCapture</t>
+          <t>CheckoutDefaultLayout</t>
         </is>
       </c>
       <c r="C72" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafSignatureCapture.tsx</t>
+          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
         </is>
       </c>
       <c r="D72" s="20" t="inlineStr">
@@ -4584,10 +4580,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G72" s="17" t="inlineStr"/>
+      <c r="G72" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep</t>
+        </is>
+      </c>
       <c r="H72" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4599,12 +4599,12 @@
       </c>
       <c r="B73" s="17" t="inlineStr">
         <is>
-          <t>CheckoutDefaultLayout</t>
+          <t>CheckoutSummaryStep</t>
         </is>
       </c>
       <c r="C73" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutDefaultLayout.tsx</t>
+          <t>components/patterns/CheckoutSummaryStep.tsx</t>
         </is>
       </c>
       <c r="D73" s="20" t="inlineStr">
@@ -4620,11 +4620,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G73" s="17" t="inlineStr">
-        <is>
-          <t>CheckoutSummaryStep</t>
-        </is>
-      </c>
+      <c r="G73" s="17" t="inlineStr"/>
       <c r="H73" s="17" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -4639,12 +4635,12 @@
       </c>
       <c r="B74" s="17" t="inlineStr">
         <is>
-          <t>CheckoutSummaryStep</t>
+          <t>DiscountCard</t>
         </is>
       </c>
       <c r="C74" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryStep.tsx</t>
+          <t>components/patterns/DiscountCard.tsx</t>
         </is>
       </c>
       <c r="D74" s="20" t="inlineStr">
@@ -4660,10 +4656,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G74" s="17" t="inlineStr"/>
+      <c r="G74" s="17" t="inlineStr">
+        <is>
+          <t>PostpaidDiscountsPanel</t>
+        </is>
+      </c>
       <c r="H74" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4675,12 +4675,12 @@
       </c>
       <c r="B75" s="17" t="inlineStr">
         <is>
-          <t>DiscountCard</t>
+          <t>FixedPlanStep</t>
         </is>
       </c>
       <c r="C75" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DiscountCard.tsx</t>
+          <t>components/patterns/FixedPlanStep.tsx</t>
         </is>
       </c>
       <c r="D75" s="20" t="inlineStr">
@@ -4696,14 +4696,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G75" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidDiscountsPanel</t>
-        </is>
-      </c>
+      <c r="G75" s="17" t="inlineStr"/>
       <c r="H75" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4715,12 +4711,12 @@
       </c>
       <c r="B76" s="17" t="inlineStr">
         <is>
-          <t>FixedPlanStep</t>
+          <t>FullTerms</t>
         </is>
       </c>
       <c r="C76" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/FixedPlanStep.tsx</t>
+          <t>components/patterns/CafTerms.tsx</t>
         </is>
       </c>
       <c r="D76" s="20" t="inlineStr">
@@ -4736,10 +4732,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G76" s="17" t="inlineStr"/>
+      <c r="G76" s="17" t="inlineStr">
+        <is>
+          <t>CafSignatureCapture</t>
+        </is>
+      </c>
       <c r="H76" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4751,12 +4751,12 @@
       </c>
       <c r="B77" s="17" t="inlineStr">
         <is>
-          <t>FullTerms</t>
+          <t>KeyInformationPanel</t>
         </is>
       </c>
       <c r="C77" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CafTerms.tsx</t>
+          <t>components/patterns/KeyInformationPanel.tsx</t>
         </is>
       </c>
       <c r="D77" s="20" t="inlineStr">
@@ -4772,11 +4772,7 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G77" s="17" t="inlineStr">
-        <is>
-          <t>CafSignatureCapture</t>
-        </is>
-      </c>
+      <c r="G77" s="17" t="inlineStr"/>
       <c r="H77" s="17" t="inlineStr">
         <is>
           <t>2026-10-15</t>
@@ -4791,12 +4787,12 @@
       </c>
       <c r="B78" s="17" t="inlineStr">
         <is>
-          <t>KeyInformationPanel</t>
+          <t>OrderConfirmationScreen</t>
         </is>
       </c>
       <c r="C78" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/KeyInformationPanel.tsx</t>
+          <t>components/patterns/OrderConfirmationScreen.tsx</t>
         </is>
       </c>
       <c r="D78" s="20" t="inlineStr">
@@ -4812,10 +4808,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G78" s="17" t="inlineStr"/>
+      <c r="G78" s="17" t="inlineStr">
+        <is>
+          <t>ActivationCompleteScreen</t>
+        </is>
+      </c>
       <c r="H78" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-18</t>
         </is>
       </c>
     </row>
@@ -4827,12 +4827,12 @@
       </c>
       <c r="B79" s="17" t="inlineStr">
         <is>
-          <t>OrderConfirmationScreen</t>
+          <t>PlanDetailsDrawer</t>
         </is>
       </c>
       <c r="C79" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/OrderConfirmationScreen.tsx</t>
+          <t>components/patterns/PlanDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D79" s="20" t="inlineStr">
@@ -4850,12 +4850,12 @@
       </c>
       <c r="G79" s="17" t="inlineStr">
         <is>
-          <t>ActivationCompleteScreen</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="H79" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -4867,12 +4867,12 @@
       </c>
       <c r="B80" s="17" t="inlineStr">
         <is>
-          <t>PlanDetailsDrawer</t>
+          <t>PlanGroupPanel</t>
         </is>
       </c>
       <c r="C80" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanDetailsDrawer.tsx</t>
+          <t>components/patterns/PlanGroupPanel.tsx</t>
         </is>
       </c>
       <c r="D80" s="20" t="inlineStr">
@@ -4895,7 +4895,7 @@
       </c>
       <c r="H80" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -4907,12 +4907,12 @@
       </c>
       <c r="B81" s="17" t="inlineStr">
         <is>
-          <t>PlanGroupPanel</t>
+          <t>PlanSearchBox</t>
         </is>
       </c>
       <c r="C81" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanGroupPanel.tsx</t>
+          <t>components/patterns/PlanSearchBox.tsx</t>
         </is>
       </c>
       <c r="D81" s="20" t="inlineStr">
@@ -4935,7 +4935,7 @@
       </c>
       <c r="H81" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -4947,12 +4947,12 @@
       </c>
       <c r="B82" s="17" t="inlineStr">
         <is>
-          <t>PlanSearchBox</t>
+          <t>PlanTabStrip</t>
         </is>
       </c>
       <c r="C82" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanSearchBox.tsx</t>
+          <t>components/patterns/PlanTabStrip.tsx</t>
         </is>
       </c>
       <c r="D82" s="20" t="inlineStr">
@@ -4987,12 +4987,12 @@
       </c>
       <c r="B83" s="17" t="inlineStr">
         <is>
-          <t>PlanTabStrip</t>
+          <t>PostpaidAddonsPanel</t>
         </is>
       </c>
       <c r="C83" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PlanTabStrip.tsx</t>
+          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
         </is>
       </c>
       <c r="D83" s="20" t="inlineStr">
@@ -5027,12 +5027,12 @@
       </c>
       <c r="B84" s="17" t="inlineStr">
         <is>
-          <t>PostpaidAddonsPanel</t>
+          <t>PostpaidDiscountsPanel</t>
         </is>
       </c>
       <c r="C84" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidAddonsPanel.tsx</t>
+          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
         </is>
       </c>
       <c r="D84" s="20" t="inlineStr">
@@ -5067,12 +5067,12 @@
       </c>
       <c r="B85" s="17" t="inlineStr">
         <is>
-          <t>PostpaidDiscountsPanel</t>
+          <t>PostpaidMonthlySummary</t>
         </is>
       </c>
       <c r="C85" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidDiscountsPanel.tsx</t>
+          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
         </is>
       </c>
       <c r="D85" s="20" t="inlineStr">
@@ -5095,7 +5095,7 @@
       </c>
       <c r="H85" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5107,12 +5107,12 @@
       </c>
       <c r="B86" s="17" t="inlineStr">
         <is>
-          <t>PostpaidMonthlySummary</t>
+          <t>PostpaidPlanAddonsStep</t>
         </is>
       </c>
       <c r="C86" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidMonthlySummary.tsx</t>
+          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
         </is>
       </c>
       <c r="D86" s="20" t="inlineStr">
@@ -5128,14 +5128,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G86" s="17" t="inlineStr">
-        <is>
-          <t>PostpaidPlanAddonsStep</t>
-        </is>
-      </c>
+      <c r="G86" s="17" t="inlineStr"/>
       <c r="H86" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5147,12 +5143,12 @@
       </c>
       <c r="B87" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanAddonsStep</t>
+          <t>PostpaidPlanCard</t>
         </is>
       </c>
       <c r="C87" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanAddonsStep.tsx</t>
+          <t>components/patterns/PostpaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D87" s="20" t="inlineStr">
@@ -5168,10 +5164,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G87" s="17" t="inlineStr"/>
+      <c r="G87" s="17" t="inlineStr">
+        <is>
+          <t>PlanGroupPanel</t>
+        </is>
+      </c>
       <c r="H87" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5183,12 +5183,12 @@
       </c>
       <c r="B88" s="17" t="inlineStr">
         <is>
-          <t>PostpaidPlanCard</t>
+          <t>PrepaidCartStep</t>
         </is>
       </c>
       <c r="C88" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PostpaidPlanCard.tsx</t>
+          <t>components/patterns/PrepaidCartStep.tsx</t>
         </is>
       </c>
       <c r="D88" s="20" t="inlineStr">
@@ -5204,14 +5204,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G88" s="17" t="inlineStr">
-        <is>
-          <t>PlanGroupPanel</t>
-        </is>
-      </c>
+      <c r="G88" s="17" t="inlineStr"/>
       <c r="H88" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5223,12 +5219,12 @@
       </c>
       <c r="B89" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCartStep</t>
+          <t>PrepaidCheckoutStep</t>
         </is>
       </c>
       <c r="C89" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCartStep.tsx</t>
+          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
         </is>
       </c>
       <c r="D89" s="20" t="inlineStr">
@@ -5247,7 +5243,7 @@
       <c r="G89" s="17" t="inlineStr"/>
       <c r="H89" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5259,12 +5255,12 @@
       </c>
       <c r="B90" s="17" t="inlineStr">
         <is>
-          <t>PrepaidCheckoutStep</t>
+          <t>PrepaidPackDetailsDrawer</t>
         </is>
       </c>
       <c r="C90" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidCheckoutStep.tsx</t>
+          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
         </is>
       </c>
       <c r="D90" s="20" t="inlineStr">
@@ -5280,7 +5276,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G90" s="17" t="inlineStr"/>
+      <c r="G90" s="17" t="inlineStr">
+        <is>
+          <t>PrepaidPlanStep</t>
+        </is>
+      </c>
       <c r="H90" s="17" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -5295,12 +5295,12 @@
       </c>
       <c r="B91" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPackDetailsDrawer</t>
+          <t>PrepaidPlanCard</t>
         </is>
       </c>
       <c r="C91" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPackDetailsDrawer.tsx</t>
+          <t>components/patterns/PrepaidPlanCard.tsx</t>
         </is>
       </c>
       <c r="D91" s="20" t="inlineStr">
@@ -5323,7 +5323,7 @@
       </c>
       <c r="H91" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5335,12 +5335,12 @@
       </c>
       <c r="B92" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanCard</t>
+          <t>PrepaidPlanStep</t>
         </is>
       </c>
       <c r="C92" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanCard.tsx</t>
+          <t>components/patterns/PrepaidPlanStep.tsx</t>
         </is>
       </c>
       <c r="D92" s="20" t="inlineStr">
@@ -5356,14 +5356,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G92" s="17" t="inlineStr">
-        <is>
-          <t>PrepaidPlanStep</t>
-        </is>
-      </c>
+      <c r="G92" s="17" t="inlineStr"/>
       <c r="H92" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5375,12 +5371,12 @@
       </c>
       <c r="B93" s="17" t="inlineStr">
         <is>
-          <t>PrepaidPlanStep</t>
+          <t>SummaryTables</t>
         </is>
       </c>
       <c r="C93" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/PrepaidPlanStep.tsx</t>
+          <t>components/patterns/CheckoutSummaryTables.tsx</t>
         </is>
       </c>
       <c r="D93" s="20" t="inlineStr">
@@ -5396,10 +5392,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G93" s="17" t="inlineStr"/>
+      <c r="G93" s="17" t="inlineStr">
+        <is>
+          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
+        </is>
+      </c>
       <c r="H93" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5411,12 +5411,12 @@
       </c>
       <c r="B94" s="17" t="inlineStr">
         <is>
-          <t>SummaryTables</t>
+          <t>WinCashPaymentStep</t>
         </is>
       </c>
       <c r="C94" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CheckoutSummaryTables.tsx</t>
+          <t>components/patterns/WinCashPaymentStep.tsx</t>
         </is>
       </c>
       <c r="D94" s="20" t="inlineStr">
@@ -5432,14 +5432,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G94" s="17" t="inlineStr">
-        <is>
-          <t>CheckoutSummaryStep, checkoutDetailedTables</t>
-        </is>
-      </c>
+      <c r="G94" s="17" t="inlineStr"/>
       <c r="H94" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5451,12 +5447,12 @@
       </c>
       <c r="B95" s="17" t="inlineStr">
         <is>
-          <t>WinCashPaymentStep</t>
+          <t>BillingAccountStep</t>
         </is>
       </c>
       <c r="C95" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/WinCashPaymentStep.tsx</t>
+          <t>components/patterns/BillingAccountStep.tsx</t>
         </is>
       </c>
       <c r="D95" s="20" t="inlineStr">
@@ -5465,17 +5461,17 @@
         </is>
       </c>
       <c r="E95" s="17" t="n">
-        <v>9</v>
+        <v>8</v>
       </c>
       <c r="F95" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, mobile-service-changes, new-connection, pre-to-post-migration, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G95" s="17" t="inlineStr"/>
       <c r="H95" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5487,12 +5483,12 @@
       </c>
       <c r="B96" s="17" t="inlineStr">
         <is>
-          <t>BillingAccountStep</t>
+          <t>BillingProfileSetupDrawer</t>
         </is>
       </c>
       <c r="C96" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingAccountStep.tsx</t>
+          <t>components/patterns/BillingProfileSetupDrawer.tsx</t>
         </is>
       </c>
       <c r="D96" s="20" t="inlineStr">
@@ -5508,10 +5504,14 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G96" s="17" t="inlineStr"/>
+      <c r="G96" s="17" t="inlineStr">
+        <is>
+          <t>BillingAccountStep</t>
+        </is>
+      </c>
       <c r="H96" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5523,12 +5523,12 @@
       </c>
       <c r="B97" s="17" t="inlineStr">
         <is>
-          <t>BillingProfileSetupDrawer</t>
+          <t>CreditLimitCard</t>
         </is>
       </c>
       <c r="C97" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BillingProfileSetupDrawer.tsx</t>
+          <t>components/patterns/CreditLimitCard.tsx</t>
         </is>
       </c>
       <c r="D97" s="20" t="inlineStr">
@@ -5544,14 +5544,10 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G97" s="17" t="inlineStr">
-        <is>
-          <t>BillingAccountStep</t>
-        </is>
-      </c>
+      <c r="G97" s="17" t="inlineStr"/>
       <c r="H97" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-26</t>
         </is>
       </c>
     </row>
@@ -5563,12 +5559,12 @@
       </c>
       <c r="B98" s="17" t="inlineStr">
         <is>
-          <t>CreditLimitCard</t>
+          <t>ZsbAddressStep</t>
         </is>
       </c>
       <c r="C98" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/CreditLimitCard.tsx</t>
+          <t>components/patterns/ZsbAddressStep.tsx</t>
         </is>
       </c>
       <c r="D98" s="20" t="inlineStr">
@@ -5584,7 +5580,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
         </is>
       </c>
-      <c r="G98" s="17" t="inlineStr"/>
+      <c r="G98" s="17" t="inlineStr">
+        <is>
+          <t>addressFromBilling</t>
+        </is>
+      </c>
       <c r="H98" s="17" t="inlineStr">
         <is>
           <t>2026-10-26</t>
@@ -5599,12 +5599,12 @@
       </c>
       <c r="B99" s="17" t="inlineStr">
         <is>
-          <t>ZsbAddressStep</t>
+          <t>AppointmentBookingStep</t>
         </is>
       </c>
       <c r="C99" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ZsbAddressStep.tsx</t>
+          <t>components/patterns/AppointmentBookingStep.tsx</t>
         </is>
       </c>
       <c r="D99" s="20" t="inlineStr">
@@ -5613,21 +5613,17 @@
         </is>
       </c>
       <c r="E99" s="17" t="n">
-        <v>8</v>
+        <v>7</v>
       </c>
       <c r="F99" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, pre-to-post-migration, administration</t>
-        </is>
-      </c>
-      <c r="G99" s="17" t="inlineStr">
-        <is>
-          <t>addressFromBilling</t>
-        </is>
-      </c>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
+        </is>
+      </c>
+      <c r="G99" s="17" t="inlineStr"/>
       <c r="H99" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5639,12 +5635,12 @@
       </c>
       <c r="B100" s="17" t="inlineStr">
         <is>
-          <t>AppointmentBookingStep</t>
+          <t>DemoFaultPanel</t>
         </is>
       </c>
       <c r="C100" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/AppointmentBookingStep.tsx</t>
+          <t>components/patterns/DemoFaultPanel.tsx</t>
         </is>
       </c>
       <c r="D100" s="20" t="inlineStr">
@@ -5653,11 +5649,11 @@
         </is>
       </c>
       <c r="E100" s="17" t="n">
-        <v>7</v>
+        <v>6</v>
       </c>
       <c r="F100" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection, administration</t>
+          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
       <c r="G100" s="17" t="inlineStr"/>
@@ -5675,12 +5671,12 @@
       </c>
       <c r="B101" s="17" t="inlineStr">
         <is>
-          <t>DemoFaultPanel</t>
+          <t>DonorAttachmentStep</t>
         </is>
       </c>
       <c r="C101" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DemoFaultPanel.tsx</t>
+          <t>components/patterns/DonorAttachmentStep.tsx</t>
         </is>
       </c>
       <c r="D101" s="20" t="inlineStr">
@@ -5711,12 +5707,12 @@
       </c>
       <c r="B102" s="17" t="inlineStr">
         <is>
-          <t>DonorAttachmentStep</t>
+          <t>DonorDetailsStep</t>
         </is>
       </c>
       <c r="C102" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorAttachmentStep.tsx</t>
+          <t>components/patterns/DonorDetailsStep.tsx</t>
         </is>
       </c>
       <c r="D102" s="20" t="inlineStr">
@@ -5732,7 +5728,11 @@
           <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
         </is>
       </c>
-      <c r="G102" s="17" t="inlineStr"/>
+      <c r="G102" s="17" t="inlineStr">
+        <is>
+          <t>DonorAttachmentStep</t>
+        </is>
+      </c>
       <c r="H102" s="17" t="inlineStr">
         <is>
           <t>2026-10-25</t>
@@ -5747,12 +5747,12 @@
       </c>
       <c r="B103" s="17" t="inlineStr">
         <is>
-          <t>DonorDetailsStep</t>
+          <t>EntityMissing</t>
         </is>
       </c>
       <c r="C103" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DonorDetailsStep.tsx</t>
+          <t>components/patterns/EntityMissing.tsx</t>
         </is>
       </c>
       <c r="D103" s="20" t="inlineStr">
@@ -5765,14 +5765,10 @@
       </c>
       <c r="F103" s="17" t="inlineStr">
         <is>
-          <t>fixed-line-fibre, fwa-5g-home, mnp-fnp-porting, mobile-postpaid, mobile-prepaid, new-connection</t>
-        </is>
-      </c>
-      <c r="G103" s="17" t="inlineStr">
-        <is>
-          <t>DonorAttachmentStep</t>
-        </is>
-      </c>
+          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
+        </is>
+      </c>
+      <c r="G103" s="17" t="inlineStr"/>
       <c r="H103" s="17" t="inlineStr">
         <is>
           <t>2026-10-25</t>
@@ -5787,12 +5783,12 @@
       </c>
       <c r="B104" s="17" t="inlineStr">
         <is>
-          <t>EntityMissing</t>
+          <t>RestrictedRowsNotice</t>
         </is>
       </c>
       <c r="C104" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/EntityMissing.tsx</t>
+          <t>components/patterns/RestrictedRowsNotice.tsx</t>
         </is>
       </c>
       <c r="D104" s="20" t="inlineStr">
@@ -5805,13 +5801,13 @@
       </c>
       <c r="F104" s="17" t="inlineStr">
         <is>
-          <t>lead-management, order-management, sim-number-management, trouble-ticketing-complaints, customer360, tasks</t>
+          <t>order-management, trouble-ticketing-complaints, orders, support, tasks, tickets</t>
         </is>
       </c>
       <c r="G104" s="17" t="inlineStr"/>
       <c r="H104" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-22</t>
         </is>
       </c>
     </row>
@@ -5823,12 +5819,12 @@
       </c>
       <c r="B105" s="17" t="inlineStr">
         <is>
-          <t>RestrictedRowsNotice</t>
+          <t>ActivityCommentsStep</t>
         </is>
       </c>
       <c r="C105" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/RestrictedRowsNotice.tsx</t>
+          <t>components/patterns/ActivityCommentsStep.tsx</t>
         </is>
       </c>
       <c r="D105" s="20" t="inlineStr">
@@ -5837,17 +5833,17 @@
         </is>
       </c>
       <c r="E105" s="17" t="n">
-        <v>6</v>
+        <v>3</v>
       </c>
       <c r="F105" s="17" t="inlineStr">
         <is>
-          <t>order-management, trouble-ticketing-complaints, orders, support, tasks, tickets</t>
+          <t>pre-to-post-migration, sim-number-management, administration</t>
         </is>
       </c>
       <c r="G105" s="17" t="inlineStr"/>
       <c r="H105" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-09-24</t>
         </is>
       </c>
     </row>
@@ -5859,12 +5855,12 @@
       </c>
       <c r="B106" s="17" t="inlineStr">
         <is>
-          <t>ActivityCommentsStep</t>
+          <t>LineSelectionStep</t>
         </is>
       </c>
       <c r="C106" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/ActivityCommentsStep.tsx</t>
+          <t>components/patterns/LineSelectionStep.tsx</t>
         </is>
       </c>
       <c r="D106" s="20" t="inlineStr">
@@ -5877,13 +5873,13 @@
       </c>
       <c r="F106" s="17" t="inlineStr">
         <is>
-          <t>pre-to-post-migration, sim-number-management, administration</t>
+          <t>mobile-service-changes, pre-to-post-migration, administration</t>
         </is>
       </c>
       <c r="G106" s="17" t="inlineStr"/>
       <c r="H106" s="17" t="inlineStr">
         <is>
-          <t>2026-09-24</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -5895,12 +5891,12 @@
       </c>
       <c r="B107" s="17" t="inlineStr">
         <is>
-          <t>LineSelectionStep</t>
+          <t>TicketCreationModal</t>
         </is>
       </c>
       <c r="C107" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/LineSelectionStep.tsx</t>
+          <t>components/patterns/TicketCreationModal.tsx</t>
         </is>
       </c>
       <c r="D107" s="20" t="inlineStr">
@@ -5913,13 +5909,13 @@
       </c>
       <c r="F107" s="17" t="inlineStr">
         <is>
-          <t>mobile-service-changes, pre-to-post-migration, administration</t>
+          <t>trouble-ticketing-complaints, customer360, support</t>
         </is>
       </c>
       <c r="G107" s="17" t="inlineStr"/>
       <c r="H107" s="17" t="inlineStr">
         <is>
-          <t>2026-10-26</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -5931,31 +5927,31 @@
       </c>
       <c r="B108" s="17" t="inlineStr">
         <is>
-          <t>TicketCreationModal</t>
+          <t>BulkOperationPortal</t>
         </is>
       </c>
       <c r="C108" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/TicketCreationModal.tsx</t>
-        </is>
-      </c>
-      <c r="D108" s="20" t="inlineStr">
-        <is>
-          <t>Shared (2+ areas)</t>
+          <t>components/patterns/BulkOperationPortal.tsx</t>
+        </is>
+      </c>
+      <c r="D108" s="21" t="inlineStr">
+        <is>
+          <t>Single area</t>
         </is>
       </c>
       <c r="E108" s="17" t="n">
-        <v>3</v>
+        <v>1</v>
       </c>
       <c r="F108" s="17" t="inlineStr">
         <is>
-          <t>trouble-ticketing-complaints, customer360, support</t>
+          <t>enterprise-iot-b2b</t>
         </is>
       </c>
       <c r="G108" s="17" t="inlineStr"/>
       <c r="H108" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-15</t>
         </is>
       </c>
     </row>
@@ -5967,12 +5963,12 @@
       </c>
       <c r="B109" s="17" t="inlineStr">
         <is>
-          <t>BulkOperationPortal</t>
+          <t>DualPlaySerialCheckStep</t>
         </is>
       </c>
       <c r="C109" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/BulkOperationPortal.tsx</t>
+          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
         </is>
       </c>
       <c r="D109" s="21" t="inlineStr">
@@ -5985,7 +5981,7 @@
       </c>
       <c r="F109" s="17" t="inlineStr">
         <is>
-          <t>enterprise-iot-b2b</t>
+          <t>fwa-5g-home</t>
         </is>
       </c>
       <c r="G109" s="17" t="inlineStr"/>
@@ -6003,12 +5999,12 @@
       </c>
       <c r="B110" s="17" t="inlineStr">
         <is>
-          <t>DualPlaySerialCheckStep</t>
+          <t>SimSwapFormStep</t>
         </is>
       </c>
       <c r="C110" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/DualPlaySerialCheckStep.tsx</t>
+          <t>components/patterns/SimSwapFormStep.tsx</t>
         </is>
       </c>
       <c r="D110" s="21" t="inlineStr">
@@ -6021,7 +6017,7 @@
       </c>
       <c r="F110" s="17" t="inlineStr">
         <is>
-          <t>fwa-5g-home</t>
+          <t>sim-number-management</t>
         </is>
       </c>
       <c r="G110" s="17" t="inlineStr"/>
@@ -6039,12 +6035,12 @@
       </c>
       <c r="B111" s="17" t="inlineStr">
         <is>
-          <t>SimSwapFormStep</t>
+          <t>VerificationGate</t>
         </is>
       </c>
       <c r="C111" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/SimSwapFormStep.tsx</t>
+          <t>components/patterns/VerificationGate.tsx</t>
         </is>
       </c>
       <c r="D111" s="21" t="inlineStr">
@@ -6057,13 +6053,13 @@
       </c>
       <c r="F111" s="17" t="inlineStr">
         <is>
-          <t>sim-number-management</t>
+          <t>customer360</t>
         </is>
       </c>
       <c r="G111" s="17" t="inlineStr"/>
       <c r="H111" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-25</t>
         </is>
       </c>
     </row>
@@ -6075,31 +6071,27 @@
       </c>
       <c r="B112" s="17" t="inlineStr">
         <is>
-          <t>VerificationGate</t>
+          <t>NewCustomerForm</t>
         </is>
       </c>
       <c r="C112" s="17" t="inlineStr">
         <is>
-          <t>components/patterns/VerificationGate.tsx</t>
-        </is>
-      </c>
-      <c r="D112" s="21" t="inlineStr">
-        <is>
-          <t>Single area</t>
+          <t>components/patterns/NewCustomerForm.tsx</t>
+        </is>
+      </c>
+      <c r="D112" s="22" t="inlineStr">
+        <is>
+          <t>No consumer</t>
         </is>
       </c>
       <c r="E112" s="17" t="n">
-        <v>1</v>
-      </c>
-      <c r="F112" s="17" t="inlineStr">
-        <is>
-          <t>customer360</t>
-        </is>
-      </c>
+        <v>0</v>
+      </c>
+      <c r="F112" s="17" t="inlineStr"/>
       <c r="G112" s="17" t="inlineStr"/>
       <c r="H112" s="17" t="inlineStr">
         <is>
-          <t>2026-10-25</t>
+          <t>2026-10-20</t>
         </is>
       </c>
     </row>
@@ -6247,7 +6239,7 @@
       <c r="G116" s="17" t="inlineStr"/>
       <c r="H116" s="17" t="inlineStr">
         <is>
-          <t>2026-10-22</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -6537,7 +6529,7 @@
       </c>
       <c r="G2" s="17" t="inlineStr">
         <is>
-          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, connectionEligibility, customer360Engine, customerChangeAudit, fibreServiceability, qnomyWalkIns, roleSwitchPurge, serviceLocationLookup, useAreaOptions, useRestrictedCustomers, configStore, entityStore</t>
+          <t>CompanySearchInput, ContactPhoneInput, CpeSerialScanner, MsisdnPicker, SimSerialScanner, SimTypeStep, AppointmentBookingStep, BillingAccountAutoResolver, BillingAccountStep, CafSignatureCapture, CafTerms, FixedPlanStep, PrepaidCartStep, PrepaidCheckoutStep, PrepaidPlanStep, TicketCreationModal, ZsbAddressStep, lineSelectionModel, useCheckoutSummary, useIdLookup, usePostpaidPlanAddons, StepSummaryPanel, stepSummary, useJourneyStartResume, useWizardDraftActions, LocationInput, activityEngine, agentProfileEngine, businessAccountEngine, connectionEligibility, customer360Engine, customerChangeAudit, fibreServiceability, qnomyWalkIns, roleSwitchPurge, serviceLocationLookup, useAreaOptions, useRestrictedCustomers, configStore, entityStore</t>
         </is>
       </c>
       <c r="H2" s="17" t="inlineStr">
@@ -6577,12 +6569,12 @@
       </c>
       <c r="G3" s="17" t="inlineStr">
         <is>
-          <t>agentPrivilegeEngine, agentProfileEngine, approvalAuthority, customer360VisibilityEngine, navigationEngine, personaEngine, qnomyQueueEngine, screenGrouping, configStore</t>
+          <t>GuidedContactStep, agentPrivilegeEngine, agentProfileEngine, approvalAuthority, customer360VisibilityEngine, journeyDocuments, navigationEngine, personaEngine, qnomyQueueEngine, screenGrouping, configStore</t>
         </is>
       </c>
       <c r="H3" s="17" t="inlineStr">
         <is>
-          <t>2026-10-18</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -7454,7 +7446,7 @@
       </c>
       <c r="H25" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -8182,7 +8174,7 @@
       </c>
       <c r="H45" s="17" t="inlineStr">
         <is>
-          <t>2026-10-23</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -8382,7 +8374,7 @@
       </c>
       <c r="H50" s="17" t="inlineStr">
         <is>
-          <t>2026-10-15</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>
@@ -9150,7 +9142,7 @@
       </c>
       <c r="H70" s="17" t="inlineStr">
         <is>
-          <t>uncommitted</t>
+          <t>2026-10-27</t>
         </is>
       </c>
     </row>

</xml_diff>